<commit_message>
docs: add use case and route map diagrams and update docs
</commit_message>
<xml_diff>
--- a/docs/Squad App Frontend IPA Zeitplan.xlsx
+++ b/docs/Squad App Frontend IPA Zeitplan.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7783F142-A185-4565-A7C4-D428AED6844F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3737EC6-FB80-45CE-89A4-10E01C4F00F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-1930" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14,6 +14,7 @@
     <definedName name="LOCAL_MYSQL_DATE_FORMAT" hidden="1">REPT(LOCAL_YEAR_FORMAT,4)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_MONTH_FORMAT,2)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_DAY_FORMAT,2)&amp;" "&amp;REPT(LOCAL_HOUR_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_MINUTE_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_SECOND_FORMAT,2)</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -926,7 +927,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1016,6 +1017,8 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1145,6 +1148,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1491,225 +1495,225 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="97" t="s">
+      <c r="A1" s="99" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="100" t="s">
+      <c r="B1" s="102" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="101"/>
-      <c r="D1" s="104" t="s">
+      <c r="C1" s="103"/>
+      <c r="D1" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="105"/>
-      <c r="F1" s="105"/>
-      <c r="G1" s="105"/>
-      <c r="H1" s="105"/>
-      <c r="I1" s="106"/>
-      <c r="J1" s="106"/>
-      <c r="K1" s="107"/>
-      <c r="L1" s="115" t="s">
+      <c r="E1" s="107"/>
+      <c r="F1" s="107"/>
+      <c r="G1" s="107"/>
+      <c r="H1" s="107"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="109"/>
+      <c r="L1" s="117" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="104" t="s">
+      <c r="M1" s="118"/>
+      <c r="N1" s="118"/>
+      <c r="O1" s="118"/>
+      <c r="P1" s="118"/>
+      <c r="Q1" s="118"/>
+      <c r="R1" s="118"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="106" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="105"/>
-      <c r="V1" s="105"/>
-      <c r="W1" s="105"/>
-      <c r="X1" s="105"/>
-      <c r="Y1" s="106"/>
-      <c r="Z1" s="106"/>
-      <c r="AA1" s="107"/>
-      <c r="AB1" s="104" t="s">
+      <c r="U1" s="107"/>
+      <c r="V1" s="107"/>
+      <c r="W1" s="107"/>
+      <c r="X1" s="107"/>
+      <c r="Y1" s="108"/>
+      <c r="Z1" s="108"/>
+      <c r="AA1" s="109"/>
+      <c r="AB1" s="106" t="s">
         <v>16</v>
       </c>
-      <c r="AC1" s="105"/>
-      <c r="AD1" s="105"/>
-      <c r="AE1" s="105"/>
-      <c r="AF1" s="105"/>
-      <c r="AG1" s="106"/>
-      <c r="AH1" s="106"/>
-      <c r="AI1" s="107"/>
-      <c r="AJ1" s="104" t="s">
+      <c r="AC1" s="107"/>
+      <c r="AD1" s="107"/>
+      <c r="AE1" s="107"/>
+      <c r="AF1" s="107"/>
+      <c r="AG1" s="108"/>
+      <c r="AH1" s="108"/>
+      <c r="AI1" s="109"/>
+      <c r="AJ1" s="106" t="s">
         <v>18</v>
       </c>
-      <c r="AK1" s="105"/>
-      <c r="AL1" s="105"/>
-      <c r="AM1" s="105"/>
-      <c r="AN1" s="105"/>
-      <c r="AO1" s="106"/>
-      <c r="AP1" s="106"/>
-      <c r="AQ1" s="107"/>
-      <c r="AR1" s="104" t="s">
+      <c r="AK1" s="107"/>
+      <c r="AL1" s="107"/>
+      <c r="AM1" s="107"/>
+      <c r="AN1" s="107"/>
+      <c r="AO1" s="108"/>
+      <c r="AP1" s="108"/>
+      <c r="AQ1" s="109"/>
+      <c r="AR1" s="106" t="s">
         <v>17</v>
       </c>
-      <c r="AS1" s="105"/>
-      <c r="AT1" s="105"/>
-      <c r="AU1" s="105"/>
-      <c r="AV1" s="105"/>
-      <c r="AW1" s="106"/>
-      <c r="AX1" s="106"/>
-      <c r="AY1" s="107"/>
-      <c r="AZ1" s="104" t="s">
+      <c r="AS1" s="107"/>
+      <c r="AT1" s="107"/>
+      <c r="AU1" s="107"/>
+      <c r="AV1" s="107"/>
+      <c r="AW1" s="108"/>
+      <c r="AX1" s="108"/>
+      <c r="AY1" s="109"/>
+      <c r="AZ1" s="106" t="s">
         <v>19</v>
       </c>
-      <c r="BA1" s="105"/>
-      <c r="BB1" s="105"/>
-      <c r="BC1" s="105"/>
-      <c r="BD1" s="105"/>
-      <c r="BE1" s="106"/>
-      <c r="BF1" s="106"/>
-      <c r="BG1" s="107"/>
-      <c r="BH1" s="104" t="s">
+      <c r="BA1" s="107"/>
+      <c r="BB1" s="107"/>
+      <c r="BC1" s="107"/>
+      <c r="BD1" s="107"/>
+      <c r="BE1" s="108"/>
+      <c r="BF1" s="108"/>
+      <c r="BG1" s="109"/>
+      <c r="BH1" s="106" t="s">
         <v>20</v>
       </c>
-      <c r="BI1" s="105"/>
-      <c r="BJ1" s="105"/>
-      <c r="BK1" s="105"/>
-      <c r="BL1" s="105"/>
-      <c r="BM1" s="106"/>
-      <c r="BN1" s="106"/>
-      <c r="BO1" s="107"/>
-      <c r="BP1" s="104" t="s">
+      <c r="BI1" s="107"/>
+      <c r="BJ1" s="107"/>
+      <c r="BK1" s="107"/>
+      <c r="BL1" s="107"/>
+      <c r="BM1" s="108"/>
+      <c r="BN1" s="108"/>
+      <c r="BO1" s="109"/>
+      <c r="BP1" s="106" t="s">
         <v>16</v>
       </c>
-      <c r="BQ1" s="105"/>
-      <c r="BR1" s="105"/>
-      <c r="BS1" s="105"/>
-      <c r="BT1" s="105"/>
-      <c r="BU1" s="106"/>
-      <c r="BV1" s="106"/>
-      <c r="BW1" s="107"/>
-      <c r="BX1" s="104" t="s">
+      <c r="BQ1" s="107"/>
+      <c r="BR1" s="107"/>
+      <c r="BS1" s="107"/>
+      <c r="BT1" s="107"/>
+      <c r="BU1" s="108"/>
+      <c r="BV1" s="108"/>
+      <c r="BW1" s="109"/>
+      <c r="BX1" s="106" t="s">
         <v>18</v>
       </c>
-      <c r="BY1" s="105"/>
-      <c r="BZ1" s="105"/>
-      <c r="CA1" s="105"/>
-      <c r="CB1" s="105"/>
-      <c r="CC1" s="106"/>
-      <c r="CD1" s="106"/>
-      <c r="CE1" s="107"/>
-      <c r="CF1" s="108" t="s">
+      <c r="BY1" s="107"/>
+      <c r="BZ1" s="107"/>
+      <c r="CA1" s="107"/>
+      <c r="CB1" s="107"/>
+      <c r="CC1" s="108"/>
+      <c r="CD1" s="108"/>
+      <c r="CE1" s="109"/>
+      <c r="CF1" s="110" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="98"/>
-      <c r="B2" s="102"/>
-      <c r="C2" s="103"/>
-      <c r="D2" s="111">
+      <c r="A2" s="100"/>
+      <c r="B2" s="104"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="113">
         <v>46083</v>
       </c>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="113"/>
-      <c r="J2" s="113"/>
-      <c r="K2" s="114"/>
-      <c r="L2" s="111">
+      <c r="E2" s="114"/>
+      <c r="F2" s="114"/>
+      <c r="G2" s="114"/>
+      <c r="H2" s="114"/>
+      <c r="I2" s="115"/>
+      <c r="J2" s="115"/>
+      <c r="K2" s="116"/>
+      <c r="L2" s="113">
         <v>46084</v>
       </c>
-      <c r="M2" s="112"/>
-      <c r="N2" s="112"/>
-      <c r="O2" s="112"/>
-      <c r="P2" s="112"/>
-      <c r="Q2" s="113"/>
-      <c r="R2" s="113"/>
-      <c r="S2" s="114"/>
-      <c r="T2" s="111">
+      <c r="M2" s="114"/>
+      <c r="N2" s="114"/>
+      <c r="O2" s="114"/>
+      <c r="P2" s="114"/>
+      <c r="Q2" s="115"/>
+      <c r="R2" s="115"/>
+      <c r="S2" s="116"/>
+      <c r="T2" s="113">
         <v>46085</v>
       </c>
-      <c r="U2" s="112"/>
-      <c r="V2" s="112"/>
-      <c r="W2" s="112"/>
-      <c r="X2" s="112"/>
-      <c r="Y2" s="113"/>
-      <c r="Z2" s="113"/>
-      <c r="AA2" s="114"/>
-      <c r="AB2" s="111">
+      <c r="U2" s="114"/>
+      <c r="V2" s="114"/>
+      <c r="W2" s="114"/>
+      <c r="X2" s="114"/>
+      <c r="Y2" s="115"/>
+      <c r="Z2" s="115"/>
+      <c r="AA2" s="116"/>
+      <c r="AB2" s="113">
         <v>46086</v>
       </c>
-      <c r="AC2" s="112"/>
-      <c r="AD2" s="112"/>
-      <c r="AE2" s="112"/>
-      <c r="AF2" s="112"/>
-      <c r="AG2" s="113"/>
-      <c r="AH2" s="113"/>
-      <c r="AI2" s="114"/>
-      <c r="AJ2" s="111">
+      <c r="AC2" s="114"/>
+      <c r="AD2" s="114"/>
+      <c r="AE2" s="114"/>
+      <c r="AF2" s="114"/>
+      <c r="AG2" s="115"/>
+      <c r="AH2" s="115"/>
+      <c r="AI2" s="116"/>
+      <c r="AJ2" s="113">
         <v>46087</v>
       </c>
-      <c r="AK2" s="112"/>
-      <c r="AL2" s="112"/>
-      <c r="AM2" s="112"/>
-      <c r="AN2" s="112"/>
-      <c r="AO2" s="113"/>
-      <c r="AP2" s="113"/>
-      <c r="AQ2" s="114"/>
-      <c r="AR2" s="111">
+      <c r="AK2" s="114"/>
+      <c r="AL2" s="114"/>
+      <c r="AM2" s="114"/>
+      <c r="AN2" s="114"/>
+      <c r="AO2" s="115"/>
+      <c r="AP2" s="115"/>
+      <c r="AQ2" s="116"/>
+      <c r="AR2" s="113">
         <v>46090</v>
       </c>
-      <c r="AS2" s="112"/>
-      <c r="AT2" s="112"/>
-      <c r="AU2" s="112"/>
-      <c r="AV2" s="112"/>
-      <c r="AW2" s="113"/>
-      <c r="AX2" s="113"/>
-      <c r="AY2" s="114"/>
-      <c r="AZ2" s="111">
+      <c r="AS2" s="114"/>
+      <c r="AT2" s="114"/>
+      <c r="AU2" s="114"/>
+      <c r="AV2" s="114"/>
+      <c r="AW2" s="115"/>
+      <c r="AX2" s="115"/>
+      <c r="AY2" s="116"/>
+      <c r="AZ2" s="113">
         <v>46091</v>
       </c>
-      <c r="BA2" s="112"/>
-      <c r="BB2" s="112"/>
-      <c r="BC2" s="112"/>
-      <c r="BD2" s="112"/>
-      <c r="BE2" s="113"/>
-      <c r="BF2" s="113"/>
-      <c r="BG2" s="114"/>
-      <c r="BH2" s="111">
+      <c r="BA2" s="114"/>
+      <c r="BB2" s="114"/>
+      <c r="BC2" s="114"/>
+      <c r="BD2" s="114"/>
+      <c r="BE2" s="115"/>
+      <c r="BF2" s="115"/>
+      <c r="BG2" s="116"/>
+      <c r="BH2" s="113">
         <v>46092</v>
       </c>
-      <c r="BI2" s="112"/>
-      <c r="BJ2" s="112"/>
-      <c r="BK2" s="112"/>
-      <c r="BL2" s="112"/>
-      <c r="BM2" s="113"/>
-      <c r="BN2" s="113"/>
-      <c r="BO2" s="114"/>
-      <c r="BP2" s="111">
+      <c r="BI2" s="114"/>
+      <c r="BJ2" s="114"/>
+      <c r="BK2" s="114"/>
+      <c r="BL2" s="114"/>
+      <c r="BM2" s="115"/>
+      <c r="BN2" s="115"/>
+      <c r="BO2" s="116"/>
+      <c r="BP2" s="113">
         <v>46093</v>
       </c>
-      <c r="BQ2" s="112"/>
-      <c r="BR2" s="112"/>
-      <c r="BS2" s="112"/>
-      <c r="BT2" s="112"/>
-      <c r="BU2" s="113"/>
-      <c r="BV2" s="113"/>
-      <c r="BW2" s="114"/>
-      <c r="BX2" s="111">
+      <c r="BQ2" s="114"/>
+      <c r="BR2" s="114"/>
+      <c r="BS2" s="114"/>
+      <c r="BT2" s="114"/>
+      <c r="BU2" s="115"/>
+      <c r="BV2" s="115"/>
+      <c r="BW2" s="116"/>
+      <c r="BX2" s="113">
         <v>46094</v>
       </c>
-      <c r="BY2" s="112"/>
-      <c r="BZ2" s="112"/>
-      <c r="CA2" s="112"/>
-      <c r="CB2" s="112"/>
-      <c r="CC2" s="113"/>
-      <c r="CD2" s="113"/>
-      <c r="CE2" s="114"/>
-      <c r="CF2" s="109"/>
+      <c r="BY2" s="114"/>
+      <c r="BZ2" s="114"/>
+      <c r="CA2" s="114"/>
+      <c r="CB2" s="114"/>
+      <c r="CC2" s="115"/>
+      <c r="CD2" s="115"/>
+      <c r="CE2" s="116"/>
+      <c r="CF2" s="111"/>
     </row>
     <row r="3" spans="1:92" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="99"/>
+      <c r="A3" s="101"/>
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
@@ -1956,16 +1960,16 @@
       <c r="CE3" s="11">
         <v>8</v>
       </c>
-      <c r="CF3" s="110"/>
+      <c r="CF3" s="112"/>
     </row>
     <row r="4" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="83" t="s">
+      <c r="A4" s="85" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="81">
+      <c r="B4" s="83">
         <v>4</v>
       </c>
-      <c r="C4" s="79">
+      <c r="C4" s="81">
         <v>0.5</v>
       </c>
       <c r="D4" s="12"/>
@@ -2048,16 +2052,16 @@
       <c r="CC4" s="16"/>
       <c r="CD4" s="14"/>
       <c r="CE4" s="53"/>
-      <c r="CF4" s="75"/>
+      <c r="CF4" s="77"/>
       <c r="CH4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="CI4" s="3"/>
     </row>
     <row r="5" spans="1:92" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="90"/>
-      <c r="B5" s="88"/>
-      <c r="C5" s="86"/>
+      <c r="A5" s="92"/>
+      <c r="B5" s="90"/>
+      <c r="C5" s="88"/>
       <c r="D5" s="17"/>
       <c r="E5" s="18"/>
       <c r="F5" s="18"/>
@@ -2138,20 +2142,20 @@
       <c r="CC5" s="26"/>
       <c r="CD5" s="19"/>
       <c r="CE5" s="19"/>
-      <c r="CF5" s="76"/>
+      <c r="CF5" s="78"/>
       <c r="CH5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="CI5" s="5"/>
     </row>
     <row r="6" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A6" s="83" t="s">
+      <c r="A6" s="85" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="81">
+      <c r="B6" s="83">
         <v>2</v>
       </c>
-      <c r="C6" s="79">
+      <c r="C6" s="81">
         <v>2</v>
       </c>
       <c r="D6" s="58"/>
@@ -2234,12 +2238,12 @@
       <c r="CC6" s="26"/>
       <c r="CD6" s="19"/>
       <c r="CE6" s="19"/>
-      <c r="CF6" s="76"/>
+      <c r="CF6" s="78"/>
     </row>
     <row r="7" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A7" s="90"/>
-      <c r="B7" s="88"/>
-      <c r="C7" s="86"/>
+      <c r="A7" s="92"/>
+      <c r="B7" s="90"/>
+      <c r="C7" s="88"/>
       <c r="D7" s="69"/>
       <c r="E7" s="70"/>
       <c r="F7" s="28"/>
@@ -2320,16 +2324,16 @@
       <c r="CC7" s="26"/>
       <c r="CD7" s="19"/>
       <c r="CE7" s="19"/>
-      <c r="CF7" s="76"/>
+      <c r="CF7" s="78"/>
     </row>
     <row r="8" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="83" t="s">
+      <c r="A8" s="85" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="81">
+      <c r="B8" s="83">
         <v>14</v>
       </c>
-      <c r="C8" s="79">
+      <c r="C8" s="81">
         <v>1.5</v>
       </c>
       <c r="D8" s="27"/>
@@ -2412,12 +2416,12 @@
       <c r="CC8" s="26"/>
       <c r="CD8" s="19"/>
       <c r="CE8" s="19"/>
-      <c r="CF8" s="76"/>
+      <c r="CF8" s="78"/>
     </row>
     <row r="9" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="90"/>
-      <c r="B9" s="88"/>
-      <c r="C9" s="86"/>
+      <c r="A9" s="92"/>
+      <c r="B9" s="90"/>
+      <c r="C9" s="88"/>
       <c r="D9" s="27"/>
       <c r="E9" s="28"/>
       <c r="F9" s="70"/>
@@ -2498,16 +2502,16 @@
       <c r="CC9" s="26"/>
       <c r="CD9" s="19"/>
       <c r="CE9" s="19"/>
-      <c r="CF9" s="76"/>
+      <c r="CF9" s="78"/>
     </row>
     <row r="10" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="83" t="s">
+      <c r="A10" s="85" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="81">
+      <c r="B10" s="83">
         <v>1</v>
       </c>
-      <c r="C10" s="79">
+      <c r="C10" s="81">
         <v>1</v>
       </c>
       <c r="D10" s="27"/>
@@ -2590,12 +2594,12 @@
       <c r="CC10" s="26"/>
       <c r="CD10" s="19"/>
       <c r="CE10" s="19"/>
-      <c r="CF10" s="76"/>
+      <c r="CF10" s="78"/>
     </row>
     <row r="11" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="90"/>
-      <c r="B11" s="88"/>
-      <c r="C11" s="86"/>
+      <c r="A11" s="92"/>
+      <c r="B11" s="90"/>
+      <c r="C11" s="88"/>
       <c r="D11" s="27"/>
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
@@ -2676,16 +2680,16 @@
       <c r="CC11" s="26"/>
       <c r="CD11" s="19"/>
       <c r="CE11" s="19"/>
-      <c r="CF11" s="76"/>
+      <c r="CF11" s="78"/>
     </row>
     <row r="12" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A12" s="83" t="s">
+      <c r="A12" s="85" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="81">
+      <c r="B12" s="83">
         <v>3</v>
       </c>
-      <c r="C12" s="79">
+      <c r="C12" s="81">
         <v>0</v>
       </c>
       <c r="D12" s="17"/>
@@ -2768,12 +2772,12 @@
       <c r="CC12" s="26"/>
       <c r="CD12" s="19"/>
       <c r="CE12" s="19"/>
-      <c r="CF12" s="76"/>
+      <c r="CF12" s="78"/>
     </row>
     <row r="13" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="84"/>
-      <c r="B13" s="82"/>
-      <c r="C13" s="80"/>
+      <c r="A13" s="86"/>
+      <c r="B13" s="84"/>
+      <c r="C13" s="82"/>
       <c r="D13" s="29"/>
       <c r="E13" s="30"/>
       <c r="F13" s="30"/>
@@ -2784,7 +2788,7 @@
       <c r="K13" s="32"/>
       <c r="L13" s="29"/>
       <c r="M13" s="30"/>
-      <c r="N13" s="30"/>
+      <c r="N13" s="120"/>
       <c r="O13" s="30"/>
       <c r="P13" s="30"/>
       <c r="Q13" s="31"/>
@@ -2854,16 +2858,16 @@
       <c r="CC13" s="33"/>
       <c r="CD13" s="34"/>
       <c r="CE13" s="31"/>
-      <c r="CF13" s="77"/>
+      <c r="CF13" s="79"/>
     </row>
     <row r="14" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A14" s="89" t="s">
+      <c r="A14" s="91" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="87">
+      <c r="B14" s="89">
         <v>1</v>
       </c>
-      <c r="C14" s="85">
+      <c r="C14" s="87">
         <v>1</v>
       </c>
       <c r="D14" s="35"/>
@@ -2946,14 +2950,14 @@
       <c r="CC14" s="16"/>
       <c r="CD14" s="14"/>
       <c r="CE14" s="14"/>
-      <c r="CF14" s="78" t="s">
+      <c r="CF14" s="80" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="90"/>
-      <c r="B15" s="88"/>
-      <c r="C15" s="86"/>
+      <c r="A15" s="92"/>
+      <c r="B15" s="90"/>
+      <c r="C15" s="88"/>
       <c r="D15" s="17"/>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
@@ -3034,16 +3038,16 @@
       <c r="CC15" s="26"/>
       <c r="CD15" s="19"/>
       <c r="CE15" s="19"/>
-      <c r="CF15" s="76"/>
+      <c r="CF15" s="78"/>
     </row>
     <row r="16" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A16" s="89" t="s">
+      <c r="A16" s="91" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="87">
+      <c r="B16" s="89">
         <v>1</v>
       </c>
-      <c r="C16" s="85">
+      <c r="C16" s="87">
         <v>1</v>
       </c>
       <c r="D16" s="12"/>
@@ -3126,7 +3130,7 @@
       <c r="CC16" s="16"/>
       <c r="CD16" s="14"/>
       <c r="CE16" s="14"/>
-      <c r="CF16" s="78" t="s">
+      <c r="CF16" s="80" t="s">
         <v>7</v>
       </c>
       <c r="CJ16" s="4"/>
@@ -3135,9 +3139,9 @@
       <c r="CN16" s="4"/>
     </row>
     <row r="17" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A17" s="90"/>
-      <c r="B17" s="88"/>
-      <c r="C17" s="86"/>
+      <c r="A17" s="92"/>
+      <c r="B17" s="90"/>
+      <c r="C17" s="88"/>
       <c r="D17" s="17"/>
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
@@ -3218,20 +3222,20 @@
       <c r="CC17" s="26"/>
       <c r="CD17" s="19"/>
       <c r="CE17" s="19"/>
-      <c r="CF17" s="76"/>
+      <c r="CF17" s="78"/>
       <c r="CJ17" s="4"/>
       <c r="CK17" s="4"/>
       <c r="CM17" s="4"/>
       <c r="CN17" s="4"/>
     </row>
     <row r="18" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A18" s="83" t="s">
+      <c r="A18" s="85" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="81">
+      <c r="B18" s="83">
         <v>1</v>
       </c>
-      <c r="C18" s="79">
+      <c r="C18" s="81">
         <v>1</v>
       </c>
       <c r="D18" s="17"/>
@@ -3314,7 +3318,7 @@
       <c r="CC18" s="26"/>
       <c r="CD18" s="19"/>
       <c r="CE18" s="19"/>
-      <c r="CF18" s="76"/>
+      <c r="CF18" s="78"/>
       <c r="CI18" s="4"/>
       <c r="CJ18" s="4"/>
       <c r="CK18" s="4"/>
@@ -3322,9 +3326,9 @@
       <c r="CN18" s="4"/>
     </row>
     <row r="19" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A19" s="90"/>
-      <c r="B19" s="88"/>
-      <c r="C19" s="86"/>
+      <c r="A19" s="92"/>
+      <c r="B19" s="90"/>
+      <c r="C19" s="88"/>
       <c r="D19" s="17"/>
       <c r="E19" s="18"/>
       <c r="F19" s="18"/>
@@ -3405,16 +3409,16 @@
       <c r="CC19" s="26"/>
       <c r="CD19" s="19"/>
       <c r="CE19" s="19"/>
-      <c r="CF19" s="76"/>
+      <c r="CF19" s="78"/>
     </row>
     <row r="20" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="83" t="s">
+      <c r="A20" s="85" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="81">
+      <c r="B20" s="83">
         <v>1.5</v>
       </c>
-      <c r="C20" s="79">
+      <c r="C20" s="81">
         <v>0</v>
       </c>
       <c r="D20" s="17"/>
@@ -3497,13 +3501,13 @@
       <c r="CC20" s="26"/>
       <c r="CD20" s="19"/>
       <c r="CE20" s="19"/>
-      <c r="CF20" s="76"/>
+      <c r="CF20" s="78"/>
       <c r="CJ20" s="4"/>
     </row>
     <row r="21" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="90"/>
-      <c r="B21" s="88"/>
-      <c r="C21" s="86"/>
+      <c r="A21" s="92"/>
+      <c r="B21" s="90"/>
+      <c r="C21" s="88"/>
       <c r="D21" s="17"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -3512,8 +3516,8 @@
       <c r="I21" s="19"/>
       <c r="J21" s="19"/>
       <c r="K21" s="20"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="18"/>
+      <c r="L21" s="75"/>
+      <c r="M21" s="76"/>
       <c r="N21" s="18"/>
       <c r="O21" s="18"/>
       <c r="P21" s="18"/>
@@ -3584,7 +3588,7 @@
       <c r="CC21" s="26"/>
       <c r="CD21" s="19"/>
       <c r="CE21" s="19"/>
-      <c r="CF21" s="76"/>
+      <c r="CF21" s="78"/>
       <c r="CI21" s="4"/>
       <c r="CJ21" s="4"/>
       <c r="CM21" s="4"/>
@@ -3592,13 +3596,13 @@
       <c r="CO21" s="4"/>
     </row>
     <row r="22" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="95" t="s">
+      <c r="A22" s="97" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="81">
+      <c r="B22" s="83">
         <v>1.5</v>
       </c>
-      <c r="C22" s="79">
+      <c r="C22" s="81">
         <v>0</v>
       </c>
       <c r="D22" s="17"/>
@@ -3681,7 +3685,7 @@
       <c r="CC22" s="26"/>
       <c r="CD22" s="19"/>
       <c r="CE22" s="19"/>
-      <c r="CF22" s="76"/>
+      <c r="CF22" s="78"/>
       <c r="CI22" s="4"/>
       <c r="CJ22" s="4"/>
       <c r="CM22" s="4"/>
@@ -3689,9 +3693,9 @@
       <c r="CO22" s="4"/>
     </row>
     <row r="23" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="96"/>
-      <c r="B23" s="88"/>
-      <c r="C23" s="86"/>
+      <c r="A23" s="98"/>
+      <c r="B23" s="90"/>
+      <c r="C23" s="88"/>
       <c r="D23" s="17"/>
       <c r="E23" s="18"/>
       <c r="F23" s="18"/>
@@ -3703,7 +3707,7 @@
       <c r="L23" s="17"/>
       <c r="M23" s="18"/>
       <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
+      <c r="O23" s="71"/>
       <c r="P23" s="18"/>
       <c r="Q23" s="19"/>
       <c r="R23" s="19"/>
@@ -3772,7 +3776,7 @@
       <c r="CC23" s="26"/>
       <c r="CD23" s="19"/>
       <c r="CE23" s="19"/>
-      <c r="CF23" s="76"/>
+      <c r="CF23" s="78"/>
       <c r="CI23" s="4"/>
       <c r="CJ23" s="4"/>
       <c r="CM23" s="4"/>
@@ -3780,13 +3784,13 @@
       <c r="CO23" s="4"/>
     </row>
     <row r="24" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A24" s="83" t="s">
+      <c r="A24" s="85" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="81">
+      <c r="B24" s="83">
         <v>2</v>
       </c>
-      <c r="C24" s="79">
+      <c r="C24" s="81">
         <v>0</v>
       </c>
       <c r="D24" s="17"/>
@@ -3869,7 +3873,7 @@
       <c r="CC24" s="26"/>
       <c r="CD24" s="19"/>
       <c r="CE24" s="19"/>
-      <c r="CF24" s="76"/>
+      <c r="CF24" s="78"/>
       <c r="CJ24" s="4"/>
       <c r="CK24" s="4"/>
       <c r="CM24" s="4"/>
@@ -3877,9 +3881,9 @@
       <c r="CO24" s="4"/>
     </row>
     <row r="25" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="84"/>
-      <c r="B25" s="82"/>
-      <c r="C25" s="80"/>
+      <c r="A25" s="86"/>
+      <c r="B25" s="84"/>
+      <c r="C25" s="82"/>
       <c r="D25" s="37"/>
       <c r="E25" s="38"/>
       <c r="F25" s="38"/>
@@ -3960,19 +3964,19 @@
       <c r="CC25" s="40"/>
       <c r="CD25" s="34"/>
       <c r="CE25" s="34"/>
-      <c r="CF25" s="77"/>
+      <c r="CF25" s="79"/>
       <c r="CK25" s="4"/>
       <c r="CL25" s="4"/>
       <c r="CM25" s="4"/>
     </row>
     <row r="26" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A26" s="89" t="s">
+      <c r="A26" s="91" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="87">
+      <c r="B26" s="89">
         <v>2</v>
       </c>
-      <c r="C26" s="85">
+      <c r="C26" s="87">
         <v>0</v>
       </c>
       <c r="D26" s="12"/>
@@ -4055,14 +4059,14 @@
       <c r="CC26" s="16"/>
       <c r="CD26" s="14"/>
       <c r="CE26" s="14"/>
-      <c r="CF26" s="78" t="s">
+      <c r="CF26" s="80" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="84"/>
-      <c r="B27" s="82"/>
-      <c r="C27" s="80"/>
+      <c r="A27" s="86"/>
+      <c r="B27" s="84"/>
+      <c r="C27" s="82"/>
       <c r="D27" s="37"/>
       <c r="E27" s="38"/>
       <c r="F27" s="38"/>
@@ -4143,16 +4147,16 @@
       <c r="CC27" s="40"/>
       <c r="CD27" s="34"/>
       <c r="CE27" s="34"/>
-      <c r="CF27" s="77"/>
+      <c r="CF27" s="79"/>
     </row>
     <row r="28" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A28" s="89" t="s">
+      <c r="A28" s="91" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="87">
+      <c r="B28" s="89">
         <v>1</v>
       </c>
-      <c r="C28" s="85">
+      <c r="C28" s="87">
         <v>0</v>
       </c>
       <c r="D28" s="12"/>
@@ -4235,14 +4239,14 @@
       <c r="CC28" s="16"/>
       <c r="CD28" s="14"/>
       <c r="CE28" s="14"/>
-      <c r="CF28" s="78" t="s">
+      <c r="CF28" s="80" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A29" s="90"/>
-      <c r="B29" s="88"/>
-      <c r="C29" s="86"/>
+      <c r="A29" s="92"/>
+      <c r="B29" s="90"/>
+      <c r="C29" s="88"/>
       <c r="D29" s="17"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
@@ -4323,16 +4327,16 @@
       <c r="CC29" s="26"/>
       <c r="CD29" s="19"/>
       <c r="CE29" s="19"/>
-      <c r="CF29" s="76"/>
+      <c r="CF29" s="78"/>
     </row>
     <row r="30" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="83" t="s">
+      <c r="A30" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="81">
+      <c r="B30" s="83">
         <v>2</v>
       </c>
-      <c r="C30" s="79">
+      <c r="C30" s="81">
         <v>0</v>
       </c>
       <c r="D30" s="17"/>
@@ -4415,12 +4419,12 @@
       <c r="CC30" s="26"/>
       <c r="CD30" s="19"/>
       <c r="CE30" s="19"/>
-      <c r="CF30" s="76"/>
+      <c r="CF30" s="78"/>
     </row>
     <row r="31" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="90"/>
-      <c r="B31" s="88"/>
-      <c r="C31" s="86"/>
+      <c r="A31" s="92"/>
+      <c r="B31" s="90"/>
+      <c r="C31" s="88"/>
       <c r="D31" s="17"/>
       <c r="E31" s="18"/>
       <c r="F31" s="18"/>
@@ -4501,16 +4505,16 @@
       <c r="CC31" s="26"/>
       <c r="CD31" s="19"/>
       <c r="CE31" s="19"/>
-      <c r="CF31" s="76"/>
+      <c r="CF31" s="78"/>
     </row>
     <row r="32" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A32" s="83" t="s">
+      <c r="A32" s="85" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="81">
+      <c r="B32" s="83">
         <v>4</v>
       </c>
-      <c r="C32" s="79">
+      <c r="C32" s="81">
         <v>0</v>
       </c>
       <c r="D32" s="17"/>
@@ -4593,12 +4597,12 @@
       <c r="CC32" s="26"/>
       <c r="CD32" s="19"/>
       <c r="CE32" s="19"/>
-      <c r="CF32" s="76"/>
+      <c r="CF32" s="78"/>
     </row>
     <row r="33" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A33" s="90"/>
-      <c r="B33" s="88"/>
-      <c r="C33" s="86"/>
+      <c r="A33" s="92"/>
+      <c r="B33" s="90"/>
+      <c r="C33" s="88"/>
       <c r="D33" s="17"/>
       <c r="E33" s="18"/>
       <c r="F33" s="18"/>
@@ -4679,16 +4683,16 @@
       <c r="CC33" s="26"/>
       <c r="CD33" s="19"/>
       <c r="CE33" s="19"/>
-      <c r="CF33" s="76"/>
+      <c r="CF33" s="78"/>
     </row>
     <row r="34" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A34" s="83" t="s">
+      <c r="A34" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="81">
+      <c r="B34" s="83">
         <v>4</v>
       </c>
-      <c r="C34" s="79">
+      <c r="C34" s="81">
         <v>0</v>
       </c>
       <c r="D34" s="17"/>
@@ -4771,12 +4775,12 @@
       <c r="CC34" s="26"/>
       <c r="CD34" s="19"/>
       <c r="CE34" s="19"/>
-      <c r="CF34" s="76"/>
+      <c r="CF34" s="78"/>
     </row>
     <row r="35" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A35" s="90"/>
-      <c r="B35" s="88"/>
-      <c r="C35" s="86"/>
+      <c r="A35" s="92"/>
+      <c r="B35" s="90"/>
+      <c r="C35" s="88"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
       <c r="F35" s="18"/>
@@ -4857,16 +4861,16 @@
       <c r="CC35" s="26"/>
       <c r="CD35" s="19"/>
       <c r="CE35" s="19"/>
-      <c r="CF35" s="76"/>
+      <c r="CF35" s="78"/>
     </row>
     <row r="36" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A36" s="83" t="s">
+      <c r="A36" s="85" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="81">
+      <c r="B36" s="83">
         <v>9</v>
       </c>
-      <c r="C36" s="79">
+      <c r="C36" s="81">
         <v>0</v>
       </c>
       <c r="D36" s="17"/>
@@ -4949,12 +4953,12 @@
       <c r="CC36" s="26"/>
       <c r="CD36" s="19"/>
       <c r="CE36" s="19"/>
-      <c r="CF36" s="76"/>
+      <c r="CF36" s="78"/>
     </row>
     <row r="37" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A37" s="90"/>
-      <c r="B37" s="88"/>
-      <c r="C37" s="86"/>
+      <c r="A37" s="92"/>
+      <c r="B37" s="90"/>
+      <c r="C37" s="88"/>
       <c r="D37" s="17"/>
       <c r="E37" s="18"/>
       <c r="F37" s="18"/>
@@ -5035,16 +5039,16 @@
       <c r="CC37" s="26"/>
       <c r="CD37" s="19"/>
       <c r="CE37" s="19"/>
-      <c r="CF37" s="76"/>
+      <c r="CF37" s="78"/>
     </row>
     <row r="38" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A38" s="93" t="s">
+      <c r="A38" s="95" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="81">
+      <c r="B38" s="83">
         <v>5</v>
       </c>
-      <c r="C38" s="79">
+      <c r="C38" s="81">
         <v>0</v>
       </c>
       <c r="D38" s="17"/>
@@ -5127,12 +5131,12 @@
       <c r="CC38" s="26"/>
       <c r="CD38" s="19"/>
       <c r="CE38" s="19"/>
-      <c r="CF38" s="76"/>
+      <c r="CF38" s="78"/>
     </row>
     <row r="39" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A39" s="94"/>
-      <c r="B39" s="88"/>
-      <c r="C39" s="86"/>
+      <c r="A39" s="96"/>
+      <c r="B39" s="90"/>
+      <c r="C39" s="88"/>
       <c r="D39" s="17"/>
       <c r="E39" s="18"/>
       <c r="F39" s="18"/>
@@ -5213,16 +5217,16 @@
       <c r="CC39" s="26"/>
       <c r="CD39" s="19"/>
       <c r="CE39" s="19"/>
-      <c r="CF39" s="76"/>
+      <c r="CF39" s="78"/>
     </row>
     <row r="40" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A40" s="93" t="s">
+      <c r="A40" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="81">
+      <c r="B40" s="83">
         <v>4</v>
       </c>
-      <c r="C40" s="79">
+      <c r="C40" s="81">
         <v>0</v>
       </c>
       <c r="D40" s="17"/>
@@ -5305,12 +5309,12 @@
       <c r="CC40" s="26"/>
       <c r="CD40" s="19"/>
       <c r="CE40" s="19"/>
-      <c r="CF40" s="76"/>
+      <c r="CF40" s="78"/>
     </row>
     <row r="41" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A41" s="94"/>
-      <c r="B41" s="88"/>
-      <c r="C41" s="86"/>
+      <c r="A41" s="96"/>
+      <c r="B41" s="90"/>
+      <c r="C41" s="88"/>
       <c r="D41" s="17"/>
       <c r="E41" s="18"/>
       <c r="F41" s="18"/>
@@ -5391,16 +5395,16 @@
       <c r="CC41" s="26"/>
       <c r="CD41" s="19"/>
       <c r="CE41" s="19"/>
-      <c r="CF41" s="76"/>
+      <c r="CF41" s="78"/>
     </row>
     <row r="42" spans="1:84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="83" t="s">
+      <c r="A42" s="85" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="81">
+      <c r="B42" s="83">
         <v>2</v>
       </c>
-      <c r="C42" s="79">
+      <c r="C42" s="81">
         <v>0</v>
       </c>
       <c r="D42" s="17"/>
@@ -5483,12 +5487,12 @@
       <c r="CC42" s="26"/>
       <c r="CD42" s="19"/>
       <c r="CE42" s="19"/>
-      <c r="CF42" s="76"/>
+      <c r="CF42" s="78"/>
     </row>
     <row r="43" spans="1:84" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="90"/>
-      <c r="B43" s="88"/>
-      <c r="C43" s="86"/>
+      <c r="A43" s="92"/>
+      <c r="B43" s="90"/>
+      <c r="C43" s="88"/>
       <c r="D43" s="17"/>
       <c r="E43" s="18"/>
       <c r="F43" s="18"/>
@@ -5569,16 +5573,16 @@
       <c r="CC43" s="26"/>
       <c r="CD43" s="19"/>
       <c r="CE43" s="19"/>
-      <c r="CF43" s="76"/>
+      <c r="CF43" s="78"/>
     </row>
     <row r="44" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A44" s="89" t="s">
+      <c r="A44" s="91" t="s">
         <v>22</v>
       </c>
-      <c r="B44" s="87">
+      <c r="B44" s="89">
         <v>5</v>
       </c>
-      <c r="C44" s="85">
+      <c r="C44" s="87">
         <v>0</v>
       </c>
       <c r="D44" s="12"/>
@@ -5661,14 +5665,14 @@
       <c r="CC44" s="16"/>
       <c r="CD44" s="14"/>
       <c r="CE44" s="14"/>
-      <c r="CF44" s="78" t="s">
+      <c r="CF44" s="80" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:84" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="90"/>
-      <c r="B45" s="88"/>
-      <c r="C45" s="86"/>
+      <c r="A45" s="92"/>
+      <c r="B45" s="90"/>
+      <c r="C45" s="88"/>
       <c r="D45" s="17"/>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -5749,16 +5753,16 @@
       <c r="CC45" s="26"/>
       <c r="CD45" s="19"/>
       <c r="CE45" s="19"/>
-      <c r="CF45" s="76"/>
+      <c r="CF45" s="78"/>
     </row>
     <row r="46" spans="1:84" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="83" t="s">
+      <c r="A46" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="81">
+      <c r="B46" s="83">
         <v>3</v>
       </c>
-      <c r="C46" s="79">
+      <c r="C46" s="81">
         <v>0</v>
       </c>
       <c r="D46" s="17"/>
@@ -5841,12 +5845,12 @@
       <c r="CC46" s="26"/>
       <c r="CD46" s="19"/>
       <c r="CE46" s="19"/>
-      <c r="CF46" s="76"/>
+      <c r="CF46" s="78"/>
     </row>
     <row r="47" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="84"/>
-      <c r="B47" s="82"/>
-      <c r="C47" s="80"/>
+      <c r="A47" s="86"/>
+      <c r="B47" s="84"/>
+      <c r="C47" s="82"/>
       <c r="D47" s="37"/>
       <c r="E47" s="38"/>
       <c r="F47" s="38"/>
@@ -5927,16 +5931,16 @@
       <c r="CC47" s="40"/>
       <c r="CD47" s="34"/>
       <c r="CE47" s="34"/>
-      <c r="CF47" s="77"/>
+      <c r="CF47" s="79"/>
     </row>
     <row r="48" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="89" t="s">
+      <c r="A48" s="91" t="s">
         <v>23</v>
       </c>
-      <c r="B48" s="87">
+      <c r="B48" s="89">
         <v>3</v>
       </c>
-      <c r="C48" s="91">
+      <c r="C48" s="93">
         <v>0</v>
       </c>
       <c r="D48" s="43"/>
@@ -6019,14 +6023,14 @@
       <c r="CC48" s="48"/>
       <c r="CD48" s="45"/>
       <c r="CE48" s="48"/>
-      <c r="CF48" s="78" t="s">
+      <c r="CF48" s="80" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="84"/>
-      <c r="B49" s="82"/>
-      <c r="C49" s="92"/>
+      <c r="A49" s="86"/>
+      <c r="B49" s="84"/>
+      <c r="C49" s="94"/>
       <c r="D49" s="37"/>
       <c r="E49" s="34"/>
       <c r="F49" s="34"/>
@@ -6107,16 +6111,16 @@
       <c r="CC49" s="34"/>
       <c r="CD49" s="34"/>
       <c r="CE49" s="39"/>
-      <c r="CF49" s="77"/>
+      <c r="CF49" s="79"/>
     </row>
     <row r="50" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="89" t="s">
+      <c r="A50" s="91" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="87">
+      <c r="B50" s="89">
         <v>5</v>
       </c>
-      <c r="C50" s="91">
+      <c r="C50" s="93">
         <v>0</v>
       </c>
       <c r="D50" s="54"/>
@@ -6199,12 +6203,12 @@
       <c r="CC50" s="65"/>
       <c r="CD50" s="66"/>
       <c r="CE50" s="65"/>
-      <c r="CF50" s="78"/>
+      <c r="CF50" s="80"/>
     </row>
     <row r="51" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="84"/>
-      <c r="B51" s="82"/>
-      <c r="C51" s="92"/>
+      <c r="A51" s="86"/>
+      <c r="B51" s="84"/>
+      <c r="C51" s="94"/>
       <c r="D51" s="17"/>
       <c r="E51" s="19"/>
       <c r="F51" s="19"/>
@@ -6285,7 +6289,7 @@
       <c r="CC51" s="19"/>
       <c r="CD51" s="19"/>
       <c r="CE51" s="20"/>
-      <c r="CF51" s="77"/>
+      <c r="CF51" s="79"/>
     </row>
     <row r="52" spans="1:84" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="49" t="s">

</xml_diff>

<commit_message>
feat: add initial route structure and update documentation
</commit_message>
<xml_diff>
--- a/docs/Squad App Frontend IPA Zeitplan.xlsx
+++ b/docs/Squad App Frontend IPA Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3737EC6-FB80-45CE-89A4-10E01C4F00F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92EAD709-4347-4C64-B885-9BD2CE47605A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-1930" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -927,7 +927,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1149,6 +1149,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2077,7 +2081,7 @@
       <c r="P5" s="18"/>
       <c r="Q5" s="19"/>
       <c r="R5" s="19"/>
-      <c r="S5" s="20"/>
+      <c r="S5" s="74"/>
       <c r="T5" s="21"/>
       <c r="U5" s="22"/>
       <c r="V5" s="22"/>
@@ -2690,7 +2694,7 @@
         <v>3</v>
       </c>
       <c r="C12" s="81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="17"/>
       <c r="E12" s="18"/>
@@ -3419,7 +3423,7 @@
         <v>1.5</v>
       </c>
       <c r="C20" s="81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D20" s="17"/>
       <c r="E20" s="18"/>
@@ -3517,7 +3521,7 @@
       <c r="J21" s="19"/>
       <c r="K21" s="20"/>
       <c r="L21" s="75"/>
-      <c r="M21" s="76"/>
+      <c r="M21" s="123"/>
       <c r="N21" s="18"/>
       <c r="O21" s="18"/>
       <c r="P21" s="18"/>
@@ -3603,7 +3607,7 @@
         <v>1.5</v>
       </c>
       <c r="C22" s="81">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="17"/>
       <c r="E22" s="18"/>
@@ -3705,9 +3709,9 @@
       <c r="J23" s="19"/>
       <c r="K23" s="20"/>
       <c r="L23" s="17"/>
-      <c r="M23" s="18"/>
+      <c r="M23" s="71"/>
       <c r="N23" s="18"/>
-      <c r="O23" s="71"/>
+      <c r="O23" s="18"/>
       <c r="P23" s="18"/>
       <c r="Q23" s="19"/>
       <c r="R23" s="19"/>
@@ -3895,9 +3899,9 @@
       <c r="L25" s="37"/>
       <c r="M25" s="38"/>
       <c r="N25" s="38"/>
-      <c r="O25" s="38"/>
-      <c r="P25" s="38"/>
-      <c r="Q25" s="34"/>
+      <c r="O25" s="121"/>
+      <c r="P25" s="121"/>
+      <c r="Q25" s="124"/>
       <c r="R25" s="34"/>
       <c r="S25" s="39"/>
       <c r="T25" s="37"/>
@@ -4080,8 +4084,8 @@
       <c r="N27" s="38"/>
       <c r="O27" s="38"/>
       <c r="P27" s="38"/>
-      <c r="Q27" s="34"/>
-      <c r="R27" s="34"/>
+      <c r="Q27" s="122"/>
+      <c r="R27" s="122"/>
       <c r="S27" s="39"/>
       <c r="T27" s="37"/>
       <c r="U27" s="38"/>
@@ -4263,7 +4267,7 @@
       <c r="Q29" s="19"/>
       <c r="R29" s="19"/>
       <c r="S29" s="20"/>
-      <c r="T29" s="17"/>
+      <c r="T29" s="76"/>
       <c r="U29" s="18"/>
       <c r="V29" s="18"/>
       <c r="W29" s="18"/>
@@ -6301,7 +6305,7 @@
       </c>
       <c r="C52" s="50">
         <f>SUM(C4:C51)</f>
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="CD52" s="2"/>
       <c r="CE52" s="2"/>

</xml_diff>

<commit_message>
docs: update time table and documentation
</commit_message>
<xml_diff>
--- a/docs/Squad App Frontend IPA Zeitplan.xlsx
+++ b/docs/Squad App Frontend IPA Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92EAD709-4347-4C64-B885-9BD2CE47605A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E57B16F-4CE8-42C7-A47D-FF80ED6BA526}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-1930" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14,7 +14,6 @@
     <definedName name="LOCAL_MYSQL_DATE_FORMAT" hidden="1">REPT(LOCAL_YEAR_FORMAT,4)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_MONTH_FORMAT,2)&amp;LOCAL_DATE_SEPARATOR&amp;REPT(LOCAL_DAY_FORMAT,2)&amp;" "&amp;REPT(LOCAL_HOUR_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_MINUTE_FORMAT,2)&amp;LOCAL_TIME_SEPARATOR&amp;REPT(LOCAL_SECOND_FORMAT,2)</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -927,7 +926,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1019,72 +1018,11 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1148,11 +1086,73 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1499,225 +1499,225 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="99" t="s">
+      <c r="A1" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="102" t="s">
+      <c r="B1" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="103"/>
-      <c r="D1" s="106" t="s">
+      <c r="C1" s="86"/>
+      <c r="D1" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="107"/>
-      <c r="F1" s="107"/>
-      <c r="G1" s="107"/>
-      <c r="H1" s="107"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="109"/>
-      <c r="L1" s="117" t="s">
+      <c r="E1" s="90"/>
+      <c r="F1" s="90"/>
+      <c r="G1" s="90"/>
+      <c r="H1" s="90"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="92"/>
+      <c r="L1" s="100" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
-      <c r="P1" s="118"/>
-      <c r="Q1" s="118"/>
-      <c r="R1" s="118"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="106" t="s">
+      <c r="M1" s="101"/>
+      <c r="N1" s="101"/>
+      <c r="O1" s="101"/>
+      <c r="P1" s="101"/>
+      <c r="Q1" s="101"/>
+      <c r="R1" s="101"/>
+      <c r="S1" s="102"/>
+      <c r="T1" s="89" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="107"/>
-      <c r="V1" s="107"/>
-      <c r="W1" s="107"/>
-      <c r="X1" s="107"/>
-      <c r="Y1" s="108"/>
-      <c r="Z1" s="108"/>
-      <c r="AA1" s="109"/>
-      <c r="AB1" s="106" t="s">
+      <c r="U1" s="90"/>
+      <c r="V1" s="90"/>
+      <c r="W1" s="90"/>
+      <c r="X1" s="90"/>
+      <c r="Y1" s="91"/>
+      <c r="Z1" s="91"/>
+      <c r="AA1" s="92"/>
+      <c r="AB1" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="AC1" s="107"/>
-      <c r="AD1" s="107"/>
-      <c r="AE1" s="107"/>
-      <c r="AF1" s="107"/>
-      <c r="AG1" s="108"/>
-      <c r="AH1" s="108"/>
-      <c r="AI1" s="109"/>
-      <c r="AJ1" s="106" t="s">
+      <c r="AC1" s="90"/>
+      <c r="AD1" s="90"/>
+      <c r="AE1" s="90"/>
+      <c r="AF1" s="90"/>
+      <c r="AG1" s="91"/>
+      <c r="AH1" s="91"/>
+      <c r="AI1" s="92"/>
+      <c r="AJ1" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="AK1" s="107"/>
-      <c r="AL1" s="107"/>
-      <c r="AM1" s="107"/>
-      <c r="AN1" s="107"/>
-      <c r="AO1" s="108"/>
-      <c r="AP1" s="108"/>
-      <c r="AQ1" s="109"/>
-      <c r="AR1" s="106" t="s">
+      <c r="AK1" s="90"/>
+      <c r="AL1" s="90"/>
+      <c r="AM1" s="90"/>
+      <c r="AN1" s="90"/>
+      <c r="AO1" s="91"/>
+      <c r="AP1" s="91"/>
+      <c r="AQ1" s="92"/>
+      <c r="AR1" s="89" t="s">
         <v>17</v>
       </c>
-      <c r="AS1" s="107"/>
-      <c r="AT1" s="107"/>
-      <c r="AU1" s="107"/>
-      <c r="AV1" s="107"/>
-      <c r="AW1" s="108"/>
-      <c r="AX1" s="108"/>
-      <c r="AY1" s="109"/>
-      <c r="AZ1" s="106" t="s">
+      <c r="AS1" s="90"/>
+      <c r="AT1" s="90"/>
+      <c r="AU1" s="90"/>
+      <c r="AV1" s="90"/>
+      <c r="AW1" s="91"/>
+      <c r="AX1" s="91"/>
+      <c r="AY1" s="92"/>
+      <c r="AZ1" s="89" t="s">
         <v>19</v>
       </c>
-      <c r="BA1" s="107"/>
-      <c r="BB1" s="107"/>
-      <c r="BC1" s="107"/>
-      <c r="BD1" s="107"/>
-      <c r="BE1" s="108"/>
-      <c r="BF1" s="108"/>
-      <c r="BG1" s="109"/>
-      <c r="BH1" s="106" t="s">
+      <c r="BA1" s="90"/>
+      <c r="BB1" s="90"/>
+      <c r="BC1" s="90"/>
+      <c r="BD1" s="90"/>
+      <c r="BE1" s="91"/>
+      <c r="BF1" s="91"/>
+      <c r="BG1" s="92"/>
+      <c r="BH1" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="BI1" s="107"/>
-      <c r="BJ1" s="107"/>
-      <c r="BK1" s="107"/>
-      <c r="BL1" s="107"/>
-      <c r="BM1" s="108"/>
-      <c r="BN1" s="108"/>
-      <c r="BO1" s="109"/>
-      <c r="BP1" s="106" t="s">
+      <c r="BI1" s="90"/>
+      <c r="BJ1" s="90"/>
+      <c r="BK1" s="90"/>
+      <c r="BL1" s="90"/>
+      <c r="BM1" s="91"/>
+      <c r="BN1" s="91"/>
+      <c r="BO1" s="92"/>
+      <c r="BP1" s="89" t="s">
         <v>16</v>
       </c>
-      <c r="BQ1" s="107"/>
-      <c r="BR1" s="107"/>
-      <c r="BS1" s="107"/>
-      <c r="BT1" s="107"/>
-      <c r="BU1" s="108"/>
-      <c r="BV1" s="108"/>
-      <c r="BW1" s="109"/>
-      <c r="BX1" s="106" t="s">
+      <c r="BQ1" s="90"/>
+      <c r="BR1" s="90"/>
+      <c r="BS1" s="90"/>
+      <c r="BT1" s="90"/>
+      <c r="BU1" s="91"/>
+      <c r="BV1" s="91"/>
+      <c r="BW1" s="92"/>
+      <c r="BX1" s="89" t="s">
         <v>18</v>
       </c>
-      <c r="BY1" s="107"/>
-      <c r="BZ1" s="107"/>
-      <c r="CA1" s="107"/>
-      <c r="CB1" s="107"/>
-      <c r="CC1" s="108"/>
-      <c r="CD1" s="108"/>
-      <c r="CE1" s="109"/>
-      <c r="CF1" s="110" t="s">
+      <c r="BY1" s="90"/>
+      <c r="BZ1" s="90"/>
+      <c r="CA1" s="90"/>
+      <c r="CB1" s="90"/>
+      <c r="CC1" s="91"/>
+      <c r="CD1" s="91"/>
+      <c r="CE1" s="92"/>
+      <c r="CF1" s="93" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="100"/>
-      <c r="B2" s="104"/>
-      <c r="C2" s="105"/>
-      <c r="D2" s="113">
+      <c r="A2" s="83"/>
+      <c r="B2" s="87"/>
+      <c r="C2" s="88"/>
+      <c r="D2" s="96">
         <v>46083</v>
       </c>
-      <c r="E2" s="114"/>
-      <c r="F2" s="114"/>
-      <c r="G2" s="114"/>
-      <c r="H2" s="114"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="113">
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="98"/>
+      <c r="J2" s="98"/>
+      <c r="K2" s="99"/>
+      <c r="L2" s="96">
         <v>46084</v>
       </c>
-      <c r="M2" s="114"/>
-      <c r="N2" s="114"/>
-      <c r="O2" s="114"/>
-      <c r="P2" s="114"/>
-      <c r="Q2" s="115"/>
-      <c r="R2" s="115"/>
-      <c r="S2" s="116"/>
-      <c r="T2" s="113">
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="97"/>
+      <c r="Q2" s="98"/>
+      <c r="R2" s="98"/>
+      <c r="S2" s="99"/>
+      <c r="T2" s="96">
         <v>46085</v>
       </c>
-      <c r="U2" s="114"/>
-      <c r="V2" s="114"/>
-      <c r="W2" s="114"/>
-      <c r="X2" s="114"/>
-      <c r="Y2" s="115"/>
-      <c r="Z2" s="115"/>
-      <c r="AA2" s="116"/>
-      <c r="AB2" s="113">
+      <c r="U2" s="97"/>
+      <c r="V2" s="97"/>
+      <c r="W2" s="97"/>
+      <c r="X2" s="97"/>
+      <c r="Y2" s="98"/>
+      <c r="Z2" s="98"/>
+      <c r="AA2" s="99"/>
+      <c r="AB2" s="96">
         <v>46086</v>
       </c>
-      <c r="AC2" s="114"/>
-      <c r="AD2" s="114"/>
-      <c r="AE2" s="114"/>
-      <c r="AF2" s="114"/>
-      <c r="AG2" s="115"/>
-      <c r="AH2" s="115"/>
-      <c r="AI2" s="116"/>
-      <c r="AJ2" s="113">
+      <c r="AC2" s="97"/>
+      <c r="AD2" s="97"/>
+      <c r="AE2" s="97"/>
+      <c r="AF2" s="97"/>
+      <c r="AG2" s="98"/>
+      <c r="AH2" s="98"/>
+      <c r="AI2" s="99"/>
+      <c r="AJ2" s="96">
         <v>46087</v>
       </c>
-      <c r="AK2" s="114"/>
-      <c r="AL2" s="114"/>
-      <c r="AM2" s="114"/>
-      <c r="AN2" s="114"/>
-      <c r="AO2" s="115"/>
-      <c r="AP2" s="115"/>
-      <c r="AQ2" s="116"/>
-      <c r="AR2" s="113">
+      <c r="AK2" s="97"/>
+      <c r="AL2" s="97"/>
+      <c r="AM2" s="97"/>
+      <c r="AN2" s="97"/>
+      <c r="AO2" s="98"/>
+      <c r="AP2" s="98"/>
+      <c r="AQ2" s="99"/>
+      <c r="AR2" s="96">
         <v>46090</v>
       </c>
-      <c r="AS2" s="114"/>
-      <c r="AT2" s="114"/>
-      <c r="AU2" s="114"/>
-      <c r="AV2" s="114"/>
-      <c r="AW2" s="115"/>
-      <c r="AX2" s="115"/>
-      <c r="AY2" s="116"/>
-      <c r="AZ2" s="113">
+      <c r="AS2" s="97"/>
+      <c r="AT2" s="97"/>
+      <c r="AU2" s="97"/>
+      <c r="AV2" s="97"/>
+      <c r="AW2" s="98"/>
+      <c r="AX2" s="98"/>
+      <c r="AY2" s="99"/>
+      <c r="AZ2" s="96">
         <v>46091</v>
       </c>
-      <c r="BA2" s="114"/>
-      <c r="BB2" s="114"/>
-      <c r="BC2" s="114"/>
-      <c r="BD2" s="114"/>
-      <c r="BE2" s="115"/>
-      <c r="BF2" s="115"/>
-      <c r="BG2" s="116"/>
-      <c r="BH2" s="113">
+      <c r="BA2" s="97"/>
+      <c r="BB2" s="97"/>
+      <c r="BC2" s="97"/>
+      <c r="BD2" s="97"/>
+      <c r="BE2" s="98"/>
+      <c r="BF2" s="98"/>
+      <c r="BG2" s="99"/>
+      <c r="BH2" s="96">
         <v>46092</v>
       </c>
-      <c r="BI2" s="114"/>
-      <c r="BJ2" s="114"/>
-      <c r="BK2" s="114"/>
-      <c r="BL2" s="114"/>
-      <c r="BM2" s="115"/>
-      <c r="BN2" s="115"/>
-      <c r="BO2" s="116"/>
-      <c r="BP2" s="113">
+      <c r="BI2" s="97"/>
+      <c r="BJ2" s="97"/>
+      <c r="BK2" s="97"/>
+      <c r="BL2" s="97"/>
+      <c r="BM2" s="98"/>
+      <c r="BN2" s="98"/>
+      <c r="BO2" s="99"/>
+      <c r="BP2" s="96">
         <v>46093</v>
       </c>
-      <c r="BQ2" s="114"/>
-      <c r="BR2" s="114"/>
-      <c r="BS2" s="114"/>
-      <c r="BT2" s="114"/>
-      <c r="BU2" s="115"/>
-      <c r="BV2" s="115"/>
-      <c r="BW2" s="116"/>
-      <c r="BX2" s="113">
+      <c r="BQ2" s="97"/>
+      <c r="BR2" s="97"/>
+      <c r="BS2" s="97"/>
+      <c r="BT2" s="97"/>
+      <c r="BU2" s="98"/>
+      <c r="BV2" s="98"/>
+      <c r="BW2" s="99"/>
+      <c r="BX2" s="96">
         <v>46094</v>
       </c>
-      <c r="BY2" s="114"/>
-      <c r="BZ2" s="114"/>
-      <c r="CA2" s="114"/>
-      <c r="CB2" s="114"/>
-      <c r="CC2" s="115"/>
-      <c r="CD2" s="115"/>
-      <c r="CE2" s="116"/>
-      <c r="CF2" s="111"/>
+      <c r="BY2" s="97"/>
+      <c r="BZ2" s="97"/>
+      <c r="CA2" s="97"/>
+      <c r="CB2" s="97"/>
+      <c r="CC2" s="98"/>
+      <c r="CD2" s="98"/>
+      <c r="CE2" s="99"/>
+      <c r="CF2" s="94"/>
     </row>
     <row r="3" spans="1:92" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="101"/>
+      <c r="A3" s="84"/>
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
@@ -1964,16 +1964,16 @@
       <c r="CE3" s="11">
         <v>8</v>
       </c>
-      <c r="CF3" s="112"/>
+      <c r="CF3" s="95"/>
     </row>
     <row r="4" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="85" t="s">
+      <c r="A4" s="109" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="83">
+      <c r="B4" s="105">
         <v>4</v>
       </c>
-      <c r="C4" s="81">
+      <c r="C4" s="107">
         <v>0.5</v>
       </c>
       <c r="D4" s="12"/>
@@ -2056,16 +2056,16 @@
       <c r="CC4" s="16"/>
       <c r="CD4" s="14"/>
       <c r="CE4" s="53"/>
-      <c r="CF4" s="77"/>
+      <c r="CF4" s="124"/>
       <c r="CH4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="CI4" s="3"/>
     </row>
     <row r="5" spans="1:92" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="92"/>
-      <c r="B5" s="90"/>
-      <c r="C5" s="88"/>
+      <c r="A5" s="110"/>
+      <c r="B5" s="106"/>
+      <c r="C5" s="108"/>
       <c r="D5" s="17"/>
       <c r="E5" s="18"/>
       <c r="F5" s="18"/>
@@ -2089,7 +2089,7 @@
       <c r="X5" s="22"/>
       <c r="Y5" s="23"/>
       <c r="Z5" s="18"/>
-      <c r="AA5" s="20"/>
+      <c r="AA5" s="74"/>
       <c r="AB5" s="21"/>
       <c r="AC5" s="22"/>
       <c r="AD5" s="22"/>
@@ -2146,20 +2146,20 @@
       <c r="CC5" s="26"/>
       <c r="CD5" s="19"/>
       <c r="CE5" s="19"/>
-      <c r="CF5" s="78"/>
+      <c r="CF5" s="123"/>
       <c r="CH5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="CI5" s="5"/>
     </row>
     <row r="6" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A6" s="85" t="s">
+      <c r="A6" s="109" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="83">
+      <c r="B6" s="105">
         <v>2</v>
       </c>
-      <c r="C6" s="81">
+      <c r="C6" s="107">
         <v>2</v>
       </c>
       <c r="D6" s="58"/>
@@ -2242,12 +2242,12 @@
       <c r="CC6" s="26"/>
       <c r="CD6" s="19"/>
       <c r="CE6" s="19"/>
-      <c r="CF6" s="78"/>
+      <c r="CF6" s="123"/>
     </row>
     <row r="7" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A7" s="92"/>
-      <c r="B7" s="90"/>
-      <c r="C7" s="88"/>
+      <c r="A7" s="110"/>
+      <c r="B7" s="106"/>
+      <c r="C7" s="108"/>
       <c r="D7" s="69"/>
       <c r="E7" s="70"/>
       <c r="F7" s="28"/>
@@ -2328,16 +2328,16 @@
       <c r="CC7" s="26"/>
       <c r="CD7" s="19"/>
       <c r="CE7" s="19"/>
-      <c r="CF7" s="78"/>
+      <c r="CF7" s="123"/>
     </row>
     <row r="8" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="85" t="s">
+      <c r="A8" s="109" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="83">
+      <c r="B8" s="105">
         <v>14</v>
       </c>
-      <c r="C8" s="81">
+      <c r="C8" s="107">
         <v>1.5</v>
       </c>
       <c r="D8" s="27"/>
@@ -2420,12 +2420,12 @@
       <c r="CC8" s="26"/>
       <c r="CD8" s="19"/>
       <c r="CE8" s="19"/>
-      <c r="CF8" s="78"/>
+      <c r="CF8" s="123"/>
     </row>
     <row r="9" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="92"/>
-      <c r="B9" s="90"/>
-      <c r="C9" s="88"/>
+      <c r="A9" s="110"/>
+      <c r="B9" s="106"/>
+      <c r="C9" s="108"/>
       <c r="D9" s="27"/>
       <c r="E9" s="28"/>
       <c r="F9" s="70"/>
@@ -2448,7 +2448,7 @@
       <c r="W9" s="18"/>
       <c r="X9" s="18"/>
       <c r="Y9" s="19"/>
-      <c r="Z9" s="18"/>
+      <c r="Z9" s="71"/>
       <c r="AA9" s="20"/>
       <c r="AB9" s="17"/>
       <c r="AC9" s="18"/>
@@ -2506,16 +2506,16 @@
       <c r="CC9" s="26"/>
       <c r="CD9" s="19"/>
       <c r="CE9" s="19"/>
-      <c r="CF9" s="78"/>
+      <c r="CF9" s="123"/>
     </row>
     <row r="10" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="85" t="s">
+      <c r="A10" s="109" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="83">
+      <c r="B10" s="105">
         <v>1</v>
       </c>
-      <c r="C10" s="81">
+      <c r="C10" s="107">
         <v>1</v>
       </c>
       <c r="D10" s="27"/>
@@ -2598,12 +2598,12 @@
       <c r="CC10" s="26"/>
       <c r="CD10" s="19"/>
       <c r="CE10" s="19"/>
-      <c r="CF10" s="78"/>
+      <c r="CF10" s="123"/>
     </row>
     <row r="11" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="92"/>
-      <c r="B11" s="90"/>
-      <c r="C11" s="88"/>
+      <c r="A11" s="110"/>
+      <c r="B11" s="106"/>
+      <c r="C11" s="108"/>
       <c r="D11" s="27"/>
       <c r="E11" s="28"/>
       <c r="F11" s="28"/>
@@ -2684,16 +2684,16 @@
       <c r="CC11" s="26"/>
       <c r="CD11" s="19"/>
       <c r="CE11" s="19"/>
-      <c r="CF11" s="78"/>
+      <c r="CF11" s="123"/>
     </row>
     <row r="12" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A12" s="85" t="s">
+      <c r="A12" s="109" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="83">
+      <c r="B12" s="105">
         <v>3</v>
       </c>
-      <c r="C12" s="81">
+      <c r="C12" s="107">
         <v>1</v>
       </c>
       <c r="D12" s="17"/>
@@ -2776,12 +2776,12 @@
       <c r="CC12" s="26"/>
       <c r="CD12" s="19"/>
       <c r="CE12" s="19"/>
-      <c r="CF12" s="78"/>
+      <c r="CF12" s="123"/>
     </row>
     <row r="13" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="86"/>
-      <c r="B13" s="84"/>
-      <c r="C13" s="82"/>
+      <c r="A13" s="112"/>
+      <c r="B13" s="114"/>
+      <c r="C13" s="116"/>
       <c r="D13" s="29"/>
       <c r="E13" s="30"/>
       <c r="F13" s="30"/>
@@ -2792,7 +2792,7 @@
       <c r="K13" s="32"/>
       <c r="L13" s="29"/>
       <c r="M13" s="30"/>
-      <c r="N13" s="120"/>
+      <c r="N13" s="77"/>
       <c r="O13" s="30"/>
       <c r="P13" s="30"/>
       <c r="Q13" s="31"/>
@@ -2862,16 +2862,16 @@
       <c r="CC13" s="33"/>
       <c r="CD13" s="34"/>
       <c r="CE13" s="31"/>
-      <c r="CF13" s="79"/>
+      <c r="CF13" s="122"/>
     </row>
     <row r="14" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A14" s="91" t="s">
+      <c r="A14" s="111" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="89">
+      <c r="B14" s="113">
         <v>1</v>
       </c>
-      <c r="C14" s="87">
+      <c r="C14" s="115">
         <v>1</v>
       </c>
       <c r="D14" s="35"/>
@@ -2954,14 +2954,14 @@
       <c r="CC14" s="16"/>
       <c r="CD14" s="14"/>
       <c r="CE14" s="14"/>
-      <c r="CF14" s="80" t="s">
+      <c r="CF14" s="121" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="92"/>
-      <c r="B15" s="90"/>
-      <c r="C15" s="88"/>
+      <c r="A15" s="110"/>
+      <c r="B15" s="106"/>
+      <c r="C15" s="108"/>
       <c r="D15" s="17"/>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
@@ -3042,16 +3042,16 @@
       <c r="CC15" s="26"/>
       <c r="CD15" s="19"/>
       <c r="CE15" s="19"/>
-      <c r="CF15" s="78"/>
+      <c r="CF15" s="123"/>
     </row>
     <row r="16" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A16" s="91" t="s">
+      <c r="A16" s="111" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="89">
+      <c r="B16" s="113">
         <v>1</v>
       </c>
-      <c r="C16" s="87">
+      <c r="C16" s="115">
         <v>1</v>
       </c>
       <c r="D16" s="12"/>
@@ -3134,7 +3134,7 @@
       <c r="CC16" s="16"/>
       <c r="CD16" s="14"/>
       <c r="CE16" s="14"/>
-      <c r="CF16" s="80" t="s">
+      <c r="CF16" s="121" t="s">
         <v>7</v>
       </c>
       <c r="CJ16" s="4"/>
@@ -3143,9 +3143,9 @@
       <c r="CN16" s="4"/>
     </row>
     <row r="17" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A17" s="92"/>
-      <c r="B17" s="90"/>
-      <c r="C17" s="88"/>
+      <c r="A17" s="110"/>
+      <c r="B17" s="106"/>
+      <c r="C17" s="108"/>
       <c r="D17" s="17"/>
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
@@ -3226,20 +3226,20 @@
       <c r="CC17" s="26"/>
       <c r="CD17" s="19"/>
       <c r="CE17" s="19"/>
-      <c r="CF17" s="78"/>
+      <c r="CF17" s="123"/>
       <c r="CJ17" s="4"/>
       <c r="CK17" s="4"/>
       <c r="CM17" s="4"/>
       <c r="CN17" s="4"/>
     </row>
     <row r="18" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A18" s="85" t="s">
+      <c r="A18" s="109" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="83">
+      <c r="B18" s="105">
         <v>1</v>
       </c>
-      <c r="C18" s="81">
+      <c r="C18" s="107">
         <v>1</v>
       </c>
       <c r="D18" s="17"/>
@@ -3322,7 +3322,7 @@
       <c r="CC18" s="26"/>
       <c r="CD18" s="19"/>
       <c r="CE18" s="19"/>
-      <c r="CF18" s="78"/>
+      <c r="CF18" s="123"/>
       <c r="CI18" s="4"/>
       <c r="CJ18" s="4"/>
       <c r="CK18" s="4"/>
@@ -3330,9 +3330,9 @@
       <c r="CN18" s="4"/>
     </row>
     <row r="19" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A19" s="92"/>
-      <c r="B19" s="90"/>
-      <c r="C19" s="88"/>
+      <c r="A19" s="110"/>
+      <c r="B19" s="106"/>
+      <c r="C19" s="108"/>
       <c r="D19" s="17"/>
       <c r="E19" s="18"/>
       <c r="F19" s="18"/>
@@ -3413,16 +3413,16 @@
       <c r="CC19" s="26"/>
       <c r="CD19" s="19"/>
       <c r="CE19" s="19"/>
-      <c r="CF19" s="78"/>
+      <c r="CF19" s="123"/>
     </row>
     <row r="20" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="85" t="s">
+      <c r="A20" s="109" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="83">
+      <c r="B20" s="105">
         <v>1.5</v>
       </c>
-      <c r="C20" s="81">
+      <c r="C20" s="107">
         <v>1</v>
       </c>
       <c r="D20" s="17"/>
@@ -3505,13 +3505,13 @@
       <c r="CC20" s="26"/>
       <c r="CD20" s="19"/>
       <c r="CE20" s="19"/>
-      <c r="CF20" s="78"/>
+      <c r="CF20" s="123"/>
       <c r="CJ20" s="4"/>
     </row>
     <row r="21" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="92"/>
-      <c r="B21" s="90"/>
-      <c r="C21" s="88"/>
+      <c r="A21" s="110"/>
+      <c r="B21" s="106"/>
+      <c r="C21" s="108"/>
       <c r="D21" s="17"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -3521,7 +3521,7 @@
       <c r="J21" s="19"/>
       <c r="K21" s="20"/>
       <c r="L21" s="75"/>
-      <c r="M21" s="123"/>
+      <c r="M21" s="80"/>
       <c r="N21" s="18"/>
       <c r="O21" s="18"/>
       <c r="P21" s="18"/>
@@ -3592,7 +3592,7 @@
       <c r="CC21" s="26"/>
       <c r="CD21" s="19"/>
       <c r="CE21" s="19"/>
-      <c r="CF21" s="78"/>
+      <c r="CF21" s="123"/>
       <c r="CI21" s="4"/>
       <c r="CJ21" s="4"/>
       <c r="CM21" s="4"/>
@@ -3600,13 +3600,13 @@
       <c r="CO21" s="4"/>
     </row>
     <row r="22" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="97" t="s">
+      <c r="A22" s="117" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="83">
+      <c r="B22" s="105">
         <v>1.5</v>
       </c>
-      <c r="C22" s="81">
+      <c r="C22" s="107">
         <v>1</v>
       </c>
       <c r="D22" s="17"/>
@@ -3689,7 +3689,7 @@
       <c r="CC22" s="26"/>
       <c r="CD22" s="19"/>
       <c r="CE22" s="19"/>
-      <c r="CF22" s="78"/>
+      <c r="CF22" s="123"/>
       <c r="CI22" s="4"/>
       <c r="CJ22" s="4"/>
       <c r="CM22" s="4"/>
@@ -3697,9 +3697,9 @@
       <c r="CO22" s="4"/>
     </row>
     <row r="23" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="98"/>
-      <c r="B23" s="90"/>
-      <c r="C23" s="88"/>
+      <c r="A23" s="118"/>
+      <c r="B23" s="106"/>
+      <c r="C23" s="108"/>
       <c r="D23" s="17"/>
       <c r="E23" s="18"/>
       <c r="F23" s="18"/>
@@ -3780,7 +3780,7 @@
       <c r="CC23" s="26"/>
       <c r="CD23" s="19"/>
       <c r="CE23" s="19"/>
-      <c r="CF23" s="78"/>
+      <c r="CF23" s="123"/>
       <c r="CI23" s="4"/>
       <c r="CJ23" s="4"/>
       <c r="CM23" s="4"/>
@@ -3788,13 +3788,13 @@
       <c r="CO23" s="4"/>
     </row>
     <row r="24" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A24" s="85" t="s">
+      <c r="A24" s="109" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="83">
+      <c r="B24" s="105">
         <v>2</v>
       </c>
-      <c r="C24" s="81">
+      <c r="C24" s="107">
         <v>0</v>
       </c>
       <c r="D24" s="17"/>
@@ -3877,7 +3877,7 @@
       <c r="CC24" s="26"/>
       <c r="CD24" s="19"/>
       <c r="CE24" s="19"/>
-      <c r="CF24" s="78"/>
+      <c r="CF24" s="123"/>
       <c r="CJ24" s="4"/>
       <c r="CK24" s="4"/>
       <c r="CM24" s="4"/>
@@ -3885,9 +3885,9 @@
       <c r="CO24" s="4"/>
     </row>
     <row r="25" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="86"/>
-      <c r="B25" s="84"/>
-      <c r="C25" s="82"/>
+      <c r="A25" s="112"/>
+      <c r="B25" s="114"/>
+      <c r="C25" s="116"/>
       <c r="D25" s="37"/>
       <c r="E25" s="38"/>
       <c r="F25" s="38"/>
@@ -3899,9 +3899,9 @@
       <c r="L25" s="37"/>
       <c r="M25" s="38"/>
       <c r="N25" s="38"/>
-      <c r="O25" s="121"/>
-      <c r="P25" s="121"/>
-      <c r="Q25" s="124"/>
+      <c r="O25" s="78"/>
+      <c r="P25" s="78"/>
+      <c r="Q25" s="81"/>
       <c r="R25" s="34"/>
       <c r="S25" s="39"/>
       <c r="T25" s="37"/>
@@ -3968,19 +3968,19 @@
       <c r="CC25" s="40"/>
       <c r="CD25" s="34"/>
       <c r="CE25" s="34"/>
-      <c r="CF25" s="79"/>
+      <c r="CF25" s="122"/>
       <c r="CK25" s="4"/>
       <c r="CL25" s="4"/>
       <c r="CM25" s="4"/>
     </row>
     <row r="26" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A26" s="91" t="s">
+      <c r="A26" s="111" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="89">
+      <c r="B26" s="113">
         <v>2</v>
       </c>
-      <c r="C26" s="87">
+      <c r="C26" s="115">
         <v>0</v>
       </c>
       <c r="D26" s="12"/>
@@ -4063,14 +4063,14 @@
       <c r="CC26" s="16"/>
       <c r="CD26" s="14"/>
       <c r="CE26" s="14"/>
-      <c r="CF26" s="80" t="s">
+      <c r="CF26" s="121" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="86"/>
-      <c r="B27" s="84"/>
-      <c r="C27" s="82"/>
+      <c r="A27" s="112"/>
+      <c r="B27" s="114"/>
+      <c r="C27" s="116"/>
       <c r="D27" s="37"/>
       <c r="E27" s="38"/>
       <c r="F27" s="38"/>
@@ -4084,8 +4084,8 @@
       <c r="N27" s="38"/>
       <c r="O27" s="38"/>
       <c r="P27" s="38"/>
-      <c r="Q27" s="122"/>
-      <c r="R27" s="122"/>
+      <c r="Q27" s="79"/>
+      <c r="R27" s="79"/>
       <c r="S27" s="39"/>
       <c r="T27" s="37"/>
       <c r="U27" s="38"/>
@@ -4151,16 +4151,16 @@
       <c r="CC27" s="40"/>
       <c r="CD27" s="34"/>
       <c r="CE27" s="34"/>
-      <c r="CF27" s="79"/>
+      <c r="CF27" s="122"/>
     </row>
     <row r="28" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A28" s="91" t="s">
+      <c r="A28" s="111" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="89">
+      <c r="B28" s="113">
         <v>1</v>
       </c>
-      <c r="C28" s="87">
+      <c r="C28" s="115">
         <v>0</v>
       </c>
       <c r="D28" s="12"/>
@@ -4243,14 +4243,14 @@
       <c r="CC28" s="16"/>
       <c r="CD28" s="14"/>
       <c r="CE28" s="14"/>
-      <c r="CF28" s="80" t="s">
+      <c r="CF28" s="121" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A29" s="92"/>
-      <c r="B29" s="90"/>
-      <c r="C29" s="88"/>
+      <c r="A29" s="110"/>
+      <c r="B29" s="106"/>
+      <c r="C29" s="108"/>
       <c r="D29" s="17"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
@@ -4266,8 +4266,8 @@
       <c r="P29" s="18"/>
       <c r="Q29" s="19"/>
       <c r="R29" s="19"/>
-      <c r="S29" s="20"/>
-      <c r="T29" s="76"/>
+      <c r="S29" s="74"/>
+      <c r="T29" s="125"/>
       <c r="U29" s="18"/>
       <c r="V29" s="18"/>
       <c r="W29" s="18"/>
@@ -4331,16 +4331,16 @@
       <c r="CC29" s="26"/>
       <c r="CD29" s="19"/>
       <c r="CE29" s="19"/>
-      <c r="CF29" s="78"/>
+      <c r="CF29" s="123"/>
     </row>
     <row r="30" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="85" t="s">
+      <c r="A30" s="109" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="83">
+      <c r="B30" s="105">
         <v>2</v>
       </c>
-      <c r="C30" s="81">
+      <c r="C30" s="107">
         <v>0</v>
       </c>
       <c r="D30" s="17"/>
@@ -4423,12 +4423,12 @@
       <c r="CC30" s="26"/>
       <c r="CD30" s="19"/>
       <c r="CE30" s="19"/>
-      <c r="CF30" s="78"/>
+      <c r="CF30" s="123"/>
     </row>
     <row r="31" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="92"/>
-      <c r="B31" s="90"/>
-      <c r="C31" s="88"/>
+      <c r="A31" s="110"/>
+      <c r="B31" s="106"/>
+      <c r="C31" s="108"/>
       <c r="D31" s="17"/>
       <c r="E31" s="18"/>
       <c r="F31" s="18"/>
@@ -4445,8 +4445,8 @@
       <c r="Q31" s="19"/>
       <c r="R31" s="19"/>
       <c r="S31" s="20"/>
-      <c r="T31" s="17"/>
-      <c r="U31" s="18"/>
+      <c r="T31" s="76"/>
+      <c r="U31" s="71"/>
       <c r="V31" s="18"/>
       <c r="W31" s="18"/>
       <c r="X31" s="18"/>
@@ -4509,16 +4509,16 @@
       <c r="CC31" s="26"/>
       <c r="CD31" s="19"/>
       <c r="CE31" s="19"/>
-      <c r="CF31" s="78"/>
+      <c r="CF31" s="123"/>
     </row>
     <row r="32" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A32" s="85" t="s">
+      <c r="A32" s="109" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="83">
+      <c r="B32" s="105">
         <v>4</v>
       </c>
-      <c r="C32" s="81">
+      <c r="C32" s="107">
         <v>0</v>
       </c>
       <c r="D32" s="17"/>
@@ -4601,12 +4601,12 @@
       <c r="CC32" s="26"/>
       <c r="CD32" s="19"/>
       <c r="CE32" s="19"/>
-      <c r="CF32" s="78"/>
+      <c r="CF32" s="123"/>
     </row>
     <row r="33" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A33" s="92"/>
-      <c r="B33" s="90"/>
-      <c r="C33" s="88"/>
+      <c r="A33" s="110"/>
+      <c r="B33" s="106"/>
+      <c r="C33" s="108"/>
       <c r="D33" s="17"/>
       <c r="E33" s="18"/>
       <c r="F33" s="18"/>
@@ -4625,10 +4625,10 @@
       <c r="S33" s="20"/>
       <c r="T33" s="17"/>
       <c r="U33" s="18"/>
-      <c r="V33" s="18"/>
-      <c r="W33" s="18"/>
-      <c r="X33" s="18"/>
-      <c r="Y33" s="19"/>
+      <c r="V33" s="71"/>
+      <c r="W33" s="71"/>
+      <c r="X33" s="71"/>
+      <c r="Y33" s="72"/>
       <c r="Z33" s="18"/>
       <c r="AA33" s="20"/>
       <c r="AB33" s="17"/>
@@ -4687,16 +4687,16 @@
       <c r="CC33" s="26"/>
       <c r="CD33" s="19"/>
       <c r="CE33" s="19"/>
-      <c r="CF33" s="78"/>
+      <c r="CF33" s="123"/>
     </row>
     <row r="34" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A34" s="85" t="s">
+      <c r="A34" s="109" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="83">
+      <c r="B34" s="105">
         <v>4</v>
       </c>
-      <c r="C34" s="81">
+      <c r="C34" s="107">
         <v>0</v>
       </c>
       <c r="D34" s="17"/>
@@ -4779,12 +4779,12 @@
       <c r="CC34" s="26"/>
       <c r="CD34" s="19"/>
       <c r="CE34" s="19"/>
-      <c r="CF34" s="78"/>
+      <c r="CF34" s="123"/>
     </row>
     <row r="35" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A35" s="92"/>
-      <c r="B35" s="90"/>
-      <c r="C35" s="88"/>
+      <c r="A35" s="110"/>
+      <c r="B35" s="106"/>
+      <c r="C35" s="108"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
       <c r="F35" s="18"/>
@@ -4808,7 +4808,7 @@
       <c r="X35" s="18"/>
       <c r="Y35" s="19"/>
       <c r="Z35" s="18"/>
-      <c r="AA35" s="20"/>
+      <c r="AA35" s="74"/>
       <c r="AB35" s="17"/>
       <c r="AC35" s="18"/>
       <c r="AD35" s="18"/>
@@ -4865,16 +4865,16 @@
       <c r="CC35" s="26"/>
       <c r="CD35" s="19"/>
       <c r="CE35" s="19"/>
-      <c r="CF35" s="78"/>
+      <c r="CF35" s="123"/>
     </row>
     <row r="36" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A36" s="85" t="s">
+      <c r="A36" s="109" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="83">
+      <c r="B36" s="105">
         <v>9</v>
       </c>
-      <c r="C36" s="81">
+      <c r="C36" s="107">
         <v>0</v>
       </c>
       <c r="D36" s="17"/>
@@ -4957,12 +4957,12 @@
       <c r="CC36" s="26"/>
       <c r="CD36" s="19"/>
       <c r="CE36" s="19"/>
-      <c r="CF36" s="78"/>
+      <c r="CF36" s="123"/>
     </row>
     <row r="37" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A37" s="92"/>
-      <c r="B37" s="90"/>
-      <c r="C37" s="88"/>
+      <c r="A37" s="110"/>
+      <c r="B37" s="106"/>
+      <c r="C37" s="108"/>
       <c r="D37" s="17"/>
       <c r="E37" s="18"/>
       <c r="F37" s="18"/>
@@ -5043,16 +5043,16 @@
       <c r="CC37" s="26"/>
       <c r="CD37" s="19"/>
       <c r="CE37" s="19"/>
-      <c r="CF37" s="78"/>
+      <c r="CF37" s="123"/>
     </row>
     <row r="38" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A38" s="95" t="s">
+      <c r="A38" s="103" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="83">
+      <c r="B38" s="105">
         <v>5</v>
       </c>
-      <c r="C38" s="81">
+      <c r="C38" s="107">
         <v>0</v>
       </c>
       <c r="D38" s="17"/>
@@ -5135,12 +5135,12 @@
       <c r="CC38" s="26"/>
       <c r="CD38" s="19"/>
       <c r="CE38" s="19"/>
-      <c r="CF38" s="78"/>
+      <c r="CF38" s="123"/>
     </row>
     <row r="39" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A39" s="96"/>
-      <c r="B39" s="90"/>
-      <c r="C39" s="88"/>
+      <c r="A39" s="104"/>
+      <c r="B39" s="106"/>
+      <c r="C39" s="108"/>
       <c r="D39" s="17"/>
       <c r="E39" s="18"/>
       <c r="F39" s="18"/>
@@ -5221,16 +5221,16 @@
       <c r="CC39" s="26"/>
       <c r="CD39" s="19"/>
       <c r="CE39" s="19"/>
-      <c r="CF39" s="78"/>
+      <c r="CF39" s="123"/>
     </row>
     <row r="40" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A40" s="95" t="s">
+      <c r="A40" s="103" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="83">
+      <c r="B40" s="105">
         <v>4</v>
       </c>
-      <c r="C40" s="81">
+      <c r="C40" s="107">
         <v>0</v>
       </c>
       <c r="D40" s="17"/>
@@ -5313,12 +5313,12 @@
       <c r="CC40" s="26"/>
       <c r="CD40" s="19"/>
       <c r="CE40" s="19"/>
-      <c r="CF40" s="78"/>
+      <c r="CF40" s="123"/>
     </row>
     <row r="41" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A41" s="96"/>
-      <c r="B41" s="90"/>
-      <c r="C41" s="88"/>
+      <c r="A41" s="104"/>
+      <c r="B41" s="106"/>
+      <c r="C41" s="108"/>
       <c r="D41" s="17"/>
       <c r="E41" s="18"/>
       <c r="F41" s="18"/>
@@ -5399,16 +5399,16 @@
       <c r="CC41" s="26"/>
       <c r="CD41" s="19"/>
       <c r="CE41" s="19"/>
-      <c r="CF41" s="78"/>
+      <c r="CF41" s="123"/>
     </row>
     <row r="42" spans="1:84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="85" t="s">
+      <c r="A42" s="109" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="83">
+      <c r="B42" s="105">
         <v>2</v>
       </c>
-      <c r="C42" s="81">
+      <c r="C42" s="107">
         <v>0</v>
       </c>
       <c r="D42" s="17"/>
@@ -5491,12 +5491,12 @@
       <c r="CC42" s="26"/>
       <c r="CD42" s="19"/>
       <c r="CE42" s="19"/>
-      <c r="CF42" s="78"/>
+      <c r="CF42" s="123"/>
     </row>
     <row r="43" spans="1:84" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="92"/>
-      <c r="B43" s="90"/>
-      <c r="C43" s="88"/>
+      <c r="A43" s="110"/>
+      <c r="B43" s="106"/>
+      <c r="C43" s="108"/>
       <c r="D43" s="17"/>
       <c r="E43" s="18"/>
       <c r="F43" s="18"/>
@@ -5577,16 +5577,16 @@
       <c r="CC43" s="26"/>
       <c r="CD43" s="19"/>
       <c r="CE43" s="19"/>
-      <c r="CF43" s="78"/>
+      <c r="CF43" s="123"/>
     </row>
     <row r="44" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A44" s="91" t="s">
+      <c r="A44" s="111" t="s">
         <v>22</v>
       </c>
-      <c r="B44" s="89">
+      <c r="B44" s="113">
         <v>5</v>
       </c>
-      <c r="C44" s="87">
+      <c r="C44" s="115">
         <v>0</v>
       </c>
       <c r="D44" s="12"/>
@@ -5669,14 +5669,14 @@
       <c r="CC44" s="16"/>
       <c r="CD44" s="14"/>
       <c r="CE44" s="14"/>
-      <c r="CF44" s="80" t="s">
+      <c r="CF44" s="121" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:84" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="92"/>
-      <c r="B45" s="90"/>
-      <c r="C45" s="88"/>
+      <c r="A45" s="110"/>
+      <c r="B45" s="106"/>
+      <c r="C45" s="108"/>
       <c r="D45" s="17"/>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -5757,16 +5757,16 @@
       <c r="CC45" s="26"/>
       <c r="CD45" s="19"/>
       <c r="CE45" s="19"/>
-      <c r="CF45" s="78"/>
+      <c r="CF45" s="123"/>
     </row>
     <row r="46" spans="1:84" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="85" t="s">
+      <c r="A46" s="109" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="83">
+      <c r="B46" s="105">
         <v>3</v>
       </c>
-      <c r="C46" s="81">
+      <c r="C46" s="107">
         <v>0</v>
       </c>
       <c r="D46" s="17"/>
@@ -5849,12 +5849,12 @@
       <c r="CC46" s="26"/>
       <c r="CD46" s="19"/>
       <c r="CE46" s="19"/>
-      <c r="CF46" s="78"/>
+      <c r="CF46" s="123"/>
     </row>
     <row r="47" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="86"/>
-      <c r="B47" s="84"/>
-      <c r="C47" s="82"/>
+      <c r="A47" s="112"/>
+      <c r="B47" s="114"/>
+      <c r="C47" s="116"/>
       <c r="D47" s="37"/>
       <c r="E47" s="38"/>
       <c r="F47" s="38"/>
@@ -5935,16 +5935,16 @@
       <c r="CC47" s="40"/>
       <c r="CD47" s="34"/>
       <c r="CE47" s="34"/>
-      <c r="CF47" s="79"/>
+      <c r="CF47" s="122"/>
     </row>
     <row r="48" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="91" t="s">
+      <c r="A48" s="111" t="s">
         <v>23</v>
       </c>
-      <c r="B48" s="89">
+      <c r="B48" s="113">
         <v>3</v>
       </c>
-      <c r="C48" s="93">
+      <c r="C48" s="119">
         <v>0</v>
       </c>
       <c r="D48" s="43"/>
@@ -6027,14 +6027,14 @@
       <c r="CC48" s="48"/>
       <c r="CD48" s="45"/>
       <c r="CE48" s="48"/>
-      <c r="CF48" s="80" t="s">
+      <c r="CF48" s="121" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="86"/>
-      <c r="B49" s="84"/>
-      <c r="C49" s="94"/>
+      <c r="A49" s="112"/>
+      <c r="B49" s="114"/>
+      <c r="C49" s="120"/>
       <c r="D49" s="37"/>
       <c r="E49" s="34"/>
       <c r="F49" s="34"/>
@@ -6115,16 +6115,16 @@
       <c r="CC49" s="34"/>
       <c r="CD49" s="34"/>
       <c r="CE49" s="39"/>
-      <c r="CF49" s="79"/>
+      <c r="CF49" s="122"/>
     </row>
     <row r="50" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="91" t="s">
+      <c r="A50" s="111" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="89">
+      <c r="B50" s="113">
         <v>5</v>
       </c>
-      <c r="C50" s="93">
+      <c r="C50" s="119">
         <v>0</v>
       </c>
       <c r="D50" s="54"/>
@@ -6207,12 +6207,12 @@
       <c r="CC50" s="65"/>
       <c r="CD50" s="66"/>
       <c r="CE50" s="65"/>
-      <c r="CF50" s="80"/>
+      <c r="CF50" s="121"/>
     </row>
     <row r="51" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="86"/>
-      <c r="B51" s="84"/>
-      <c r="C51" s="94"/>
+      <c r="A51" s="112"/>
+      <c r="B51" s="114"/>
+      <c r="C51" s="120"/>
       <c r="D51" s="17"/>
       <c r="E51" s="19"/>
       <c r="F51" s="19"/>
@@ -6293,7 +6293,7 @@
       <c r="CC51" s="19"/>
       <c r="CD51" s="19"/>
       <c r="CE51" s="20"/>
-      <c r="CF51" s="79"/>
+      <c r="CF51" s="122"/>
     </row>
     <row r="52" spans="1:84" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="49" t="s">
@@ -6343,29 +6343,62 @@
     </row>
   </sheetData>
   <mergeCells count="103">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:C2"/>
-    <mergeCell ref="BP1:BW1"/>
-    <mergeCell ref="BX1:CE1"/>
-    <mergeCell ref="CF1:CF3"/>
-    <mergeCell ref="D2:K2"/>
-    <mergeCell ref="L2:S2"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AJ2:AQ2"/>
-    <mergeCell ref="AR2:AY2"/>
-    <mergeCell ref="AJ1:AQ1"/>
-    <mergeCell ref="AR1:AY1"/>
-    <mergeCell ref="AZ1:BG1"/>
-    <mergeCell ref="BH1:BO1"/>
-    <mergeCell ref="D1:K1"/>
-    <mergeCell ref="L1:S1"/>
-    <mergeCell ref="T1:AA1"/>
-    <mergeCell ref="AB1:AI1"/>
-    <mergeCell ref="AZ2:BG2"/>
-    <mergeCell ref="BH2:BO2"/>
-    <mergeCell ref="BP2:BW2"/>
-    <mergeCell ref="BX2:CE2"/>
+    <mergeCell ref="CF4:CF13"/>
+    <mergeCell ref="CF14:CF15"/>
+    <mergeCell ref="CF16:CF25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A50:A51"/>
+    <mergeCell ref="B50:B51"/>
+    <mergeCell ref="C50:C51"/>
+    <mergeCell ref="A48:A49"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="CF48:CF49"/>
+    <mergeCell ref="CF50:CF51"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="B42:B43"/>
+    <mergeCell ref="C42:C43"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="B44:B45"/>
+    <mergeCell ref="C44:C45"/>
+    <mergeCell ref="CF44:CF47"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="CF26:CF27"/>
+    <mergeCell ref="CF28:CF43"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
     <mergeCell ref="A40:A41"/>
     <mergeCell ref="B40:B41"/>
     <mergeCell ref="C40:C41"/>
@@ -6390,62 +6423,29 @@
     <mergeCell ref="B38:B39"/>
     <mergeCell ref="C38:C39"/>
     <mergeCell ref="C34:C35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="A50:A51"/>
-    <mergeCell ref="B50:B51"/>
-    <mergeCell ref="C50:C51"/>
-    <mergeCell ref="A48:A49"/>
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="CF48:CF49"/>
-    <mergeCell ref="CF50:CF51"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="B42:B43"/>
-    <mergeCell ref="C42:C43"/>
-    <mergeCell ref="A44:A45"/>
-    <mergeCell ref="B44:B45"/>
-    <mergeCell ref="C44:C45"/>
-    <mergeCell ref="CF44:CF47"/>
-    <mergeCell ref="A46:A47"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="CF26:CF27"/>
-    <mergeCell ref="CF28:CF43"/>
-    <mergeCell ref="A32:A33"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="CF4:CF13"/>
-    <mergeCell ref="CF14:CF15"/>
-    <mergeCell ref="CF16:CF25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:C2"/>
+    <mergeCell ref="BP1:BW1"/>
+    <mergeCell ref="BX1:CE1"/>
+    <mergeCell ref="CF1:CF3"/>
+    <mergeCell ref="D2:K2"/>
+    <mergeCell ref="L2:S2"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AJ2:AQ2"/>
+    <mergeCell ref="AR2:AY2"/>
+    <mergeCell ref="AJ1:AQ1"/>
+    <mergeCell ref="AR1:AY1"/>
+    <mergeCell ref="AZ1:BG1"/>
+    <mergeCell ref="BH1:BO1"/>
+    <mergeCell ref="D1:K1"/>
+    <mergeCell ref="L1:S1"/>
+    <mergeCell ref="T1:AA1"/>
+    <mergeCell ref="AB1:AI1"/>
+    <mergeCell ref="AZ2:BG2"/>
+    <mergeCell ref="BH2:BO2"/>
+    <mergeCell ref="BP2:BW2"/>
+    <mergeCell ref="BX2:CE2"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6463,6 +6463,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101000E5D27F8F9D77246958595755BE80D85" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="523cc66e991d1db8e1b1ff070bf6a3d3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="17b83e7a-435f-4364-88cb-373732b2cb78" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b191d266e13279e8e3bfd50054307905" ns2:_="">
     <xsd:import namespace="17b83e7a-435f-4364-88cb-373732b2cb78"/>
@@ -6600,12 +6606,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10E482C8-652F-469A-8C0D-A272F20BD8F0}">
   <ds:schemaRefs>
@@ -6615,6 +6615,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26B24723-3DEB-4B9B-91AB-D29006D23A51}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="17b83e7a-435f-4364-88cb-373732b2cb78"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627A0659-6CE6-4668-B0C2-81E0CF5BEAC7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6630,20 +6646,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26B24723-3DEB-4B9B-91AB-D29006D23A51}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="17b83e7a-435f-4364-88cb-373732b2cb78"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat: add squad management overview page
</commit_message>
<xml_diff>
--- a/docs/Squad App Frontend IPA Zeitplan.xlsx
+++ b/docs/Squad App Frontend IPA Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E247AF14-2C6E-4C5E-9AA7-3C62D25BC79A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19960A42-4519-4719-A676-75F63376E969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-1930" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -965,7 +965,6 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1152,6 +1151,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1498,225 +1498,225 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="104" t="s">
+      <c r="A1" s="103" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="107" t="s">
+      <c r="B1" s="106" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="108"/>
-      <c r="D1" s="111" t="s">
+      <c r="C1" s="107"/>
+      <c r="D1" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="113"/>
-      <c r="J1" s="113"/>
-      <c r="K1" s="114"/>
-      <c r="L1" s="122" t="s">
+      <c r="E1" s="111"/>
+      <c r="F1" s="111"/>
+      <c r="G1" s="111"/>
+      <c r="H1" s="111"/>
+      <c r="I1" s="112"/>
+      <c r="J1" s="112"/>
+      <c r="K1" s="113"/>
+      <c r="L1" s="121" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="123"/>
-      <c r="N1" s="123"/>
-      <c r="O1" s="123"/>
-      <c r="P1" s="123"/>
-      <c r="Q1" s="123"/>
-      <c r="R1" s="123"/>
-      <c r="S1" s="124"/>
-      <c r="T1" s="111" t="s">
+      <c r="M1" s="122"/>
+      <c r="N1" s="122"/>
+      <c r="O1" s="122"/>
+      <c r="P1" s="122"/>
+      <c r="Q1" s="122"/>
+      <c r="R1" s="122"/>
+      <c r="S1" s="123"/>
+      <c r="T1" s="110" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="112"/>
-      <c r="V1" s="112"/>
-      <c r="W1" s="112"/>
-      <c r="X1" s="112"/>
-      <c r="Y1" s="113"/>
-      <c r="Z1" s="113"/>
-      <c r="AA1" s="114"/>
-      <c r="AB1" s="111" t="s">
+      <c r="U1" s="111"/>
+      <c r="V1" s="111"/>
+      <c r="W1" s="111"/>
+      <c r="X1" s="111"/>
+      <c r="Y1" s="112"/>
+      <c r="Z1" s="112"/>
+      <c r="AA1" s="113"/>
+      <c r="AB1" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="AC1" s="112"/>
-      <c r="AD1" s="112"/>
-      <c r="AE1" s="112"/>
-      <c r="AF1" s="112"/>
-      <c r="AG1" s="113"/>
-      <c r="AH1" s="113"/>
-      <c r="AI1" s="114"/>
-      <c r="AJ1" s="111" t="s">
+      <c r="AC1" s="111"/>
+      <c r="AD1" s="111"/>
+      <c r="AE1" s="111"/>
+      <c r="AF1" s="111"/>
+      <c r="AG1" s="112"/>
+      <c r="AH1" s="112"/>
+      <c r="AI1" s="113"/>
+      <c r="AJ1" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="AK1" s="112"/>
-      <c r="AL1" s="112"/>
-      <c r="AM1" s="112"/>
-      <c r="AN1" s="112"/>
-      <c r="AO1" s="113"/>
-      <c r="AP1" s="113"/>
-      <c r="AQ1" s="114"/>
-      <c r="AR1" s="111" t="s">
+      <c r="AK1" s="111"/>
+      <c r="AL1" s="111"/>
+      <c r="AM1" s="111"/>
+      <c r="AN1" s="111"/>
+      <c r="AO1" s="112"/>
+      <c r="AP1" s="112"/>
+      <c r="AQ1" s="113"/>
+      <c r="AR1" s="110" t="s">
         <v>17</v>
       </c>
-      <c r="AS1" s="112"/>
-      <c r="AT1" s="112"/>
-      <c r="AU1" s="112"/>
-      <c r="AV1" s="112"/>
-      <c r="AW1" s="113"/>
-      <c r="AX1" s="113"/>
-      <c r="AY1" s="114"/>
-      <c r="AZ1" s="111" t="s">
+      <c r="AS1" s="111"/>
+      <c r="AT1" s="111"/>
+      <c r="AU1" s="111"/>
+      <c r="AV1" s="111"/>
+      <c r="AW1" s="112"/>
+      <c r="AX1" s="112"/>
+      <c r="AY1" s="113"/>
+      <c r="AZ1" s="110" t="s">
         <v>19</v>
       </c>
-      <c r="BA1" s="112"/>
-      <c r="BB1" s="112"/>
-      <c r="BC1" s="112"/>
-      <c r="BD1" s="112"/>
-      <c r="BE1" s="113"/>
-      <c r="BF1" s="113"/>
-      <c r="BG1" s="114"/>
-      <c r="BH1" s="111" t="s">
+      <c r="BA1" s="111"/>
+      <c r="BB1" s="111"/>
+      <c r="BC1" s="111"/>
+      <c r="BD1" s="111"/>
+      <c r="BE1" s="112"/>
+      <c r="BF1" s="112"/>
+      <c r="BG1" s="113"/>
+      <c r="BH1" s="110" t="s">
         <v>20</v>
       </c>
-      <c r="BI1" s="112"/>
-      <c r="BJ1" s="112"/>
-      <c r="BK1" s="112"/>
-      <c r="BL1" s="112"/>
-      <c r="BM1" s="113"/>
-      <c r="BN1" s="113"/>
-      <c r="BO1" s="114"/>
-      <c r="BP1" s="111" t="s">
+      <c r="BI1" s="111"/>
+      <c r="BJ1" s="111"/>
+      <c r="BK1" s="111"/>
+      <c r="BL1" s="111"/>
+      <c r="BM1" s="112"/>
+      <c r="BN1" s="112"/>
+      <c r="BO1" s="113"/>
+      <c r="BP1" s="110" t="s">
         <v>16</v>
       </c>
-      <c r="BQ1" s="112"/>
-      <c r="BR1" s="112"/>
-      <c r="BS1" s="112"/>
-      <c r="BT1" s="112"/>
-      <c r="BU1" s="113"/>
-      <c r="BV1" s="113"/>
-      <c r="BW1" s="114"/>
-      <c r="BX1" s="111" t="s">
+      <c r="BQ1" s="111"/>
+      <c r="BR1" s="111"/>
+      <c r="BS1" s="111"/>
+      <c r="BT1" s="111"/>
+      <c r="BU1" s="112"/>
+      <c r="BV1" s="112"/>
+      <c r="BW1" s="113"/>
+      <c r="BX1" s="110" t="s">
         <v>18</v>
       </c>
-      <c r="BY1" s="112"/>
-      <c r="BZ1" s="112"/>
-      <c r="CA1" s="112"/>
-      <c r="CB1" s="112"/>
-      <c r="CC1" s="113"/>
-      <c r="CD1" s="113"/>
-      <c r="CE1" s="114"/>
-      <c r="CF1" s="115" t="s">
+      <c r="BY1" s="111"/>
+      <c r="BZ1" s="111"/>
+      <c r="CA1" s="111"/>
+      <c r="CB1" s="111"/>
+      <c r="CC1" s="112"/>
+      <c r="CD1" s="112"/>
+      <c r="CE1" s="113"/>
+      <c r="CF1" s="114" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="105"/>
-      <c r="B2" s="109"/>
-      <c r="C2" s="110"/>
-      <c r="D2" s="118">
+      <c r="A2" s="104"/>
+      <c r="B2" s="108"/>
+      <c r="C2" s="109"/>
+      <c r="D2" s="117">
         <v>46083</v>
       </c>
-      <c r="E2" s="119"/>
-      <c r="F2" s="119"/>
-      <c r="G2" s="119"/>
-      <c r="H2" s="119"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="121"/>
-      <c r="L2" s="118">
+      <c r="E2" s="118"/>
+      <c r="F2" s="118"/>
+      <c r="G2" s="118"/>
+      <c r="H2" s="118"/>
+      <c r="I2" s="119"/>
+      <c r="J2" s="119"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="117">
         <v>46084</v>
       </c>
-      <c r="M2" s="119"/>
-      <c r="N2" s="119"/>
-      <c r="O2" s="119"/>
-      <c r="P2" s="119"/>
-      <c r="Q2" s="120"/>
-      <c r="R2" s="120"/>
-      <c r="S2" s="121"/>
-      <c r="T2" s="118">
+      <c r="M2" s="118"/>
+      <c r="N2" s="118"/>
+      <c r="O2" s="118"/>
+      <c r="P2" s="118"/>
+      <c r="Q2" s="119"/>
+      <c r="R2" s="119"/>
+      <c r="S2" s="120"/>
+      <c r="T2" s="117">
         <v>46085</v>
       </c>
-      <c r="U2" s="119"/>
-      <c r="V2" s="119"/>
-      <c r="W2" s="119"/>
-      <c r="X2" s="119"/>
-      <c r="Y2" s="120"/>
-      <c r="Z2" s="120"/>
-      <c r="AA2" s="121"/>
-      <c r="AB2" s="118">
+      <c r="U2" s="118"/>
+      <c r="V2" s="118"/>
+      <c r="W2" s="118"/>
+      <c r="X2" s="118"/>
+      <c r="Y2" s="119"/>
+      <c r="Z2" s="119"/>
+      <c r="AA2" s="120"/>
+      <c r="AB2" s="117">
         <v>46086</v>
       </c>
-      <c r="AC2" s="119"/>
-      <c r="AD2" s="119"/>
-      <c r="AE2" s="119"/>
-      <c r="AF2" s="119"/>
-      <c r="AG2" s="120"/>
-      <c r="AH2" s="120"/>
-      <c r="AI2" s="121"/>
-      <c r="AJ2" s="118">
+      <c r="AC2" s="118"/>
+      <c r="AD2" s="118"/>
+      <c r="AE2" s="118"/>
+      <c r="AF2" s="118"/>
+      <c r="AG2" s="119"/>
+      <c r="AH2" s="119"/>
+      <c r="AI2" s="120"/>
+      <c r="AJ2" s="117">
         <v>46087</v>
       </c>
-      <c r="AK2" s="119"/>
-      <c r="AL2" s="119"/>
-      <c r="AM2" s="119"/>
-      <c r="AN2" s="119"/>
-      <c r="AO2" s="120"/>
-      <c r="AP2" s="120"/>
-      <c r="AQ2" s="121"/>
-      <c r="AR2" s="118">
+      <c r="AK2" s="118"/>
+      <c r="AL2" s="118"/>
+      <c r="AM2" s="118"/>
+      <c r="AN2" s="118"/>
+      <c r="AO2" s="119"/>
+      <c r="AP2" s="119"/>
+      <c r="AQ2" s="120"/>
+      <c r="AR2" s="117">
         <v>46090</v>
       </c>
-      <c r="AS2" s="119"/>
-      <c r="AT2" s="119"/>
-      <c r="AU2" s="119"/>
-      <c r="AV2" s="119"/>
-      <c r="AW2" s="120"/>
-      <c r="AX2" s="120"/>
-      <c r="AY2" s="121"/>
-      <c r="AZ2" s="118">
+      <c r="AS2" s="118"/>
+      <c r="AT2" s="118"/>
+      <c r="AU2" s="118"/>
+      <c r="AV2" s="118"/>
+      <c r="AW2" s="119"/>
+      <c r="AX2" s="119"/>
+      <c r="AY2" s="120"/>
+      <c r="AZ2" s="117">
         <v>46091</v>
       </c>
-      <c r="BA2" s="119"/>
-      <c r="BB2" s="119"/>
-      <c r="BC2" s="119"/>
-      <c r="BD2" s="119"/>
-      <c r="BE2" s="120"/>
-      <c r="BF2" s="120"/>
-      <c r="BG2" s="121"/>
-      <c r="BH2" s="118">
+      <c r="BA2" s="118"/>
+      <c r="BB2" s="118"/>
+      <c r="BC2" s="118"/>
+      <c r="BD2" s="118"/>
+      <c r="BE2" s="119"/>
+      <c r="BF2" s="119"/>
+      <c r="BG2" s="120"/>
+      <c r="BH2" s="117">
         <v>46092</v>
       </c>
-      <c r="BI2" s="119"/>
-      <c r="BJ2" s="119"/>
-      <c r="BK2" s="119"/>
-      <c r="BL2" s="119"/>
-      <c r="BM2" s="120"/>
-      <c r="BN2" s="120"/>
-      <c r="BO2" s="121"/>
-      <c r="BP2" s="118">
+      <c r="BI2" s="118"/>
+      <c r="BJ2" s="118"/>
+      <c r="BK2" s="118"/>
+      <c r="BL2" s="118"/>
+      <c r="BM2" s="119"/>
+      <c r="BN2" s="119"/>
+      <c r="BO2" s="120"/>
+      <c r="BP2" s="117">
         <v>46093</v>
       </c>
-      <c r="BQ2" s="119"/>
-      <c r="BR2" s="119"/>
-      <c r="BS2" s="119"/>
-      <c r="BT2" s="119"/>
-      <c r="BU2" s="120"/>
-      <c r="BV2" s="120"/>
-      <c r="BW2" s="121"/>
-      <c r="BX2" s="118">
+      <c r="BQ2" s="118"/>
+      <c r="BR2" s="118"/>
+      <c r="BS2" s="118"/>
+      <c r="BT2" s="118"/>
+      <c r="BU2" s="119"/>
+      <c r="BV2" s="119"/>
+      <c r="BW2" s="120"/>
+      <c r="BX2" s="117">
         <v>46094</v>
       </c>
-      <c r="BY2" s="119"/>
-      <c r="BZ2" s="119"/>
-      <c r="CA2" s="119"/>
-      <c r="CB2" s="119"/>
-      <c r="CC2" s="120"/>
-      <c r="CD2" s="120"/>
-      <c r="CE2" s="121"/>
-      <c r="CF2" s="116"/>
+      <c r="BY2" s="118"/>
+      <c r="BZ2" s="118"/>
+      <c r="CA2" s="118"/>
+      <c r="CB2" s="118"/>
+      <c r="CC2" s="119"/>
+      <c r="CD2" s="119"/>
+      <c r="CE2" s="120"/>
+      <c r="CF2" s="115"/>
     </row>
     <row r="3" spans="1:92" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="106"/>
+      <c r="A3" s="105"/>
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
@@ -1963,16 +1963,16 @@
       <c r="CE3" s="11">
         <v>8</v>
       </c>
-      <c r="CF3" s="117"/>
+      <c r="CF3" s="116"/>
     </row>
     <row r="4" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="90" t="s">
+      <c r="A4" s="89" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="88">
+      <c r="B4" s="87">
         <v>4</v>
       </c>
-      <c r="C4" s="86">
+      <c r="C4" s="85">
         <v>0.5</v>
       </c>
       <c r="D4" s="12"/>
@@ -1982,7 +1982,7 @@
       <c r="H4" s="13"/>
       <c r="I4" s="14"/>
       <c r="J4" s="14"/>
-      <c r="K4" s="51"/>
+      <c r="K4" s="50"/>
       <c r="L4" s="12"/>
       <c r="M4" s="13"/>
       <c r="N4" s="13"/>
@@ -1990,7 +1990,7 @@
       <c r="P4" s="13"/>
       <c r="Q4" s="14"/>
       <c r="R4" s="14"/>
-      <c r="S4" s="52"/>
+      <c r="S4" s="51"/>
       <c r="T4" s="12"/>
       <c r="U4" s="13"/>
       <c r="V4" s="13"/>
@@ -1998,7 +1998,7 @@
       <c r="X4" s="13"/>
       <c r="Y4" s="14"/>
       <c r="Z4" s="13"/>
-      <c r="AA4" s="52"/>
+      <c r="AA4" s="51"/>
       <c r="AB4" s="12"/>
       <c r="AC4" s="13"/>
       <c r="AD4" s="13"/>
@@ -2006,7 +2006,7 @@
       <c r="AF4" s="13"/>
       <c r="AG4" s="14"/>
       <c r="AH4" s="14"/>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="12"/>
       <c r="AK4" s="13"/>
       <c r="AL4" s="13"/>
@@ -2014,7 +2014,7 @@
       <c r="AN4" s="13"/>
       <c r="AO4" s="14"/>
       <c r="AP4" s="14"/>
-      <c r="AQ4" s="52"/>
+      <c r="AQ4" s="51"/>
       <c r="AR4" s="12"/>
       <c r="AS4" s="13"/>
       <c r="AT4" s="13"/>
@@ -2022,7 +2022,7 @@
       <c r="AV4" s="13"/>
       <c r="AW4" s="14"/>
       <c r="AX4" s="13"/>
-      <c r="AY4" s="52"/>
+      <c r="AY4" s="51"/>
       <c r="AZ4" s="12"/>
       <c r="BA4" s="13"/>
       <c r="BB4" s="13"/>
@@ -2030,7 +2030,7 @@
       <c r="BD4" s="13"/>
       <c r="BE4" s="14"/>
       <c r="BF4" s="14"/>
-      <c r="BG4" s="52"/>
+      <c r="BG4" s="51"/>
       <c r="BH4" s="12"/>
       <c r="BI4" s="13"/>
       <c r="BJ4" s="13"/>
@@ -2038,7 +2038,7 @@
       <c r="BL4" s="13"/>
       <c r="BM4" s="14"/>
       <c r="BN4" s="14"/>
-      <c r="BO4" s="52"/>
+      <c r="BO4" s="51"/>
       <c r="BP4" s="12"/>
       <c r="BQ4" s="13"/>
       <c r="BR4" s="13"/>
@@ -2046,7 +2046,7 @@
       <c r="BT4" s="13"/>
       <c r="BU4" s="14"/>
       <c r="BV4" s="13"/>
-      <c r="BW4" s="52"/>
+      <c r="BW4" s="51"/>
       <c r="BX4" s="12"/>
       <c r="BY4" s="13"/>
       <c r="BZ4" s="13"/>
@@ -2054,17 +2054,17 @@
       <c r="CB4" s="13"/>
       <c r="CC4" s="16"/>
       <c r="CD4" s="14"/>
-      <c r="CE4" s="53"/>
-      <c r="CF4" s="82"/>
+      <c r="CE4" s="52"/>
+      <c r="CF4" s="81"/>
       <c r="CH4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="CI4" s="3"/>
     </row>
     <row r="5" spans="1:92" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="97"/>
-      <c r="B5" s="95"/>
-      <c r="C5" s="93"/>
+      <c r="A5" s="96"/>
+      <c r="B5" s="94"/>
+      <c r="C5" s="92"/>
       <c r="D5" s="17"/>
       <c r="E5" s="18"/>
       <c r="F5" s="18"/>
@@ -2072,7 +2072,7 @@
       <c r="H5" s="18"/>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
-      <c r="K5" s="74"/>
+      <c r="K5" s="73"/>
       <c r="L5" s="17"/>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
@@ -2080,7 +2080,7 @@
       <c r="P5" s="18"/>
       <c r="Q5" s="19"/>
       <c r="R5" s="19"/>
-      <c r="S5" s="74"/>
+      <c r="S5" s="73"/>
       <c r="T5" s="21"/>
       <c r="U5" s="22"/>
       <c r="V5" s="22"/>
@@ -2088,7 +2088,7 @@
       <c r="X5" s="22"/>
       <c r="Y5" s="23"/>
       <c r="Z5" s="18"/>
-      <c r="AA5" s="74"/>
+      <c r="AA5" s="73"/>
       <c r="AB5" s="21"/>
       <c r="AC5" s="22"/>
       <c r="AD5" s="22"/>
@@ -2096,7 +2096,7 @@
       <c r="AF5" s="22"/>
       <c r="AG5" s="23"/>
       <c r="AH5" s="23"/>
-      <c r="AI5" s="24"/>
+      <c r="AI5" s="124"/>
       <c r="AJ5" s="17"/>
       <c r="AK5" s="18"/>
       <c r="AL5" s="18"/>
@@ -2137,32 +2137,32 @@
       <c r="BU5" s="19"/>
       <c r="BV5" s="18"/>
       <c r="BW5" s="20"/>
-      <c r="BX5" s="25"/>
+      <c r="BX5" s="24"/>
       <c r="BY5" s="18"/>
       <c r="BZ5" s="18"/>
       <c r="CA5" s="18"/>
       <c r="CB5" s="18"/>
-      <c r="CC5" s="26"/>
+      <c r="CC5" s="25"/>
       <c r="CD5" s="19"/>
       <c r="CE5" s="19"/>
-      <c r="CF5" s="83"/>
+      <c r="CF5" s="82"/>
       <c r="CH5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="CI5" s="5"/>
     </row>
     <row r="6" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A6" s="90" t="s">
+      <c r="A6" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="88">
+      <c r="B6" s="87">
         <v>2</v>
       </c>
-      <c r="C6" s="86">
+      <c r="C6" s="85">
         <v>2</v>
       </c>
-      <c r="D6" s="58"/>
-      <c r="E6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="56"/>
       <c r="F6" s="18"/>
       <c r="G6" s="18"/>
       <c r="H6" s="18"/>
@@ -2232,26 +2232,26 @@
       <c r="BT6" s="18"/>
       <c r="BU6" s="19"/>
       <c r="BV6" s="18"/>
-      <c r="BW6" s="26"/>
+      <c r="BW6" s="25"/>
       <c r="BX6" s="17"/>
       <c r="BY6" s="18"/>
       <c r="BZ6" s="19"/>
       <c r="CA6" s="19"/>
       <c r="CB6" s="19"/>
-      <c r="CC6" s="26"/>
+      <c r="CC6" s="25"/>
       <c r="CD6" s="19"/>
       <c r="CE6" s="19"/>
-      <c r="CF6" s="83"/>
+      <c r="CF6" s="82"/>
     </row>
     <row r="7" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A7" s="97"/>
-      <c r="B7" s="95"/>
-      <c r="C7" s="93"/>
-      <c r="D7" s="69"/>
-      <c r="E7" s="70"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
+      <c r="A7" s="96"/>
+      <c r="B7" s="94"/>
+      <c r="C7" s="92"/>
+      <c r="D7" s="68"/>
+      <c r="E7" s="69"/>
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="27"/>
       <c r="I7" s="19"/>
       <c r="J7" s="19"/>
       <c r="K7" s="20"/>
@@ -2319,34 +2319,34 @@
       <c r="BU7" s="19"/>
       <c r="BV7" s="18"/>
       <c r="BW7" s="20"/>
-      <c r="BX7" s="25"/>
+      <c r="BX7" s="24"/>
       <c r="BY7" s="18"/>
       <c r="BZ7" s="18"/>
       <c r="CA7" s="18"/>
       <c r="CB7" s="18"/>
-      <c r="CC7" s="26"/>
+      <c r="CC7" s="25"/>
       <c r="CD7" s="19"/>
       <c r="CE7" s="19"/>
-      <c r="CF7" s="83"/>
+      <c r="CF7" s="82"/>
     </row>
     <row r="8" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="90" t="s">
+      <c r="A8" s="89" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="88">
+      <c r="B8" s="87">
         <v>14</v>
       </c>
-      <c r="C8" s="86">
+      <c r="C8" s="85">
         <v>1.5</v>
       </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="59"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="58"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
-      <c r="K8" s="63"/>
+      <c r="K8" s="62"/>
       <c r="L8" s="17"/>
       <c r="M8" s="18"/>
       <c r="N8" s="18"/>
@@ -2362,13 +2362,13 @@
       <c r="X8" s="18"/>
       <c r="Y8" s="19"/>
       <c r="Z8" s="18"/>
-      <c r="AA8" s="63"/>
+      <c r="AA8" s="62"/>
       <c r="AB8" s="17"/>
       <c r="AC8" s="18"/>
       <c r="AD8" s="18"/>
       <c r="AE8" s="18"/>
-      <c r="AF8" s="57"/>
-      <c r="AG8" s="61"/>
+      <c r="AF8" s="56"/>
+      <c r="AG8" s="60"/>
       <c r="AH8" s="19"/>
       <c r="AI8" s="20"/>
       <c r="AJ8" s="17"/>
@@ -2378,31 +2378,31 @@
       <c r="AN8" s="18"/>
       <c r="AO8" s="19"/>
       <c r="AP8" s="19"/>
-      <c r="AQ8" s="63"/>
-      <c r="AR8" s="58"/>
-      <c r="AS8" s="57"/>
+      <c r="AQ8" s="62"/>
+      <c r="AR8" s="57"/>
+      <c r="AS8" s="56"/>
       <c r="AT8" s="18"/>
       <c r="AU8" s="18"/>
       <c r="AV8" s="18"/>
       <c r="AW8" s="19"/>
       <c r="AX8" s="18"/>
       <c r="AY8" s="20"/>
-      <c r="AZ8" s="58"/>
-      <c r="BA8" s="57"/>
+      <c r="AZ8" s="57"/>
+      <c r="BA8" s="56"/>
       <c r="BB8" s="18"/>
       <c r="BC8" s="18"/>
       <c r="BD8" s="18"/>
       <c r="BE8" s="19"/>
-      <c r="BF8" s="61"/>
-      <c r="BG8" s="63"/>
+      <c r="BF8" s="60"/>
+      <c r="BG8" s="62"/>
       <c r="BH8" s="17"/>
       <c r="BI8" s="18"/>
       <c r="BJ8" s="18"/>
       <c r="BK8" s="18"/>
       <c r="BL8" s="18"/>
-      <c r="BM8" s="61"/>
-      <c r="BN8" s="61"/>
-      <c r="BO8" s="63"/>
+      <c r="BM8" s="60"/>
+      <c r="BN8" s="60"/>
+      <c r="BO8" s="62"/>
       <c r="BP8" s="17"/>
       <c r="BQ8" s="18"/>
       <c r="BR8" s="18"/>
@@ -2411,28 +2411,28 @@
       <c r="BU8" s="19"/>
       <c r="BV8" s="18"/>
       <c r="BW8" s="20"/>
-      <c r="BX8" s="25"/>
+      <c r="BX8" s="24"/>
       <c r="BY8" s="18"/>
       <c r="BZ8" s="18"/>
       <c r="CA8" s="18"/>
       <c r="CB8" s="18"/>
-      <c r="CC8" s="26"/>
+      <c r="CC8" s="25"/>
       <c r="CD8" s="19"/>
       <c r="CE8" s="19"/>
-      <c r="CF8" s="83"/>
+      <c r="CF8" s="82"/>
     </row>
     <row r="9" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="97"/>
-      <c r="B9" s="95"/>
-      <c r="C9" s="93"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="28"/>
-      <c r="F9" s="70"/>
-      <c r="G9" s="28"/>
-      <c r="H9" s="28"/>
+      <c r="A9" s="96"/>
+      <c r="B9" s="94"/>
+      <c r="C9" s="92"/>
+      <c r="D9" s="26"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="69"/>
+      <c r="G9" s="27"/>
+      <c r="H9" s="27"/>
       <c r="I9" s="19"/>
       <c r="J9" s="19"/>
-      <c r="K9" s="74"/>
+      <c r="K9" s="73"/>
       <c r="L9" s="17"/>
       <c r="M9" s="18"/>
       <c r="N9" s="18"/>
@@ -2447,13 +2447,13 @@
       <c r="W9" s="18"/>
       <c r="X9" s="18"/>
       <c r="Y9" s="19"/>
-      <c r="Z9" s="71"/>
+      <c r="Z9" s="70"/>
       <c r="AA9" s="20"/>
       <c r="AB9" s="17"/>
       <c r="AC9" s="18"/>
       <c r="AD9" s="18"/>
-      <c r="AE9" s="71"/>
-      <c r="AF9" s="71"/>
+      <c r="AE9" s="70"/>
+      <c r="AF9" s="70"/>
       <c r="AG9" s="19"/>
       <c r="AH9" s="19"/>
       <c r="AI9" s="20"/>
@@ -2497,31 +2497,31 @@
       <c r="BU9" s="19"/>
       <c r="BV9" s="18"/>
       <c r="BW9" s="20"/>
-      <c r="BX9" s="25"/>
+      <c r="BX9" s="24"/>
       <c r="BY9" s="18"/>
       <c r="BZ9" s="18"/>
       <c r="CA9" s="18"/>
       <c r="CB9" s="18"/>
-      <c r="CC9" s="26"/>
+      <c r="CC9" s="25"/>
       <c r="CD9" s="19"/>
       <c r="CE9" s="19"/>
-      <c r="CF9" s="83"/>
+      <c r="CF9" s="82"/>
     </row>
     <row r="10" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="90" t="s">
+      <c r="A10" s="89" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="88">
+      <c r="B10" s="87">
         <v>1</v>
       </c>
-      <c r="C10" s="86">
+      <c r="C10" s="85">
         <v>1</v>
       </c>
-      <c r="D10" s="27"/>
-      <c r="E10" s="28"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="28"/>
+      <c r="D10" s="26"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
+      <c r="G10" s="58"/>
+      <c r="H10" s="27"/>
       <c r="I10" s="19"/>
       <c r="J10" s="19"/>
       <c r="K10" s="20"/>
@@ -2589,25 +2589,25 @@
       <c r="BU10" s="19"/>
       <c r="BV10" s="18"/>
       <c r="BW10" s="20"/>
-      <c r="BX10" s="25"/>
+      <c r="BX10" s="24"/>
       <c r="BY10" s="18"/>
       <c r="BZ10" s="18"/>
       <c r="CA10" s="18"/>
       <c r="CB10" s="18"/>
-      <c r="CC10" s="26"/>
+      <c r="CC10" s="25"/>
       <c r="CD10" s="19"/>
       <c r="CE10" s="19"/>
-      <c r="CF10" s="83"/>
+      <c r="CF10" s="82"/>
     </row>
     <row r="11" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="97"/>
-      <c r="B11" s="95"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="27"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="70"/>
-      <c r="H11" s="28"/>
+      <c r="A11" s="96"/>
+      <c r="B11" s="94"/>
+      <c r="C11" s="92"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="27"/>
+      <c r="F11" s="27"/>
+      <c r="G11" s="69"/>
+      <c r="H11" s="27"/>
       <c r="I11" s="19"/>
       <c r="J11" s="19"/>
       <c r="K11" s="20"/>
@@ -2675,24 +2675,24 @@
       <c r="BU11" s="19"/>
       <c r="BV11" s="18"/>
       <c r="BW11" s="20"/>
-      <c r="BX11" s="25"/>
+      <c r="BX11" s="24"/>
       <c r="BY11" s="18"/>
       <c r="BZ11" s="18"/>
       <c r="CA11" s="18"/>
       <c r="CB11" s="18"/>
-      <c r="CC11" s="26"/>
+      <c r="CC11" s="25"/>
       <c r="CD11" s="19"/>
       <c r="CE11" s="19"/>
-      <c r="CF11" s="83"/>
+      <c r="CF11" s="82"/>
     </row>
     <row r="12" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A12" s="90" t="s">
+      <c r="A12" s="89" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="88">
+      <c r="B12" s="87">
         <v>3</v>
       </c>
-      <c r="C12" s="86">
+      <c r="C12" s="85">
         <v>1</v>
       </c>
       <c r="D12" s="17"/>
@@ -2705,7 +2705,7 @@
       <c r="K12" s="20"/>
       <c r="L12" s="17"/>
       <c r="M12" s="18"/>
-      <c r="N12" s="57"/>
+      <c r="N12" s="56"/>
       <c r="O12" s="18"/>
       <c r="P12" s="18"/>
       <c r="Q12" s="19"/>
@@ -2719,11 +2719,11 @@
       <c r="Y12" s="19"/>
       <c r="Z12" s="18"/>
       <c r="AA12" s="20"/>
-      <c r="AB12" s="27"/>
-      <c r="AC12" s="28"/>
-      <c r="AD12" s="28"/>
-      <c r="AE12" s="28"/>
-      <c r="AF12" s="28"/>
+      <c r="AB12" s="26"/>
+      <c r="AC12" s="27"/>
+      <c r="AD12" s="27"/>
+      <c r="AE12" s="27"/>
+      <c r="AF12" s="27"/>
       <c r="AG12" s="19"/>
       <c r="AH12" s="19"/>
       <c r="AI12" s="20"/>
@@ -2754,8 +2754,8 @@
       <c r="BH12" s="17"/>
       <c r="BI12" s="18"/>
       <c r="BJ12" s="18"/>
-      <c r="BK12" s="57"/>
-      <c r="BL12" s="57"/>
+      <c r="BK12" s="56"/>
+      <c r="BL12" s="56"/>
       <c r="BM12" s="19"/>
       <c r="BN12" s="19"/>
       <c r="BO12" s="20"/>
@@ -2772,112 +2772,112 @@
       <c r="BZ12" s="18"/>
       <c r="CA12" s="18"/>
       <c r="CB12" s="18"/>
-      <c r="CC12" s="26"/>
+      <c r="CC12" s="25"/>
       <c r="CD12" s="19"/>
       <c r="CE12" s="19"/>
-      <c r="CF12" s="83"/>
+      <c r="CF12" s="82"/>
     </row>
     <row r="13" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="91"/>
-      <c r="B13" s="89"/>
-      <c r="C13" s="87"/>
-      <c r="D13" s="29"/>
-      <c r="E13" s="30"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="31"/>
-      <c r="J13" s="31"/>
-      <c r="K13" s="32"/>
-      <c r="L13" s="29"/>
-      <c r="M13" s="30"/>
-      <c r="N13" s="77"/>
-      <c r="O13" s="30"/>
-      <c r="P13" s="30"/>
-      <c r="Q13" s="31"/>
-      <c r="R13" s="31"/>
-      <c r="S13" s="32"/>
-      <c r="T13" s="29"/>
-      <c r="U13" s="30"/>
-      <c r="V13" s="30"/>
-      <c r="W13" s="30"/>
-      <c r="X13" s="30"/>
-      <c r="Y13" s="31"/>
-      <c r="Z13" s="30"/>
-      <c r="AA13" s="32"/>
-      <c r="AB13" s="29"/>
-      <c r="AC13" s="30"/>
-      <c r="AD13" s="30"/>
-      <c r="AE13" s="30"/>
-      <c r="AF13" s="30"/>
-      <c r="AG13" s="31"/>
-      <c r="AH13" s="31"/>
-      <c r="AI13" s="32"/>
-      <c r="AJ13" s="29"/>
-      <c r="AK13" s="30"/>
-      <c r="AL13" s="30"/>
-      <c r="AM13" s="30"/>
-      <c r="AN13" s="30"/>
-      <c r="AO13" s="31"/>
-      <c r="AP13" s="31"/>
-      <c r="AQ13" s="32"/>
-      <c r="AR13" s="29"/>
-      <c r="AS13" s="30"/>
-      <c r="AT13" s="30"/>
-      <c r="AU13" s="30"/>
-      <c r="AV13" s="30"/>
-      <c r="AW13" s="31"/>
-      <c r="AX13" s="30"/>
-      <c r="AY13" s="32"/>
-      <c r="AZ13" s="29"/>
-      <c r="BA13" s="30"/>
-      <c r="BB13" s="30"/>
-      <c r="BC13" s="30"/>
-      <c r="BD13" s="30"/>
-      <c r="BE13" s="31"/>
-      <c r="BF13" s="31"/>
-      <c r="BG13" s="32"/>
-      <c r="BH13" s="29"/>
-      <c r="BI13" s="30"/>
-      <c r="BJ13" s="30"/>
-      <c r="BK13" s="30"/>
-      <c r="BL13" s="30"/>
-      <c r="BM13" s="31"/>
-      <c r="BN13" s="31"/>
-      <c r="BO13" s="32"/>
-      <c r="BP13" s="29"/>
-      <c r="BQ13" s="30"/>
-      <c r="BR13" s="30"/>
-      <c r="BS13" s="30"/>
-      <c r="BT13" s="30"/>
-      <c r="BU13" s="31"/>
-      <c r="BV13" s="30"/>
-      <c r="BW13" s="32"/>
-      <c r="BX13" s="29"/>
-      <c r="BY13" s="30"/>
-      <c r="BZ13" s="30"/>
-      <c r="CA13" s="30"/>
-      <c r="CB13" s="30"/>
-      <c r="CC13" s="33"/>
-      <c r="CD13" s="34"/>
-      <c r="CE13" s="31"/>
-      <c r="CF13" s="84"/>
+      <c r="A13" s="90"/>
+      <c r="B13" s="88"/>
+      <c r="C13" s="86"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="G13" s="29"/>
+      <c r="H13" s="29"/>
+      <c r="I13" s="30"/>
+      <c r="J13" s="30"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="29"/>
+      <c r="N13" s="76"/>
+      <c r="O13" s="29"/>
+      <c r="P13" s="29"/>
+      <c r="Q13" s="30"/>
+      <c r="R13" s="30"/>
+      <c r="S13" s="31"/>
+      <c r="T13" s="28"/>
+      <c r="U13" s="29"/>
+      <c r="V13" s="29"/>
+      <c r="W13" s="29"/>
+      <c r="X13" s="29"/>
+      <c r="Y13" s="30"/>
+      <c r="Z13" s="29"/>
+      <c r="AA13" s="31"/>
+      <c r="AB13" s="28"/>
+      <c r="AC13" s="29"/>
+      <c r="AD13" s="29"/>
+      <c r="AE13" s="29"/>
+      <c r="AF13" s="29"/>
+      <c r="AG13" s="30"/>
+      <c r="AH13" s="30"/>
+      <c r="AI13" s="31"/>
+      <c r="AJ13" s="28"/>
+      <c r="AK13" s="29"/>
+      <c r="AL13" s="29"/>
+      <c r="AM13" s="29"/>
+      <c r="AN13" s="29"/>
+      <c r="AO13" s="30"/>
+      <c r="AP13" s="30"/>
+      <c r="AQ13" s="31"/>
+      <c r="AR13" s="28"/>
+      <c r="AS13" s="29"/>
+      <c r="AT13" s="29"/>
+      <c r="AU13" s="29"/>
+      <c r="AV13" s="29"/>
+      <c r="AW13" s="30"/>
+      <c r="AX13" s="29"/>
+      <c r="AY13" s="31"/>
+      <c r="AZ13" s="28"/>
+      <c r="BA13" s="29"/>
+      <c r="BB13" s="29"/>
+      <c r="BC13" s="29"/>
+      <c r="BD13" s="29"/>
+      <c r="BE13" s="30"/>
+      <c r="BF13" s="30"/>
+      <c r="BG13" s="31"/>
+      <c r="BH13" s="28"/>
+      <c r="BI13" s="29"/>
+      <c r="BJ13" s="29"/>
+      <c r="BK13" s="29"/>
+      <c r="BL13" s="29"/>
+      <c r="BM13" s="30"/>
+      <c r="BN13" s="30"/>
+      <c r="BO13" s="31"/>
+      <c r="BP13" s="28"/>
+      <c r="BQ13" s="29"/>
+      <c r="BR13" s="29"/>
+      <c r="BS13" s="29"/>
+      <c r="BT13" s="29"/>
+      <c r="BU13" s="30"/>
+      <c r="BV13" s="29"/>
+      <c r="BW13" s="31"/>
+      <c r="BX13" s="28"/>
+      <c r="BY13" s="29"/>
+      <c r="BZ13" s="29"/>
+      <c r="CA13" s="29"/>
+      <c r="CB13" s="29"/>
+      <c r="CC13" s="32"/>
+      <c r="CD13" s="33"/>
+      <c r="CE13" s="30"/>
+      <c r="CF13" s="83"/>
     </row>
     <row r="14" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A14" s="96" t="s">
+      <c r="A14" s="95" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="94">
+      <c r="B14" s="93">
         <v>1</v>
       </c>
-      <c r="C14" s="92">
+      <c r="C14" s="91">
         <v>1</v>
       </c>
-      <c r="D14" s="35"/>
-      <c r="E14" s="36"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="60"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="35"/>
+      <c r="F14" s="35"/>
+      <c r="G14" s="35"/>
+      <c r="H14" s="59"/>
       <c r="I14" s="14"/>
       <c r="J14" s="14"/>
       <c r="K14" s="15"/>
@@ -2953,19 +2953,19 @@
       <c r="CC14" s="16"/>
       <c r="CD14" s="14"/>
       <c r="CE14" s="14"/>
-      <c r="CF14" s="85" t="s">
+      <c r="CF14" s="84" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="97"/>
-      <c r="B15" s="95"/>
-      <c r="C15" s="93"/>
+      <c r="A15" s="96"/>
+      <c r="B15" s="94"/>
+      <c r="C15" s="92"/>
       <c r="D15" s="17"/>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
       <c r="G15" s="18"/>
-      <c r="H15" s="71"/>
+      <c r="H15" s="70"/>
       <c r="I15" s="19"/>
       <c r="J15" s="19"/>
       <c r="K15" s="20"/>
@@ -3038,19 +3038,19 @@
       <c r="BZ15" s="18"/>
       <c r="CA15" s="18"/>
       <c r="CB15" s="18"/>
-      <c r="CC15" s="26"/>
+      <c r="CC15" s="25"/>
       <c r="CD15" s="19"/>
       <c r="CE15" s="19"/>
-      <c r="CF15" s="83"/>
+      <c r="CF15" s="82"/>
     </row>
     <row r="16" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A16" s="96" t="s">
+      <c r="A16" s="95" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="94">
+      <c r="B16" s="93">
         <v>1</v>
       </c>
-      <c r="C16" s="92">
+      <c r="C16" s="91">
         <v>1</v>
       </c>
       <c r="D16" s="12"/>
@@ -3058,7 +3058,7 @@
       <c r="F16" s="13"/>
       <c r="G16" s="13"/>
       <c r="H16" s="13"/>
-      <c r="I16" s="53"/>
+      <c r="I16" s="52"/>
       <c r="J16" s="14"/>
       <c r="K16" s="15"/>
       <c r="L16" s="12"/>
@@ -3133,7 +3133,7 @@
       <c r="CC16" s="16"/>
       <c r="CD16" s="14"/>
       <c r="CE16" s="14"/>
-      <c r="CF16" s="85" t="s">
+      <c r="CF16" s="84" t="s">
         <v>7</v>
       </c>
       <c r="CJ16" s="4"/>
@@ -3142,15 +3142,15 @@
       <c r="CN16" s="4"/>
     </row>
     <row r="17" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A17" s="97"/>
-      <c r="B17" s="95"/>
-      <c r="C17" s="93"/>
+      <c r="A17" s="96"/>
+      <c r="B17" s="94"/>
+      <c r="C17" s="92"/>
       <c r="D17" s="17"/>
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
       <c r="G17" s="18"/>
       <c r="H17" s="18"/>
-      <c r="I17" s="73"/>
+      <c r="I17" s="72"/>
       <c r="J17" s="19"/>
       <c r="K17" s="20"/>
       <c r="L17" s="17"/>
@@ -3222,23 +3222,23 @@
       <c r="BZ17" s="18"/>
       <c r="CA17" s="18"/>
       <c r="CB17" s="18"/>
-      <c r="CC17" s="26"/>
+      <c r="CC17" s="25"/>
       <c r="CD17" s="19"/>
       <c r="CE17" s="19"/>
-      <c r="CF17" s="83"/>
+      <c r="CF17" s="82"/>
       <c r="CJ17" s="4"/>
       <c r="CK17" s="4"/>
       <c r="CM17" s="4"/>
       <c r="CN17" s="4"/>
     </row>
     <row r="18" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A18" s="90" t="s">
+      <c r="A18" s="89" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="88">
+      <c r="B18" s="87">
         <v>1</v>
       </c>
-      <c r="C18" s="86">
+      <c r="C18" s="85">
         <v>1</v>
       </c>
       <c r="D18" s="17"/>
@@ -3247,7 +3247,7 @@
       <c r="G18" s="18"/>
       <c r="H18" s="18"/>
       <c r="I18" s="19"/>
-      <c r="J18" s="61"/>
+      <c r="J18" s="60"/>
       <c r="K18" s="20"/>
       <c r="L18" s="17"/>
       <c r="M18" s="18"/>
@@ -3318,10 +3318,10 @@
       <c r="BZ18" s="18"/>
       <c r="CA18" s="18"/>
       <c r="CB18" s="18"/>
-      <c r="CC18" s="26"/>
+      <c r="CC18" s="25"/>
       <c r="CD18" s="19"/>
       <c r="CE18" s="19"/>
-      <c r="CF18" s="83"/>
+      <c r="CF18" s="82"/>
       <c r="CI18" s="4"/>
       <c r="CJ18" s="4"/>
       <c r="CK18" s="4"/>
@@ -3329,16 +3329,16 @@
       <c r="CN18" s="4"/>
     </row>
     <row r="19" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A19" s="97"/>
-      <c r="B19" s="95"/>
-      <c r="C19" s="93"/>
+      <c r="A19" s="96"/>
+      <c r="B19" s="94"/>
+      <c r="C19" s="92"/>
       <c r="D19" s="17"/>
       <c r="E19" s="18"/>
       <c r="F19" s="18"/>
       <c r="G19" s="18"/>
       <c r="H19" s="18"/>
       <c r="I19" s="19"/>
-      <c r="J19" s="72"/>
+      <c r="J19" s="71"/>
       <c r="K19" s="20"/>
       <c r="L19" s="17"/>
       <c r="M19" s="18"/>
@@ -3409,19 +3409,19 @@
       <c r="BZ19" s="18"/>
       <c r="CA19" s="18"/>
       <c r="CB19" s="18"/>
-      <c r="CC19" s="26"/>
+      <c r="CC19" s="25"/>
       <c r="CD19" s="19"/>
       <c r="CE19" s="19"/>
-      <c r="CF19" s="83"/>
+      <c r="CF19" s="82"/>
     </row>
     <row r="20" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="90" t="s">
+      <c r="A20" s="89" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="88">
+      <c r="B20" s="87">
         <v>1.5</v>
       </c>
-      <c r="C20" s="86">
+      <c r="C20" s="85">
         <v>1</v>
       </c>
       <c r="D20" s="17"/>
@@ -3432,8 +3432,8 @@
       <c r="I20" s="19"/>
       <c r="J20" s="19"/>
       <c r="K20" s="20"/>
-      <c r="L20" s="58"/>
-      <c r="M20" s="57"/>
+      <c r="L20" s="57"/>
+      <c r="M20" s="56"/>
       <c r="N20" s="18"/>
       <c r="O20" s="18"/>
       <c r="P20" s="18"/>
@@ -3501,16 +3501,16 @@
       <c r="BZ20" s="18"/>
       <c r="CA20" s="18"/>
       <c r="CB20" s="18"/>
-      <c r="CC20" s="26"/>
+      <c r="CC20" s="25"/>
       <c r="CD20" s="19"/>
       <c r="CE20" s="19"/>
-      <c r="CF20" s="83"/>
+      <c r="CF20" s="82"/>
       <c r="CJ20" s="4"/>
     </row>
     <row r="21" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="97"/>
-      <c r="B21" s="95"/>
-      <c r="C21" s="93"/>
+      <c r="A21" s="96"/>
+      <c r="B21" s="94"/>
+      <c r="C21" s="92"/>
       <c r="D21" s="17"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -3519,8 +3519,8 @@
       <c r="I21" s="19"/>
       <c r="J21" s="19"/>
       <c r="K21" s="20"/>
-      <c r="L21" s="75"/>
-      <c r="M21" s="80"/>
+      <c r="L21" s="74"/>
+      <c r="M21" s="79"/>
       <c r="N21" s="18"/>
       <c r="O21" s="18"/>
       <c r="P21" s="18"/>
@@ -3588,10 +3588,10 @@
       <c r="BZ21" s="18"/>
       <c r="CA21" s="18"/>
       <c r="CB21" s="18"/>
-      <c r="CC21" s="26"/>
+      <c r="CC21" s="25"/>
       <c r="CD21" s="19"/>
       <c r="CE21" s="19"/>
-      <c r="CF21" s="83"/>
+      <c r="CF21" s="82"/>
       <c r="CI21" s="4"/>
       <c r="CJ21" s="4"/>
       <c r="CM21" s="4"/>
@@ -3599,13 +3599,13 @@
       <c r="CO21" s="4"/>
     </row>
     <row r="22" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="102" t="s">
+      <c r="A22" s="101" t="s">
         <v>32</v>
       </c>
-      <c r="B22" s="88">
+      <c r="B22" s="87">
         <v>1.5</v>
       </c>
-      <c r="C22" s="86">
+      <c r="C22" s="85">
         <v>1</v>
       </c>
       <c r="D22" s="17"/>
@@ -3619,7 +3619,7 @@
       <c r="L22" s="17"/>
       <c r="M22" s="18"/>
       <c r="N22" s="18"/>
-      <c r="O22" s="57"/>
+      <c r="O22" s="56"/>
       <c r="P22" s="18"/>
       <c r="Q22" s="19"/>
       <c r="R22" s="19"/>
@@ -3685,10 +3685,10 @@
       <c r="BZ22" s="18"/>
       <c r="CA22" s="18"/>
       <c r="CB22" s="18"/>
-      <c r="CC22" s="26"/>
+      <c r="CC22" s="25"/>
       <c r="CD22" s="19"/>
       <c r="CE22" s="19"/>
-      <c r="CF22" s="83"/>
+      <c r="CF22" s="82"/>
       <c r="CI22" s="4"/>
       <c r="CJ22" s="4"/>
       <c r="CM22" s="4"/>
@@ -3696,9 +3696,9 @@
       <c r="CO22" s="4"/>
     </row>
     <row r="23" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="103"/>
-      <c r="B23" s="95"/>
-      <c r="C23" s="93"/>
+      <c r="A23" s="102"/>
+      <c r="B23" s="94"/>
+      <c r="C23" s="92"/>
       <c r="D23" s="17"/>
       <c r="E23" s="18"/>
       <c r="F23" s="18"/>
@@ -3708,7 +3708,7 @@
       <c r="J23" s="19"/>
       <c r="K23" s="20"/>
       <c r="L23" s="17"/>
-      <c r="M23" s="71"/>
+      <c r="M23" s="70"/>
       <c r="N23" s="18"/>
       <c r="O23" s="18"/>
       <c r="P23" s="18"/>
@@ -3776,10 +3776,10 @@
       <c r="BZ23" s="18"/>
       <c r="CA23" s="18"/>
       <c r="CB23" s="18"/>
-      <c r="CC23" s="26"/>
+      <c r="CC23" s="25"/>
       <c r="CD23" s="19"/>
       <c r="CE23" s="19"/>
-      <c r="CF23" s="83"/>
+      <c r="CF23" s="82"/>
       <c r="CI23" s="4"/>
       <c r="CJ23" s="4"/>
       <c r="CM23" s="4"/>
@@ -3787,13 +3787,13 @@
       <c r="CO23" s="4"/>
     </row>
     <row r="24" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A24" s="90" t="s">
+      <c r="A24" s="89" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="88">
+      <c r="B24" s="87">
         <v>2</v>
       </c>
-      <c r="C24" s="86">
+      <c r="C24" s="85">
         <v>0</v>
       </c>
       <c r="D24" s="17"/>
@@ -3808,8 +3808,8 @@
       <c r="M24" s="18"/>
       <c r="N24" s="18"/>
       <c r="O24" s="18"/>
-      <c r="P24" s="57"/>
-      <c r="Q24" s="61"/>
+      <c r="P24" s="56"/>
+      <c r="Q24" s="60"/>
       <c r="R24" s="19"/>
       <c r="S24" s="20"/>
       <c r="T24" s="17"/>
@@ -3873,10 +3873,10 @@
       <c r="BZ24" s="18"/>
       <c r="CA24" s="18"/>
       <c r="CB24" s="18"/>
-      <c r="CC24" s="26"/>
+      <c r="CC24" s="25"/>
       <c r="CD24" s="19"/>
       <c r="CE24" s="19"/>
-      <c r="CF24" s="83"/>
+      <c r="CF24" s="82"/>
       <c r="CJ24" s="4"/>
       <c r="CK24" s="4"/>
       <c r="CM24" s="4"/>
@@ -3884,102 +3884,102 @@
       <c r="CO24" s="4"/>
     </row>
     <row r="25" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="91"/>
-      <c r="B25" s="89"/>
-      <c r="C25" s="87"/>
-      <c r="D25" s="37"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="38"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="34"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="39"/>
-      <c r="L25" s="37"/>
-      <c r="M25" s="38"/>
-      <c r="N25" s="38"/>
-      <c r="O25" s="78"/>
-      <c r="P25" s="78"/>
-      <c r="Q25" s="81"/>
-      <c r="R25" s="34"/>
-      <c r="S25" s="39"/>
-      <c r="T25" s="37"/>
-      <c r="U25" s="38"/>
-      <c r="V25" s="38"/>
-      <c r="W25" s="38"/>
-      <c r="X25" s="38"/>
-      <c r="Y25" s="34"/>
-      <c r="Z25" s="38"/>
-      <c r="AA25" s="39"/>
-      <c r="AB25" s="37"/>
-      <c r="AC25" s="38"/>
-      <c r="AD25" s="38"/>
-      <c r="AE25" s="38"/>
-      <c r="AF25" s="38"/>
-      <c r="AG25" s="34"/>
-      <c r="AH25" s="34"/>
-      <c r="AI25" s="39"/>
-      <c r="AJ25" s="37"/>
-      <c r="AK25" s="38"/>
-      <c r="AL25" s="38"/>
-      <c r="AM25" s="38"/>
-      <c r="AN25" s="38"/>
-      <c r="AO25" s="34"/>
-      <c r="AP25" s="34"/>
-      <c r="AQ25" s="39"/>
-      <c r="AR25" s="37"/>
-      <c r="AS25" s="38"/>
-      <c r="AT25" s="38"/>
-      <c r="AU25" s="38"/>
-      <c r="AV25" s="38"/>
-      <c r="AW25" s="34"/>
-      <c r="AX25" s="38"/>
-      <c r="AY25" s="39"/>
-      <c r="AZ25" s="37"/>
-      <c r="BA25" s="38"/>
-      <c r="BB25" s="38"/>
-      <c r="BC25" s="38"/>
-      <c r="BD25" s="38"/>
-      <c r="BE25" s="34"/>
-      <c r="BF25" s="34"/>
-      <c r="BG25" s="39"/>
-      <c r="BH25" s="37"/>
-      <c r="BI25" s="38"/>
-      <c r="BJ25" s="38"/>
-      <c r="BK25" s="38"/>
-      <c r="BL25" s="38"/>
-      <c r="BM25" s="34"/>
-      <c r="BN25" s="34"/>
-      <c r="BO25" s="39"/>
-      <c r="BP25" s="37"/>
-      <c r="BQ25" s="38"/>
-      <c r="BR25" s="38"/>
-      <c r="BS25" s="38"/>
-      <c r="BT25" s="38"/>
-      <c r="BU25" s="34"/>
-      <c r="BV25" s="38"/>
-      <c r="BW25" s="39"/>
-      <c r="BX25" s="37"/>
-      <c r="BY25" s="38"/>
-      <c r="BZ25" s="38"/>
-      <c r="CA25" s="38"/>
-      <c r="CB25" s="38"/>
-      <c r="CC25" s="40"/>
-      <c r="CD25" s="34"/>
-      <c r="CE25" s="34"/>
-      <c r="CF25" s="84"/>
+      <c r="A25" s="90"/>
+      <c r="B25" s="88"/>
+      <c r="C25" s="86"/>
+      <c r="D25" s="36"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="37"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="33"/>
+      <c r="J25" s="33"/>
+      <c r="K25" s="38"/>
+      <c r="L25" s="36"/>
+      <c r="M25" s="37"/>
+      <c r="N25" s="37"/>
+      <c r="O25" s="77"/>
+      <c r="P25" s="77"/>
+      <c r="Q25" s="80"/>
+      <c r="R25" s="33"/>
+      <c r="S25" s="38"/>
+      <c r="T25" s="36"/>
+      <c r="U25" s="37"/>
+      <c r="V25" s="37"/>
+      <c r="W25" s="37"/>
+      <c r="X25" s="37"/>
+      <c r="Y25" s="33"/>
+      <c r="Z25" s="37"/>
+      <c r="AA25" s="38"/>
+      <c r="AB25" s="36"/>
+      <c r="AC25" s="37"/>
+      <c r="AD25" s="37"/>
+      <c r="AE25" s="37"/>
+      <c r="AF25" s="37"/>
+      <c r="AG25" s="33"/>
+      <c r="AH25" s="33"/>
+      <c r="AI25" s="38"/>
+      <c r="AJ25" s="36"/>
+      <c r="AK25" s="37"/>
+      <c r="AL25" s="37"/>
+      <c r="AM25" s="37"/>
+      <c r="AN25" s="37"/>
+      <c r="AO25" s="33"/>
+      <c r="AP25" s="33"/>
+      <c r="AQ25" s="38"/>
+      <c r="AR25" s="36"/>
+      <c r="AS25" s="37"/>
+      <c r="AT25" s="37"/>
+      <c r="AU25" s="37"/>
+      <c r="AV25" s="37"/>
+      <c r="AW25" s="33"/>
+      <c r="AX25" s="37"/>
+      <c r="AY25" s="38"/>
+      <c r="AZ25" s="36"/>
+      <c r="BA25" s="37"/>
+      <c r="BB25" s="37"/>
+      <c r="BC25" s="37"/>
+      <c r="BD25" s="37"/>
+      <c r="BE25" s="33"/>
+      <c r="BF25" s="33"/>
+      <c r="BG25" s="38"/>
+      <c r="BH25" s="36"/>
+      <c r="BI25" s="37"/>
+      <c r="BJ25" s="37"/>
+      <c r="BK25" s="37"/>
+      <c r="BL25" s="37"/>
+      <c r="BM25" s="33"/>
+      <c r="BN25" s="33"/>
+      <c r="BO25" s="38"/>
+      <c r="BP25" s="36"/>
+      <c r="BQ25" s="37"/>
+      <c r="BR25" s="37"/>
+      <c r="BS25" s="37"/>
+      <c r="BT25" s="37"/>
+      <c r="BU25" s="33"/>
+      <c r="BV25" s="37"/>
+      <c r="BW25" s="38"/>
+      <c r="BX25" s="36"/>
+      <c r="BY25" s="37"/>
+      <c r="BZ25" s="37"/>
+      <c r="CA25" s="37"/>
+      <c r="CB25" s="37"/>
+      <c r="CC25" s="39"/>
+      <c r="CD25" s="33"/>
+      <c r="CE25" s="33"/>
+      <c r="CF25" s="83"/>
       <c r="CK25" s="4"/>
       <c r="CL25" s="4"/>
       <c r="CM25" s="4"/>
     </row>
     <row r="26" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A26" s="96" t="s">
+      <c r="A26" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="94">
+      <c r="B26" s="93">
         <v>2</v>
       </c>
-      <c r="C26" s="92">
+      <c r="C26" s="91">
         <v>0</v>
       </c>
       <c r="D26" s="12"/>
@@ -3996,8 +3996,8 @@
       <c r="O26" s="13"/>
       <c r="P26" s="13"/>
       <c r="Q26" s="14"/>
-      <c r="R26" s="53"/>
-      <c r="S26" s="52"/>
+      <c r="R26" s="52"/>
+      <c r="S26" s="51"/>
       <c r="T26" s="12"/>
       <c r="U26" s="13"/>
       <c r="V26" s="13"/>
@@ -4062,104 +4062,104 @@
       <c r="CC26" s="16"/>
       <c r="CD26" s="14"/>
       <c r="CE26" s="14"/>
-      <c r="CF26" s="85" t="s">
+      <c r="CF26" s="84" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="91"/>
-      <c r="B27" s="89"/>
-      <c r="C27" s="87"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="38"/>
-      <c r="F27" s="38"/>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
-      <c r="I27" s="34"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="39"/>
-      <c r="L27" s="37"/>
-      <c r="M27" s="38"/>
-      <c r="N27" s="38"/>
-      <c r="O27" s="38"/>
-      <c r="P27" s="38"/>
-      <c r="Q27" s="79"/>
-      <c r="R27" s="79"/>
-      <c r="S27" s="39"/>
-      <c r="T27" s="37"/>
-      <c r="U27" s="38"/>
-      <c r="V27" s="38"/>
-      <c r="W27" s="38"/>
-      <c r="X27" s="38"/>
-      <c r="Y27" s="34"/>
-      <c r="Z27" s="38"/>
-      <c r="AA27" s="39"/>
-      <c r="AB27" s="37"/>
-      <c r="AC27" s="38"/>
-      <c r="AD27" s="38"/>
-      <c r="AE27" s="38"/>
-      <c r="AF27" s="38"/>
-      <c r="AG27" s="34"/>
-      <c r="AH27" s="34"/>
-      <c r="AI27" s="39"/>
-      <c r="AJ27" s="37"/>
-      <c r="AK27" s="38"/>
-      <c r="AL27" s="38"/>
-      <c r="AM27" s="38"/>
-      <c r="AN27" s="38"/>
-      <c r="AO27" s="34"/>
-      <c r="AP27" s="34"/>
-      <c r="AQ27" s="39"/>
-      <c r="AR27" s="37"/>
-      <c r="AS27" s="38"/>
-      <c r="AT27" s="38"/>
-      <c r="AU27" s="38"/>
-      <c r="AV27" s="38"/>
-      <c r="AW27" s="34"/>
-      <c r="AX27" s="38"/>
-      <c r="AY27" s="39"/>
-      <c r="AZ27" s="37"/>
-      <c r="BA27" s="38"/>
-      <c r="BB27" s="38"/>
-      <c r="BC27" s="38"/>
-      <c r="BD27" s="38"/>
-      <c r="BE27" s="34"/>
-      <c r="BF27" s="34"/>
-      <c r="BG27" s="39"/>
-      <c r="BH27" s="37"/>
-      <c r="BI27" s="38"/>
-      <c r="BJ27" s="38"/>
-      <c r="BK27" s="38"/>
-      <c r="BL27" s="38"/>
-      <c r="BM27" s="34"/>
-      <c r="BN27" s="34"/>
-      <c r="BO27" s="39"/>
-      <c r="BP27" s="37"/>
-      <c r="BQ27" s="38"/>
-      <c r="BR27" s="38"/>
-      <c r="BS27" s="38"/>
-      <c r="BT27" s="38"/>
-      <c r="BU27" s="34"/>
-      <c r="BV27" s="38"/>
-      <c r="BW27" s="39"/>
-      <c r="BX27" s="37"/>
-      <c r="BY27" s="38"/>
-      <c r="BZ27" s="38"/>
-      <c r="CA27" s="38"/>
-      <c r="CB27" s="38"/>
-      <c r="CC27" s="40"/>
-      <c r="CD27" s="34"/>
-      <c r="CE27" s="34"/>
-      <c r="CF27" s="84"/>
+      <c r="A27" s="90"/>
+      <c r="B27" s="88"/>
+      <c r="C27" s="86"/>
+      <c r="D27" s="36"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="33"/>
+      <c r="J27" s="33"/>
+      <c r="K27" s="38"/>
+      <c r="L27" s="36"/>
+      <c r="M27" s="37"/>
+      <c r="N27" s="37"/>
+      <c r="O27" s="37"/>
+      <c r="P27" s="37"/>
+      <c r="Q27" s="78"/>
+      <c r="R27" s="78"/>
+      <c r="S27" s="38"/>
+      <c r="T27" s="36"/>
+      <c r="U27" s="37"/>
+      <c r="V27" s="37"/>
+      <c r="W27" s="37"/>
+      <c r="X27" s="37"/>
+      <c r="Y27" s="33"/>
+      <c r="Z27" s="37"/>
+      <c r="AA27" s="38"/>
+      <c r="AB27" s="36"/>
+      <c r="AC27" s="37"/>
+      <c r="AD27" s="37"/>
+      <c r="AE27" s="37"/>
+      <c r="AF27" s="37"/>
+      <c r="AG27" s="33"/>
+      <c r="AH27" s="33"/>
+      <c r="AI27" s="38"/>
+      <c r="AJ27" s="36"/>
+      <c r="AK27" s="37"/>
+      <c r="AL27" s="37"/>
+      <c r="AM27" s="37"/>
+      <c r="AN27" s="37"/>
+      <c r="AO27" s="33"/>
+      <c r="AP27" s="33"/>
+      <c r="AQ27" s="38"/>
+      <c r="AR27" s="36"/>
+      <c r="AS27" s="37"/>
+      <c r="AT27" s="37"/>
+      <c r="AU27" s="37"/>
+      <c r="AV27" s="37"/>
+      <c r="AW27" s="33"/>
+      <c r="AX27" s="37"/>
+      <c r="AY27" s="38"/>
+      <c r="AZ27" s="36"/>
+      <c r="BA27" s="37"/>
+      <c r="BB27" s="37"/>
+      <c r="BC27" s="37"/>
+      <c r="BD27" s="37"/>
+      <c r="BE27" s="33"/>
+      <c r="BF27" s="33"/>
+      <c r="BG27" s="38"/>
+      <c r="BH27" s="36"/>
+      <c r="BI27" s="37"/>
+      <c r="BJ27" s="37"/>
+      <c r="BK27" s="37"/>
+      <c r="BL27" s="37"/>
+      <c r="BM27" s="33"/>
+      <c r="BN27" s="33"/>
+      <c r="BO27" s="38"/>
+      <c r="BP27" s="36"/>
+      <c r="BQ27" s="37"/>
+      <c r="BR27" s="37"/>
+      <c r="BS27" s="37"/>
+      <c r="BT27" s="37"/>
+      <c r="BU27" s="33"/>
+      <c r="BV27" s="37"/>
+      <c r="BW27" s="38"/>
+      <c r="BX27" s="36"/>
+      <c r="BY27" s="37"/>
+      <c r="BZ27" s="37"/>
+      <c r="CA27" s="37"/>
+      <c r="CB27" s="37"/>
+      <c r="CC27" s="39"/>
+      <c r="CD27" s="33"/>
+      <c r="CE27" s="33"/>
+      <c r="CF27" s="83"/>
     </row>
     <row r="28" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A28" s="96" t="s">
+      <c r="A28" s="95" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="94">
+      <c r="B28" s="93">
         <v>1</v>
       </c>
-      <c r="C28" s="92">
+      <c r="C28" s="91">
         <v>0</v>
       </c>
       <c r="D28" s="12"/>
@@ -4178,7 +4178,7 @@
       <c r="Q28" s="14"/>
       <c r="R28" s="14"/>
       <c r="S28" s="15"/>
-      <c r="T28" s="62"/>
+      <c r="T28" s="61"/>
       <c r="U28" s="13"/>
       <c r="V28" s="13"/>
       <c r="W28" s="13"/>
@@ -4242,14 +4242,14 @@
       <c r="CC28" s="16"/>
       <c r="CD28" s="14"/>
       <c r="CE28" s="14"/>
-      <c r="CF28" s="85" t="s">
+      <c r="CF28" s="84" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A29" s="97"/>
-      <c r="B29" s="95"/>
-      <c r="C29" s="93"/>
+      <c r="A29" s="96"/>
+      <c r="B29" s="94"/>
+      <c r="C29" s="92"/>
       <c r="D29" s="17"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
@@ -4265,8 +4265,8 @@
       <c r="P29" s="18"/>
       <c r="Q29" s="19"/>
       <c r="R29" s="19"/>
-      <c r="S29" s="74"/>
-      <c r="T29" s="80"/>
+      <c r="S29" s="73"/>
+      <c r="T29" s="79"/>
       <c r="U29" s="18"/>
       <c r="V29" s="18"/>
       <c r="W29" s="18"/>
@@ -4327,19 +4327,19 @@
       <c r="BZ29" s="18"/>
       <c r="CA29" s="18"/>
       <c r="CB29" s="18"/>
-      <c r="CC29" s="26"/>
+      <c r="CC29" s="25"/>
       <c r="CD29" s="19"/>
       <c r="CE29" s="19"/>
-      <c r="CF29" s="83"/>
+      <c r="CF29" s="82"/>
     </row>
     <row r="30" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="90" t="s">
+      <c r="A30" s="89" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="88">
+      <c r="B30" s="87">
         <v>2</v>
       </c>
-      <c r="C30" s="86">
+      <c r="C30" s="85">
         <v>0</v>
       </c>
       <c r="D30" s="17"/>
@@ -4359,8 +4359,8 @@
       <c r="R30" s="19"/>
       <c r="S30" s="20"/>
       <c r="T30" s="17"/>
-      <c r="U30" s="57"/>
-      <c r="V30" s="57"/>
+      <c r="U30" s="56"/>
+      <c r="V30" s="56"/>
       <c r="W30" s="18"/>
       <c r="X30" s="18"/>
       <c r="Y30" s="19"/>
@@ -4419,15 +4419,15 @@
       <c r="BZ30" s="18"/>
       <c r="CA30" s="18"/>
       <c r="CB30" s="18"/>
-      <c r="CC30" s="26"/>
+      <c r="CC30" s="25"/>
       <c r="CD30" s="19"/>
       <c r="CE30" s="19"/>
-      <c r="CF30" s="83"/>
+      <c r="CF30" s="82"/>
     </row>
     <row r="31" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="97"/>
-      <c r="B31" s="95"/>
-      <c r="C31" s="93"/>
+      <c r="A31" s="96"/>
+      <c r="B31" s="94"/>
+      <c r="C31" s="92"/>
       <c r="D31" s="17"/>
       <c r="E31" s="18"/>
       <c r="F31" s="18"/>
@@ -4444,8 +4444,8 @@
       <c r="Q31" s="19"/>
       <c r="R31" s="19"/>
       <c r="S31" s="20"/>
-      <c r="T31" s="76"/>
-      <c r="U31" s="71"/>
+      <c r="T31" s="75"/>
+      <c r="U31" s="70"/>
       <c r="V31" s="18"/>
       <c r="W31" s="18"/>
       <c r="X31" s="18"/>
@@ -4505,19 +4505,19 @@
       <c r="BZ31" s="18"/>
       <c r="CA31" s="18"/>
       <c r="CB31" s="18"/>
-      <c r="CC31" s="26"/>
+      <c r="CC31" s="25"/>
       <c r="CD31" s="19"/>
       <c r="CE31" s="19"/>
-      <c r="CF31" s="83"/>
+      <c r="CF31" s="82"/>
     </row>
     <row r="32" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A32" s="90" t="s">
+      <c r="A32" s="89" t="s">
         <v>34</v>
       </c>
-      <c r="B32" s="88">
+      <c r="B32" s="87">
         <v>4</v>
       </c>
-      <c r="C32" s="86">
+      <c r="C32" s="85">
         <v>0</v>
       </c>
       <c r="D32" s="17"/>
@@ -4539,11 +4539,11 @@
       <c r="T32" s="17"/>
       <c r="U32" s="18"/>
       <c r="V32" s="18"/>
-      <c r="W32" s="57"/>
-      <c r="X32" s="57"/>
-      <c r="Y32" s="61"/>
-      <c r="Z32" s="57"/>
-      <c r="AA32" s="41"/>
+      <c r="W32" s="56"/>
+      <c r="X32" s="56"/>
+      <c r="Y32" s="60"/>
+      <c r="Z32" s="56"/>
+      <c r="AA32" s="40"/>
       <c r="AB32" s="17"/>
       <c r="AC32" s="18"/>
       <c r="AD32" s="18"/>
@@ -4597,15 +4597,15 @@
       <c r="BZ32" s="18"/>
       <c r="CA32" s="18"/>
       <c r="CB32" s="18"/>
-      <c r="CC32" s="26"/>
+      <c r="CC32" s="25"/>
       <c r="CD32" s="19"/>
       <c r="CE32" s="19"/>
-      <c r="CF32" s="83"/>
+      <c r="CF32" s="82"/>
     </row>
     <row r="33" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A33" s="97"/>
-      <c r="B33" s="95"/>
-      <c r="C33" s="93"/>
+      <c r="A33" s="96"/>
+      <c r="B33" s="94"/>
+      <c r="C33" s="92"/>
       <c r="D33" s="17"/>
       <c r="E33" s="18"/>
       <c r="F33" s="18"/>
@@ -4624,10 +4624,10 @@
       <c r="S33" s="20"/>
       <c r="T33" s="17"/>
       <c r="U33" s="18"/>
-      <c r="V33" s="71"/>
-      <c r="W33" s="71"/>
-      <c r="X33" s="71"/>
-      <c r="Y33" s="72"/>
+      <c r="V33" s="70"/>
+      <c r="W33" s="70"/>
+      <c r="X33" s="70"/>
+      <c r="Y33" s="71"/>
       <c r="Z33" s="18"/>
       <c r="AA33" s="20"/>
       <c r="AB33" s="17"/>
@@ -4683,19 +4683,19 @@
       <c r="BZ33" s="18"/>
       <c r="CA33" s="18"/>
       <c r="CB33" s="18"/>
-      <c r="CC33" s="26"/>
+      <c r="CC33" s="25"/>
       <c r="CD33" s="19"/>
       <c r="CE33" s="19"/>
-      <c r="CF33" s="83"/>
+      <c r="CF33" s="82"/>
     </row>
     <row r="34" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A34" s="90" t="s">
+      <c r="A34" s="89" t="s">
         <v>35</v>
       </c>
-      <c r="B34" s="88">
+      <c r="B34" s="87">
         <v>4</v>
       </c>
-      <c r="C34" s="86">
+      <c r="C34" s="85">
         <v>0</v>
       </c>
       <c r="D34" s="17"/>
@@ -4722,10 +4722,10 @@
       <c r="Y34" s="19"/>
       <c r="Z34" s="18"/>
       <c r="AA34" s="20"/>
-      <c r="AB34" s="58"/>
-      <c r="AC34" s="57"/>
-      <c r="AD34" s="57"/>
-      <c r="AE34" s="57"/>
+      <c r="AB34" s="57"/>
+      <c r="AC34" s="56"/>
+      <c r="AD34" s="56"/>
+      <c r="AE34" s="56"/>
       <c r="AF34" s="18"/>
       <c r="AG34" s="19"/>
       <c r="AH34" s="19"/>
@@ -4775,15 +4775,15 @@
       <c r="BZ34" s="18"/>
       <c r="CA34" s="18"/>
       <c r="CB34" s="18"/>
-      <c r="CC34" s="26"/>
+      <c r="CC34" s="25"/>
       <c r="CD34" s="19"/>
       <c r="CE34" s="19"/>
-      <c r="CF34" s="83"/>
+      <c r="CF34" s="82"/>
     </row>
     <row r="35" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A35" s="97"/>
-      <c r="B35" s="95"/>
-      <c r="C35" s="93"/>
+      <c r="A35" s="96"/>
+      <c r="B35" s="94"/>
+      <c r="C35" s="92"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
       <c r="F35" s="18"/>
@@ -4807,10 +4807,10 @@
       <c r="X35" s="18"/>
       <c r="Y35" s="19"/>
       <c r="Z35" s="18"/>
-      <c r="AA35" s="74"/>
-      <c r="AB35" s="76"/>
-      <c r="AC35" s="71"/>
-      <c r="AD35" s="71"/>
+      <c r="AA35" s="73"/>
+      <c r="AB35" s="75"/>
+      <c r="AC35" s="70"/>
+      <c r="AD35" s="70"/>
       <c r="AE35" s="18"/>
       <c r="AF35" s="18"/>
       <c r="AG35" s="19"/>
@@ -4861,19 +4861,19 @@
       <c r="BZ35" s="18"/>
       <c r="CA35" s="18"/>
       <c r="CB35" s="18"/>
-      <c r="CC35" s="26"/>
+      <c r="CC35" s="25"/>
       <c r="CD35" s="19"/>
       <c r="CE35" s="19"/>
-      <c r="CF35" s="83"/>
+      <c r="CF35" s="82"/>
     </row>
     <row r="36" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A36" s="90" t="s">
+      <c r="A36" s="89" t="s">
         <v>38</v>
       </c>
-      <c r="B36" s="88">
+      <c r="B36" s="87">
         <v>9</v>
       </c>
-      <c r="C36" s="86">
+      <c r="C36" s="85">
         <v>0</v>
       </c>
       <c r="D36" s="17"/>
@@ -4906,15 +4906,15 @@
       <c r="AE36" s="18"/>
       <c r="AF36" s="18"/>
       <c r="AG36" s="19"/>
-      <c r="AH36" s="61"/>
-      <c r="AI36" s="63"/>
-      <c r="AJ36" s="58"/>
-      <c r="AK36" s="57"/>
-      <c r="AL36" s="57"/>
-      <c r="AM36" s="57"/>
-      <c r="AN36" s="57"/>
-      <c r="AO36" s="61"/>
-      <c r="AP36" s="61"/>
+      <c r="AH36" s="60"/>
+      <c r="AI36" s="62"/>
+      <c r="AJ36" s="57"/>
+      <c r="AK36" s="56"/>
+      <c r="AL36" s="56"/>
+      <c r="AM36" s="56"/>
+      <c r="AN36" s="56"/>
+      <c r="AO36" s="60"/>
+      <c r="AP36" s="60"/>
       <c r="AQ36" s="20"/>
       <c r="AR36" s="17"/>
       <c r="AS36" s="18"/>
@@ -4953,15 +4953,15 @@
       <c r="BZ36" s="18"/>
       <c r="CA36" s="18"/>
       <c r="CB36" s="18"/>
-      <c r="CC36" s="26"/>
+      <c r="CC36" s="25"/>
       <c r="CD36" s="19"/>
       <c r="CE36" s="19"/>
-      <c r="CF36" s="83"/>
+      <c r="CF36" s="82"/>
     </row>
     <row r="37" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A37" s="97"/>
-      <c r="B37" s="95"/>
-      <c r="C37" s="93"/>
+      <c r="A37" s="96"/>
+      <c r="B37" s="94"/>
+      <c r="C37" s="92"/>
       <c r="D37" s="17"/>
       <c r="E37" s="18"/>
       <c r="F37" s="18"/>
@@ -4991,9 +4991,9 @@
       <c r="AD37" s="18"/>
       <c r="AE37" s="18"/>
       <c r="AF37" s="18"/>
-      <c r="AG37" s="19"/>
-      <c r="AH37" s="19"/>
-      <c r="AI37" s="20"/>
+      <c r="AG37" s="71"/>
+      <c r="AH37" s="71"/>
+      <c r="AI37" s="73"/>
       <c r="AJ37" s="17"/>
       <c r="AK37" s="18"/>
       <c r="AL37" s="18"/>
@@ -5039,19 +5039,19 @@
       <c r="BZ37" s="18"/>
       <c r="CA37" s="18"/>
       <c r="CB37" s="18"/>
-      <c r="CC37" s="26"/>
+      <c r="CC37" s="25"/>
       <c r="CD37" s="19"/>
       <c r="CE37" s="19"/>
-      <c r="CF37" s="83"/>
+      <c r="CF37" s="82"/>
     </row>
     <row r="38" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A38" s="100" t="s">
+      <c r="A38" s="99" t="s">
         <v>39</v>
       </c>
-      <c r="B38" s="88">
+      <c r="B38" s="87">
         <v>5</v>
       </c>
-      <c r="C38" s="86">
+      <c r="C38" s="85">
         <v>0</v>
       </c>
       <c r="D38" s="17"/>
@@ -5076,7 +5076,7 @@
       <c r="W38" s="18"/>
       <c r="X38" s="18"/>
       <c r="Y38" s="19"/>
-      <c r="Z38" s="26"/>
+      <c r="Z38" s="25"/>
       <c r="AA38" s="20"/>
       <c r="AB38" s="17"/>
       <c r="AC38" s="18"/>
@@ -5096,11 +5096,11 @@
       <c r="AQ38" s="20"/>
       <c r="AR38" s="17"/>
       <c r="AS38" s="18"/>
-      <c r="AT38" s="57"/>
-      <c r="AU38" s="57"/>
-      <c r="AV38" s="57"/>
-      <c r="AW38" s="61"/>
-      <c r="AX38" s="57"/>
+      <c r="AT38" s="56"/>
+      <c r="AU38" s="56"/>
+      <c r="AV38" s="56"/>
+      <c r="AW38" s="60"/>
+      <c r="AX38" s="56"/>
       <c r="AY38" s="20"/>
       <c r="AZ38" s="17"/>
       <c r="BA38" s="18"/>
@@ -5131,15 +5131,15 @@
       <c r="BZ38" s="18"/>
       <c r="CA38" s="18"/>
       <c r="CB38" s="18"/>
-      <c r="CC38" s="26"/>
+      <c r="CC38" s="25"/>
       <c r="CD38" s="19"/>
       <c r="CE38" s="19"/>
-      <c r="CF38" s="83"/>
+      <c r="CF38" s="82"/>
     </row>
     <row r="39" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A39" s="101"/>
-      <c r="B39" s="95"/>
-      <c r="C39" s="93"/>
+      <c r="A39" s="100"/>
+      <c r="B39" s="94"/>
+      <c r="C39" s="92"/>
       <c r="D39" s="17"/>
       <c r="E39" s="18"/>
       <c r="F39" s="18"/>
@@ -5163,7 +5163,7 @@
       <c r="X39" s="18"/>
       <c r="Y39" s="19"/>
       <c r="Z39" s="18"/>
-      <c r="AA39" s="42"/>
+      <c r="AA39" s="41"/>
       <c r="AB39" s="17"/>
       <c r="AC39" s="18"/>
       <c r="AD39" s="18"/>
@@ -5217,19 +5217,19 @@
       <c r="BZ39" s="18"/>
       <c r="CA39" s="18"/>
       <c r="CB39" s="18"/>
-      <c r="CC39" s="26"/>
+      <c r="CC39" s="25"/>
       <c r="CD39" s="19"/>
       <c r="CE39" s="19"/>
-      <c r="CF39" s="83"/>
+      <c r="CF39" s="82"/>
     </row>
     <row r="40" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A40" s="100" t="s">
+      <c r="A40" s="99" t="s">
         <v>40</v>
       </c>
-      <c r="B40" s="88">
+      <c r="B40" s="87">
         <v>4</v>
       </c>
-      <c r="C40" s="86">
+      <c r="C40" s="85">
         <v>0</v>
       </c>
       <c r="D40" s="17"/>
@@ -5282,10 +5282,10 @@
       <c r="AY40" s="20"/>
       <c r="AZ40" s="17"/>
       <c r="BA40" s="18"/>
-      <c r="BB40" s="57"/>
-      <c r="BC40" s="57"/>
-      <c r="BD40" s="57"/>
-      <c r="BE40" s="61"/>
+      <c r="BB40" s="56"/>
+      <c r="BC40" s="56"/>
+      <c r="BD40" s="56"/>
+      <c r="BE40" s="60"/>
       <c r="BF40" s="19"/>
       <c r="BG40" s="20"/>
       <c r="BH40" s="17"/>
@@ -5309,15 +5309,15 @@
       <c r="BZ40" s="18"/>
       <c r="CA40" s="18"/>
       <c r="CB40" s="18"/>
-      <c r="CC40" s="26"/>
+      <c r="CC40" s="25"/>
       <c r="CD40" s="19"/>
       <c r="CE40" s="19"/>
-      <c r="CF40" s="83"/>
+      <c r="CF40" s="82"/>
     </row>
     <row r="41" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A41" s="101"/>
-      <c r="B41" s="95"/>
-      <c r="C41" s="93"/>
+      <c r="A41" s="100"/>
+      <c r="B41" s="94"/>
+      <c r="C41" s="92"/>
       <c r="D41" s="17"/>
       <c r="E41" s="18"/>
       <c r="F41" s="18"/>
@@ -5395,19 +5395,19 @@
       <c r="BZ41" s="18"/>
       <c r="CA41" s="18"/>
       <c r="CB41" s="18"/>
-      <c r="CC41" s="26"/>
+      <c r="CC41" s="25"/>
       <c r="CD41" s="19"/>
       <c r="CE41" s="19"/>
-      <c r="CF41" s="83"/>
+      <c r="CF41" s="82"/>
     </row>
     <row r="42" spans="1:84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="90" t="s">
+      <c r="A42" s="89" t="s">
         <v>41</v>
       </c>
-      <c r="B42" s="88">
+      <c r="B42" s="87">
         <v>2</v>
       </c>
-      <c r="C42" s="86">
+      <c r="C42" s="85">
         <v>0</v>
       </c>
       <c r="D42" s="17"/>
@@ -5466,8 +5466,8 @@
       <c r="BE42" s="19"/>
       <c r="BF42" s="19"/>
       <c r="BG42" s="20"/>
-      <c r="BH42" s="58"/>
-      <c r="BI42" s="57"/>
+      <c r="BH42" s="57"/>
+      <c r="BI42" s="56"/>
       <c r="BJ42" s="18"/>
       <c r="BK42" s="18"/>
       <c r="BL42" s="18"/>
@@ -5487,15 +5487,15 @@
       <c r="BZ42" s="18"/>
       <c r="CA42" s="18"/>
       <c r="CB42" s="18"/>
-      <c r="CC42" s="26"/>
+      <c r="CC42" s="25"/>
       <c r="CD42" s="19"/>
       <c r="CE42" s="19"/>
-      <c r="CF42" s="83"/>
+      <c r="CF42" s="82"/>
     </row>
     <row r="43" spans="1:84" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="97"/>
-      <c r="B43" s="95"/>
-      <c r="C43" s="93"/>
+      <c r="A43" s="96"/>
+      <c r="B43" s="94"/>
+      <c r="C43" s="92"/>
       <c r="D43" s="17"/>
       <c r="E43" s="18"/>
       <c r="F43" s="18"/>
@@ -5573,19 +5573,19 @@
       <c r="BZ43" s="18"/>
       <c r="CA43" s="18"/>
       <c r="CB43" s="18"/>
-      <c r="CC43" s="26"/>
+      <c r="CC43" s="25"/>
       <c r="CD43" s="19"/>
       <c r="CE43" s="19"/>
-      <c r="CF43" s="83"/>
+      <c r="CF43" s="82"/>
     </row>
     <row r="44" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A44" s="96" t="s">
+      <c r="A44" s="95" t="s">
         <v>22</v>
       </c>
-      <c r="B44" s="94">
+      <c r="B44" s="93">
         <v>5</v>
       </c>
-      <c r="C44" s="92">
+      <c r="C44" s="91">
         <v>0</v>
       </c>
       <c r="D44" s="12"/>
@@ -5652,11 +5652,11 @@
       <c r="BM44" s="14"/>
       <c r="BN44" s="14"/>
       <c r="BO44" s="15"/>
-      <c r="BP44" s="62"/>
-      <c r="BQ44" s="68"/>
-      <c r="BR44" s="68"/>
-      <c r="BS44" s="68"/>
-      <c r="BT44" s="68"/>
+      <c r="BP44" s="61"/>
+      <c r="BQ44" s="67"/>
+      <c r="BR44" s="67"/>
+      <c r="BS44" s="67"/>
+      <c r="BT44" s="67"/>
       <c r="BU44" s="14"/>
       <c r="BV44" s="13"/>
       <c r="BW44" s="15"/>
@@ -5668,14 +5668,14 @@
       <c r="CC44" s="16"/>
       <c r="CD44" s="14"/>
       <c r="CE44" s="14"/>
-      <c r="CF44" s="85" t="s">
+      <c r="CF44" s="84" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:84" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="97"/>
-      <c r="B45" s="95"/>
-      <c r="C45" s="93"/>
+      <c r="A45" s="96"/>
+      <c r="B45" s="94"/>
+      <c r="C45" s="92"/>
       <c r="D45" s="17"/>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -5753,19 +5753,19 @@
       <c r="BZ45" s="18"/>
       <c r="CA45" s="18"/>
       <c r="CB45" s="18"/>
-      <c r="CC45" s="26"/>
+      <c r="CC45" s="25"/>
       <c r="CD45" s="19"/>
       <c r="CE45" s="19"/>
-      <c r="CF45" s="83"/>
+      <c r="CF45" s="82"/>
     </row>
     <row r="46" spans="1:84" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="90" t="s">
+      <c r="A46" s="89" t="s">
         <v>37</v>
       </c>
-      <c r="B46" s="88">
+      <c r="B46" s="87">
         <v>3</v>
       </c>
-      <c r="C46" s="86">
+      <c r="C46" s="85">
         <v>0</v>
       </c>
       <c r="D46" s="17"/>
@@ -5807,7 +5807,7 @@
       <c r="AN46" s="18"/>
       <c r="AO46" s="19"/>
       <c r="AP46" s="19"/>
-      <c r="AQ46" s="42"/>
+      <c r="AQ46" s="41"/>
       <c r="AR46" s="17"/>
       <c r="AS46" s="18"/>
       <c r="AT46" s="18"/>
@@ -5837,381 +5837,381 @@
       <c r="BR46" s="18"/>
       <c r="BS46" s="18"/>
       <c r="BT46" s="18"/>
-      <c r="BU46" s="61"/>
-      <c r="BV46" s="57"/>
-      <c r="BW46" s="63"/>
+      <c r="BU46" s="60"/>
+      <c r="BV46" s="56"/>
+      <c r="BW46" s="62"/>
       <c r="BX46" s="17"/>
       <c r="BY46" s="18"/>
       <c r="BZ46" s="18"/>
       <c r="CA46" s="18"/>
       <c r="CB46" s="18"/>
-      <c r="CC46" s="26"/>
+      <c r="CC46" s="25"/>
       <c r="CD46" s="19"/>
       <c r="CE46" s="19"/>
-      <c r="CF46" s="83"/>
+      <c r="CF46" s="82"/>
     </row>
     <row r="47" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="91"/>
-      <c r="B47" s="89"/>
-      <c r="C47" s="87"/>
-      <c r="D47" s="37"/>
-      <c r="E47" s="38"/>
-      <c r="F47" s="38"/>
-      <c r="G47" s="38"/>
-      <c r="H47" s="38"/>
-      <c r="I47" s="34"/>
-      <c r="J47" s="34"/>
-      <c r="K47" s="39"/>
-      <c r="L47" s="37"/>
-      <c r="M47" s="38"/>
-      <c r="N47" s="38"/>
-      <c r="O47" s="38"/>
-      <c r="P47" s="38"/>
-      <c r="Q47" s="34"/>
-      <c r="R47" s="34"/>
-      <c r="S47" s="39"/>
-      <c r="T47" s="37"/>
-      <c r="U47" s="38"/>
-      <c r="V47" s="38"/>
-      <c r="W47" s="38"/>
-      <c r="X47" s="38"/>
-      <c r="Y47" s="34"/>
-      <c r="Z47" s="38"/>
-      <c r="AA47" s="39"/>
-      <c r="AB47" s="37"/>
-      <c r="AC47" s="38"/>
-      <c r="AD47" s="38"/>
-      <c r="AE47" s="38"/>
-      <c r="AF47" s="38"/>
-      <c r="AG47" s="34"/>
-      <c r="AH47" s="34"/>
-      <c r="AI47" s="39"/>
-      <c r="AJ47" s="37"/>
-      <c r="AK47" s="38"/>
-      <c r="AL47" s="34"/>
-      <c r="AM47" s="38"/>
-      <c r="AN47" s="38"/>
-      <c r="AO47" s="34"/>
-      <c r="AP47" s="34"/>
-      <c r="AQ47" s="39"/>
-      <c r="AR47" s="37"/>
-      <c r="AS47" s="38"/>
-      <c r="AT47" s="38"/>
-      <c r="AU47" s="38"/>
-      <c r="AV47" s="38"/>
-      <c r="AW47" s="34"/>
-      <c r="AX47" s="38"/>
-      <c r="AY47" s="39"/>
-      <c r="AZ47" s="37"/>
-      <c r="BA47" s="38"/>
-      <c r="BB47" s="38"/>
-      <c r="BC47" s="38"/>
-      <c r="BD47" s="38"/>
-      <c r="BE47" s="34"/>
-      <c r="BF47" s="34"/>
-      <c r="BG47" s="39"/>
-      <c r="BH47" s="37"/>
-      <c r="BI47" s="38"/>
-      <c r="BJ47" s="38"/>
-      <c r="BK47" s="38"/>
-      <c r="BL47" s="38"/>
-      <c r="BM47" s="34"/>
-      <c r="BN47" s="34"/>
-      <c r="BO47" s="39"/>
-      <c r="BP47" s="37"/>
-      <c r="BQ47" s="38"/>
-      <c r="BR47" s="38"/>
-      <c r="BS47" s="38"/>
-      <c r="BT47" s="38"/>
-      <c r="BU47" s="34"/>
-      <c r="BV47" s="38"/>
-      <c r="BW47" s="39"/>
-      <c r="BX47" s="37"/>
-      <c r="BY47" s="38"/>
-      <c r="BZ47" s="38"/>
-      <c r="CA47" s="38"/>
-      <c r="CB47" s="38"/>
-      <c r="CC47" s="40"/>
-      <c r="CD47" s="34"/>
-      <c r="CE47" s="34"/>
-      <c r="CF47" s="84"/>
+      <c r="A47" s="90"/>
+      <c r="B47" s="88"/>
+      <c r="C47" s="86"/>
+      <c r="D47" s="36"/>
+      <c r="E47" s="37"/>
+      <c r="F47" s="37"/>
+      <c r="G47" s="37"/>
+      <c r="H47" s="37"/>
+      <c r="I47" s="33"/>
+      <c r="J47" s="33"/>
+      <c r="K47" s="38"/>
+      <c r="L47" s="36"/>
+      <c r="M47" s="37"/>
+      <c r="N47" s="37"/>
+      <c r="O47" s="37"/>
+      <c r="P47" s="37"/>
+      <c r="Q47" s="33"/>
+      <c r="R47" s="33"/>
+      <c r="S47" s="38"/>
+      <c r="T47" s="36"/>
+      <c r="U47" s="37"/>
+      <c r="V47" s="37"/>
+      <c r="W47" s="37"/>
+      <c r="X47" s="37"/>
+      <c r="Y47" s="33"/>
+      <c r="Z47" s="37"/>
+      <c r="AA47" s="38"/>
+      <c r="AB47" s="36"/>
+      <c r="AC47" s="37"/>
+      <c r="AD47" s="37"/>
+      <c r="AE47" s="37"/>
+      <c r="AF47" s="37"/>
+      <c r="AG47" s="33"/>
+      <c r="AH47" s="33"/>
+      <c r="AI47" s="38"/>
+      <c r="AJ47" s="36"/>
+      <c r="AK47" s="37"/>
+      <c r="AL47" s="33"/>
+      <c r="AM47" s="37"/>
+      <c r="AN47" s="37"/>
+      <c r="AO47" s="33"/>
+      <c r="AP47" s="33"/>
+      <c r="AQ47" s="38"/>
+      <c r="AR47" s="36"/>
+      <c r="AS47" s="37"/>
+      <c r="AT47" s="37"/>
+      <c r="AU47" s="37"/>
+      <c r="AV47" s="37"/>
+      <c r="AW47" s="33"/>
+      <c r="AX47" s="37"/>
+      <c r="AY47" s="38"/>
+      <c r="AZ47" s="36"/>
+      <c r="BA47" s="37"/>
+      <c r="BB47" s="37"/>
+      <c r="BC47" s="37"/>
+      <c r="BD47" s="37"/>
+      <c r="BE47" s="33"/>
+      <c r="BF47" s="33"/>
+      <c r="BG47" s="38"/>
+      <c r="BH47" s="36"/>
+      <c r="BI47" s="37"/>
+      <c r="BJ47" s="37"/>
+      <c r="BK47" s="37"/>
+      <c r="BL47" s="37"/>
+      <c r="BM47" s="33"/>
+      <c r="BN47" s="33"/>
+      <c r="BO47" s="38"/>
+      <c r="BP47" s="36"/>
+      <c r="BQ47" s="37"/>
+      <c r="BR47" s="37"/>
+      <c r="BS47" s="37"/>
+      <c r="BT47" s="37"/>
+      <c r="BU47" s="33"/>
+      <c r="BV47" s="37"/>
+      <c r="BW47" s="38"/>
+      <c r="BX47" s="36"/>
+      <c r="BY47" s="37"/>
+      <c r="BZ47" s="37"/>
+      <c r="CA47" s="37"/>
+      <c r="CB47" s="37"/>
+      <c r="CC47" s="39"/>
+      <c r="CD47" s="33"/>
+      <c r="CE47" s="33"/>
+      <c r="CF47" s="83"/>
     </row>
     <row r="48" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="96" t="s">
+      <c r="A48" s="95" t="s">
         <v>23</v>
       </c>
-      <c r="B48" s="94">
+      <c r="B48" s="93">
         <v>3</v>
       </c>
-      <c r="C48" s="98">
+      <c r="C48" s="97">
         <v>0</v>
       </c>
-      <c r="D48" s="43"/>
-      <c r="E48" s="44"/>
-      <c r="F48" s="44"/>
-      <c r="G48" s="44"/>
-      <c r="H48" s="44"/>
-      <c r="I48" s="45"/>
-      <c r="J48" s="45"/>
-      <c r="K48" s="46"/>
-      <c r="L48" s="43"/>
-      <c r="M48" s="44"/>
-      <c r="N48" s="44"/>
-      <c r="O48" s="44"/>
-      <c r="P48" s="44"/>
-      <c r="Q48" s="45"/>
-      <c r="R48" s="45"/>
-      <c r="S48" s="46"/>
-      <c r="T48" s="43"/>
-      <c r="U48" s="44"/>
-      <c r="V48" s="44"/>
-      <c r="W48" s="44"/>
-      <c r="X48" s="44"/>
-      <c r="Y48" s="45"/>
-      <c r="Z48" s="44"/>
-      <c r="AA48" s="46"/>
-      <c r="AB48" s="43"/>
-      <c r="AC48" s="44"/>
-      <c r="AD48" s="44"/>
-      <c r="AE48" s="44"/>
-      <c r="AF48" s="44"/>
-      <c r="AG48" s="45"/>
-      <c r="AH48" s="45"/>
-      <c r="AI48" s="46"/>
-      <c r="AJ48" s="43"/>
-      <c r="AK48" s="44"/>
-      <c r="AL48" s="45"/>
-      <c r="AM48" s="44"/>
-      <c r="AN48" s="44"/>
-      <c r="AO48" s="45"/>
-      <c r="AP48" s="45"/>
-      <c r="AQ48" s="46"/>
-      <c r="AR48" s="43"/>
-      <c r="AS48" s="44"/>
-      <c r="AT48" s="44"/>
-      <c r="AU48" s="44"/>
-      <c r="AV48" s="44"/>
-      <c r="AW48" s="45"/>
-      <c r="AX48" s="44"/>
-      <c r="AY48" s="46"/>
-      <c r="AZ48" s="43"/>
-      <c r="BA48" s="44"/>
-      <c r="BB48" s="44"/>
-      <c r="BC48" s="44"/>
-      <c r="BD48" s="44"/>
-      <c r="BE48" s="45"/>
-      <c r="BF48" s="45"/>
-      <c r="BG48" s="47"/>
-      <c r="BH48" s="44"/>
-      <c r="BI48" s="44"/>
-      <c r="BJ48" s="44"/>
-      <c r="BK48" s="44"/>
-      <c r="BL48" s="44"/>
-      <c r="BM48" s="45"/>
-      <c r="BN48" s="45"/>
-      <c r="BO48" s="47"/>
-      <c r="BP48" s="44"/>
-      <c r="BQ48" s="44"/>
-      <c r="BR48" s="44"/>
-      <c r="BS48" s="44"/>
-      <c r="BT48" s="44"/>
-      <c r="BU48" s="45"/>
-      <c r="BV48" s="44"/>
-      <c r="BW48" s="47"/>
-      <c r="BX48" s="67"/>
-      <c r="BY48" s="67"/>
-      <c r="BZ48" s="67"/>
-      <c r="CA48" s="44"/>
-      <c r="CB48" s="44"/>
-      <c r="CC48" s="48"/>
-      <c r="CD48" s="45"/>
-      <c r="CE48" s="48"/>
-      <c r="CF48" s="85" t="s">
+      <c r="D48" s="42"/>
+      <c r="E48" s="43"/>
+      <c r="F48" s="43"/>
+      <c r="G48" s="43"/>
+      <c r="H48" s="43"/>
+      <c r="I48" s="44"/>
+      <c r="J48" s="44"/>
+      <c r="K48" s="45"/>
+      <c r="L48" s="42"/>
+      <c r="M48" s="43"/>
+      <c r="N48" s="43"/>
+      <c r="O48" s="43"/>
+      <c r="P48" s="43"/>
+      <c r="Q48" s="44"/>
+      <c r="R48" s="44"/>
+      <c r="S48" s="45"/>
+      <c r="T48" s="42"/>
+      <c r="U48" s="43"/>
+      <c r="V48" s="43"/>
+      <c r="W48" s="43"/>
+      <c r="X48" s="43"/>
+      <c r="Y48" s="44"/>
+      <c r="Z48" s="43"/>
+      <c r="AA48" s="45"/>
+      <c r="AB48" s="42"/>
+      <c r="AC48" s="43"/>
+      <c r="AD48" s="43"/>
+      <c r="AE48" s="43"/>
+      <c r="AF48" s="43"/>
+      <c r="AG48" s="44"/>
+      <c r="AH48" s="44"/>
+      <c r="AI48" s="45"/>
+      <c r="AJ48" s="42"/>
+      <c r="AK48" s="43"/>
+      <c r="AL48" s="44"/>
+      <c r="AM48" s="43"/>
+      <c r="AN48" s="43"/>
+      <c r="AO48" s="44"/>
+      <c r="AP48" s="44"/>
+      <c r="AQ48" s="45"/>
+      <c r="AR48" s="42"/>
+      <c r="AS48" s="43"/>
+      <c r="AT48" s="43"/>
+      <c r="AU48" s="43"/>
+      <c r="AV48" s="43"/>
+      <c r="AW48" s="44"/>
+      <c r="AX48" s="43"/>
+      <c r="AY48" s="45"/>
+      <c r="AZ48" s="42"/>
+      <c r="BA48" s="43"/>
+      <c r="BB48" s="43"/>
+      <c r="BC48" s="43"/>
+      <c r="BD48" s="43"/>
+      <c r="BE48" s="44"/>
+      <c r="BF48" s="44"/>
+      <c r="BG48" s="46"/>
+      <c r="BH48" s="43"/>
+      <c r="BI48" s="43"/>
+      <c r="BJ48" s="43"/>
+      <c r="BK48" s="43"/>
+      <c r="BL48" s="43"/>
+      <c r="BM48" s="44"/>
+      <c r="BN48" s="44"/>
+      <c r="BO48" s="46"/>
+      <c r="BP48" s="43"/>
+      <c r="BQ48" s="43"/>
+      <c r="BR48" s="43"/>
+      <c r="BS48" s="43"/>
+      <c r="BT48" s="43"/>
+      <c r="BU48" s="44"/>
+      <c r="BV48" s="43"/>
+      <c r="BW48" s="46"/>
+      <c r="BX48" s="66"/>
+      <c r="BY48" s="66"/>
+      <c r="BZ48" s="66"/>
+      <c r="CA48" s="43"/>
+      <c r="CB48" s="43"/>
+      <c r="CC48" s="47"/>
+      <c r="CD48" s="44"/>
+      <c r="CE48" s="47"/>
+      <c r="CF48" s="84" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="91"/>
-      <c r="B49" s="89"/>
-      <c r="C49" s="99"/>
-      <c r="D49" s="37"/>
-      <c r="E49" s="34"/>
-      <c r="F49" s="34"/>
-      <c r="G49" s="34"/>
-      <c r="H49" s="34"/>
-      <c r="I49" s="34"/>
-      <c r="J49" s="34"/>
-      <c r="K49" s="39"/>
-      <c r="L49" s="38"/>
-      <c r="M49" s="34"/>
-      <c r="N49" s="34"/>
-      <c r="O49" s="34"/>
-      <c r="P49" s="34"/>
-      <c r="Q49" s="34"/>
-      <c r="R49" s="34"/>
-      <c r="S49" s="39"/>
-      <c r="T49" s="38"/>
-      <c r="U49" s="34"/>
-      <c r="V49" s="34"/>
-      <c r="W49" s="34"/>
-      <c r="X49" s="34"/>
-      <c r="Y49" s="34"/>
-      <c r="Z49" s="34"/>
-      <c r="AA49" s="39"/>
-      <c r="AB49" s="38"/>
-      <c r="AC49" s="34"/>
-      <c r="AD49" s="34"/>
-      <c r="AE49" s="34"/>
-      <c r="AF49" s="34"/>
-      <c r="AG49" s="34"/>
-      <c r="AH49" s="34"/>
-      <c r="AI49" s="39"/>
-      <c r="AJ49" s="38"/>
-      <c r="AK49" s="34"/>
-      <c r="AL49" s="34"/>
-      <c r="AM49" s="34"/>
-      <c r="AN49" s="34"/>
-      <c r="AO49" s="34"/>
-      <c r="AP49" s="34"/>
-      <c r="AQ49" s="39"/>
-      <c r="AR49" s="38"/>
-      <c r="AS49" s="34"/>
-      <c r="AT49" s="34"/>
-      <c r="AU49" s="34"/>
-      <c r="AV49" s="34"/>
-      <c r="AW49" s="34"/>
-      <c r="AX49" s="34"/>
-      <c r="AY49" s="39"/>
-      <c r="AZ49" s="38"/>
-      <c r="BA49" s="34"/>
-      <c r="BB49" s="34"/>
-      <c r="BC49" s="34"/>
-      <c r="BD49" s="34"/>
-      <c r="BE49" s="34"/>
-      <c r="BF49" s="34"/>
-      <c r="BG49" s="39"/>
-      <c r="BH49" s="38"/>
-      <c r="BI49" s="34"/>
-      <c r="BJ49" s="34"/>
-      <c r="BK49" s="34"/>
-      <c r="BL49" s="34"/>
-      <c r="BM49" s="34"/>
-      <c r="BN49" s="34"/>
-      <c r="BO49" s="39"/>
-      <c r="BP49" s="38"/>
-      <c r="BQ49" s="34"/>
-      <c r="BR49" s="34"/>
-      <c r="BS49" s="34"/>
-      <c r="BT49" s="34"/>
-      <c r="BU49" s="34"/>
-      <c r="BV49" s="34"/>
-      <c r="BW49" s="39"/>
-      <c r="BX49" s="38"/>
-      <c r="BY49" s="34"/>
-      <c r="BZ49" s="34"/>
-      <c r="CA49" s="34"/>
-      <c r="CB49" s="34"/>
-      <c r="CC49" s="34"/>
-      <c r="CD49" s="34"/>
-      <c r="CE49" s="39"/>
-      <c r="CF49" s="84"/>
+      <c r="A49" s="90"/>
+      <c r="B49" s="88"/>
+      <c r="C49" s="98"/>
+      <c r="D49" s="36"/>
+      <c r="E49" s="33"/>
+      <c r="F49" s="33"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="33"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="33"/>
+      <c r="K49" s="38"/>
+      <c r="L49" s="37"/>
+      <c r="M49" s="33"/>
+      <c r="N49" s="33"/>
+      <c r="O49" s="33"/>
+      <c r="P49" s="33"/>
+      <c r="Q49" s="33"/>
+      <c r="R49" s="33"/>
+      <c r="S49" s="38"/>
+      <c r="T49" s="37"/>
+      <c r="U49" s="33"/>
+      <c r="V49" s="33"/>
+      <c r="W49" s="33"/>
+      <c r="X49" s="33"/>
+      <c r="Y49" s="33"/>
+      <c r="Z49" s="33"/>
+      <c r="AA49" s="38"/>
+      <c r="AB49" s="37"/>
+      <c r="AC49" s="33"/>
+      <c r="AD49" s="33"/>
+      <c r="AE49" s="33"/>
+      <c r="AF49" s="33"/>
+      <c r="AG49" s="33"/>
+      <c r="AH49" s="33"/>
+      <c r="AI49" s="38"/>
+      <c r="AJ49" s="37"/>
+      <c r="AK49" s="33"/>
+      <c r="AL49" s="33"/>
+      <c r="AM49" s="33"/>
+      <c r="AN49" s="33"/>
+      <c r="AO49" s="33"/>
+      <c r="AP49" s="33"/>
+      <c r="AQ49" s="38"/>
+      <c r="AR49" s="37"/>
+      <c r="AS49" s="33"/>
+      <c r="AT49" s="33"/>
+      <c r="AU49" s="33"/>
+      <c r="AV49" s="33"/>
+      <c r="AW49" s="33"/>
+      <c r="AX49" s="33"/>
+      <c r="AY49" s="38"/>
+      <c r="AZ49" s="37"/>
+      <c r="BA49" s="33"/>
+      <c r="BB49" s="33"/>
+      <c r="BC49" s="33"/>
+      <c r="BD49" s="33"/>
+      <c r="BE49" s="33"/>
+      <c r="BF49" s="33"/>
+      <c r="BG49" s="38"/>
+      <c r="BH49" s="37"/>
+      <c r="BI49" s="33"/>
+      <c r="BJ49" s="33"/>
+      <c r="BK49" s="33"/>
+      <c r="BL49" s="33"/>
+      <c r="BM49" s="33"/>
+      <c r="BN49" s="33"/>
+      <c r="BO49" s="38"/>
+      <c r="BP49" s="37"/>
+      <c r="BQ49" s="33"/>
+      <c r="BR49" s="33"/>
+      <c r="BS49" s="33"/>
+      <c r="BT49" s="33"/>
+      <c r="BU49" s="33"/>
+      <c r="BV49" s="33"/>
+      <c r="BW49" s="38"/>
+      <c r="BX49" s="37"/>
+      <c r="BY49" s="33"/>
+      <c r="BZ49" s="33"/>
+      <c r="CA49" s="33"/>
+      <c r="CB49" s="33"/>
+      <c r="CC49" s="33"/>
+      <c r="CD49" s="33"/>
+      <c r="CE49" s="38"/>
+      <c r="CF49" s="83"/>
     </row>
     <row r="50" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="96" t="s">
+      <c r="A50" s="95" t="s">
         <v>24</v>
       </c>
-      <c r="B50" s="94">
+      <c r="B50" s="93">
         <v>5</v>
       </c>
-      <c r="C50" s="98">
+      <c r="C50" s="97">
         <v>0</v>
       </c>
-      <c r="D50" s="54"/>
-      <c r="E50" s="55"/>
-      <c r="F50" s="55"/>
-      <c r="G50" s="55"/>
-      <c r="H50" s="55"/>
-      <c r="I50" s="56"/>
-      <c r="J50" s="56"/>
-      <c r="K50" s="47"/>
-      <c r="L50" s="54"/>
-      <c r="M50" s="55"/>
-      <c r="N50" s="55"/>
-      <c r="O50" s="55"/>
-      <c r="P50" s="55"/>
-      <c r="Q50" s="56"/>
-      <c r="R50" s="56"/>
-      <c r="S50" s="47"/>
-      <c r="T50" s="54"/>
-      <c r="U50" s="55"/>
-      <c r="V50" s="55"/>
-      <c r="W50" s="55"/>
-      <c r="X50" s="55"/>
-      <c r="Y50" s="56"/>
-      <c r="Z50" s="55"/>
-      <c r="AA50" s="47"/>
-      <c r="AB50" s="54"/>
-      <c r="AC50" s="55"/>
-      <c r="AD50" s="55"/>
-      <c r="AE50" s="55"/>
-      <c r="AF50" s="55"/>
-      <c r="AG50" s="56"/>
-      <c r="AH50" s="56"/>
-      <c r="AI50" s="47"/>
-      <c r="AJ50" s="54"/>
-      <c r="AK50" s="55"/>
-      <c r="AL50" s="56"/>
-      <c r="AM50" s="55"/>
-      <c r="AN50" s="55"/>
-      <c r="AO50" s="56"/>
-      <c r="AP50" s="56"/>
-      <c r="AQ50" s="47"/>
-      <c r="AR50" s="54"/>
-      <c r="AS50" s="55"/>
-      <c r="AT50" s="55"/>
-      <c r="AU50" s="55"/>
-      <c r="AV50" s="55"/>
-      <c r="AW50" s="56"/>
-      <c r="AX50" s="55"/>
-      <c r="AY50" s="47"/>
-      <c r="AZ50" s="54"/>
-      <c r="BA50" s="55"/>
-      <c r="BB50" s="55"/>
-      <c r="BC50" s="55"/>
-      <c r="BD50" s="55"/>
-      <c r="BE50" s="56"/>
-      <c r="BF50" s="56"/>
-      <c r="BG50" s="47"/>
-      <c r="BH50" s="55"/>
-      <c r="BI50" s="55"/>
-      <c r="BJ50" s="55"/>
-      <c r="BK50" s="55"/>
-      <c r="BL50" s="55"/>
-      <c r="BM50" s="56"/>
-      <c r="BN50" s="56"/>
-      <c r="BO50" s="47"/>
-      <c r="BP50" s="55"/>
-      <c r="BQ50" s="55"/>
-      <c r="BR50" s="55"/>
-      <c r="BS50" s="55"/>
-      <c r="BT50" s="55"/>
-      <c r="BU50" s="56"/>
-      <c r="BV50" s="55"/>
+      <c r="D50" s="53"/>
+      <c r="E50" s="54"/>
+      <c r="F50" s="54"/>
+      <c r="G50" s="54"/>
+      <c r="H50" s="54"/>
+      <c r="I50" s="55"/>
+      <c r="J50" s="55"/>
+      <c r="K50" s="46"/>
+      <c r="L50" s="53"/>
+      <c r="M50" s="54"/>
+      <c r="N50" s="54"/>
+      <c r="O50" s="54"/>
+      <c r="P50" s="54"/>
+      <c r="Q50" s="55"/>
+      <c r="R50" s="55"/>
+      <c r="S50" s="46"/>
+      <c r="T50" s="53"/>
+      <c r="U50" s="54"/>
+      <c r="V50" s="54"/>
+      <c r="W50" s="54"/>
+      <c r="X50" s="54"/>
+      <c r="Y50" s="55"/>
+      <c r="Z50" s="54"/>
+      <c r="AA50" s="46"/>
+      <c r="AB50" s="53"/>
+      <c r="AC50" s="54"/>
+      <c r="AD50" s="54"/>
+      <c r="AE50" s="54"/>
+      <c r="AF50" s="54"/>
+      <c r="AG50" s="55"/>
+      <c r="AH50" s="55"/>
+      <c r="AI50" s="46"/>
+      <c r="AJ50" s="53"/>
+      <c r="AK50" s="54"/>
+      <c r="AL50" s="55"/>
+      <c r="AM50" s="54"/>
+      <c r="AN50" s="54"/>
+      <c r="AO50" s="55"/>
+      <c r="AP50" s="55"/>
+      <c r="AQ50" s="46"/>
+      <c r="AR50" s="53"/>
+      <c r="AS50" s="54"/>
+      <c r="AT50" s="54"/>
+      <c r="AU50" s="54"/>
+      <c r="AV50" s="54"/>
+      <c r="AW50" s="55"/>
+      <c r="AX50" s="54"/>
+      <c r="AY50" s="46"/>
+      <c r="AZ50" s="53"/>
+      <c r="BA50" s="54"/>
+      <c r="BB50" s="54"/>
+      <c r="BC50" s="54"/>
+      <c r="BD50" s="54"/>
+      <c r="BE50" s="55"/>
+      <c r="BF50" s="55"/>
+      <c r="BG50" s="46"/>
+      <c r="BH50" s="54"/>
+      <c r="BI50" s="54"/>
+      <c r="BJ50" s="54"/>
+      <c r="BK50" s="54"/>
+      <c r="BL50" s="54"/>
+      <c r="BM50" s="55"/>
+      <c r="BN50" s="55"/>
+      <c r="BO50" s="46"/>
+      <c r="BP50" s="54"/>
+      <c r="BQ50" s="54"/>
+      <c r="BR50" s="54"/>
+      <c r="BS50" s="54"/>
+      <c r="BT50" s="54"/>
+      <c r="BU50" s="55"/>
+      <c r="BV50" s="54"/>
       <c r="BW50" s="15"/>
-      <c r="BX50" s="55"/>
-      <c r="BY50" s="55"/>
-      <c r="BZ50" s="55"/>
-      <c r="CA50" s="64"/>
-      <c r="CB50" s="64"/>
-      <c r="CC50" s="65"/>
-      <c r="CD50" s="66"/>
-      <c r="CE50" s="65"/>
-      <c r="CF50" s="85"/>
+      <c r="BX50" s="54"/>
+      <c r="BY50" s="54"/>
+      <c r="BZ50" s="54"/>
+      <c r="CA50" s="63"/>
+      <c r="CB50" s="63"/>
+      <c r="CC50" s="64"/>
+      <c r="CD50" s="65"/>
+      <c r="CE50" s="64"/>
+      <c r="CF50" s="84"/>
     </row>
     <row r="51" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="91"/>
-      <c r="B51" s="89"/>
-      <c r="C51" s="99"/>
+      <c r="A51" s="90"/>
+      <c r="B51" s="88"/>
+      <c r="C51" s="98"/>
       <c r="D51" s="17"/>
       <c r="E51" s="19"/>
       <c r="F51" s="19"/>
@@ -6292,17 +6292,17 @@
       <c r="CC51" s="19"/>
       <c r="CD51" s="19"/>
       <c r="CE51" s="20"/>
-      <c r="CF51" s="84"/>
+      <c r="CF51" s="83"/>
     </row>
     <row r="52" spans="1:84" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="49" t="s">
+      <c r="A52" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="B52" s="50">
+      <c r="B52" s="49">
         <f>SUM(B4:B51)</f>
         <v>81</v>
       </c>
-      <c r="C52" s="50">
+      <c r="C52" s="49">
         <f>SUM(C4:C51)</f>
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
feat: improve squad builder UI and update documentation
</commit_message>
<xml_diff>
--- a/docs/Squad App Frontend IPA Zeitplan.xlsx
+++ b/docs/Squad App Frontend IPA Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D70889-5471-4C38-8136-E16A90C65AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17A32890-6728-4F98-838F-F433468ECD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-1930" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -926,7 +926,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1152,6 +1152,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -2136,7 +2137,7 @@
       <c r="BT5" s="18"/>
       <c r="BU5" s="19"/>
       <c r="BV5" s="18"/>
-      <c r="BW5" s="20"/>
+      <c r="BW5" s="73"/>
       <c r="BX5" s="24"/>
       <c r="BY5" s="18"/>
       <c r="BZ5" s="18"/>
@@ -2489,7 +2490,7 @@
       <c r="BM9" s="71"/>
       <c r="BN9" s="71"/>
       <c r="BO9" s="73"/>
-      <c r="BP9" s="17"/>
+      <c r="BP9" s="75"/>
       <c r="BQ9" s="18"/>
       <c r="BR9" s="18"/>
       <c r="BS9" s="18"/>
@@ -5740,11 +5741,11 @@
       <c r="BM45" s="19"/>
       <c r="BN45" s="19"/>
       <c r="BO45" s="20"/>
-      <c r="BP45" s="75"/>
+      <c r="BP45" s="17"/>
       <c r="BQ45" s="70"/>
       <c r="BR45" s="70"/>
       <c r="BS45" s="70"/>
-      <c r="BT45" s="18"/>
+      <c r="BT45" s="70"/>
       <c r="BU45" s="19"/>
       <c r="BV45" s="18"/>
       <c r="BW45" s="20"/>
@@ -5923,9 +5924,9 @@
       <c r="BR47" s="37"/>
       <c r="BS47" s="37"/>
       <c r="BT47" s="37"/>
-      <c r="BU47" s="33"/>
-      <c r="BV47" s="37"/>
-      <c r="BW47" s="38"/>
+      <c r="BU47" s="78"/>
+      <c r="BV47" s="77"/>
+      <c r="BW47" s="125"/>
       <c r="BX47" s="36"/>
       <c r="BY47" s="37"/>
       <c r="BZ47" s="37"/>

</xml_diff>

<commit_message>
docs: finalize IPA documentation and timetable
</commit_message>
<xml_diff>
--- a/docs/Squad App Frontend IPA Zeitplan.xlsx
+++ b/docs/Squad App Frontend IPA Zeitplan.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17A32890-6728-4F98-838F-F433468ECD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E43DC341-3B33-42B6-8183-87E872C943D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-1930" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -109,9 +109,6 @@
     <t>Reflexion &amp; Fazit</t>
   </si>
   <si>
-    <t>Dokumentation abschliesen</t>
-  </si>
-  <si>
     <t>Dokumentation</t>
   </si>
   <si>
@@ -164,6 +161,9 @@
   </si>
   <si>
     <t>Arbeitsjournal führen</t>
+  </si>
+  <si>
+    <t>Dokumentation abschliessen</t>
   </si>
 </sst>
 </file>
@@ -1023,6 +1023,73 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1086,73 +1153,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1499,225 +1499,225 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="105" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="85" t="s">
+      <c r="B1" s="108" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="86"/>
-      <c r="D1" s="89" t="s">
+      <c r="C1" s="109"/>
+      <c r="D1" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="90"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="92"/>
-      <c r="L1" s="100" t="s">
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+      <c r="H1" s="113"/>
+      <c r="I1" s="114"/>
+      <c r="J1" s="114"/>
+      <c r="K1" s="115"/>
+      <c r="L1" s="123" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="101"/>
-      <c r="N1" s="101"/>
-      <c r="O1" s="101"/>
-      <c r="P1" s="101"/>
-      <c r="Q1" s="101"/>
-      <c r="R1" s="101"/>
-      <c r="S1" s="102"/>
-      <c r="T1" s="89" t="s">
+      <c r="M1" s="124"/>
+      <c r="N1" s="124"/>
+      <c r="O1" s="124"/>
+      <c r="P1" s="124"/>
+      <c r="Q1" s="124"/>
+      <c r="R1" s="124"/>
+      <c r="S1" s="125"/>
+      <c r="T1" s="112" t="s">
         <v>15</v>
       </c>
-      <c r="U1" s="90"/>
-      <c r="V1" s="90"/>
-      <c r="W1" s="90"/>
-      <c r="X1" s="90"/>
-      <c r="Y1" s="91"/>
-      <c r="Z1" s="91"/>
-      <c r="AA1" s="92"/>
-      <c r="AB1" s="89" t="s">
+      <c r="U1" s="113"/>
+      <c r="V1" s="113"/>
+      <c r="W1" s="113"/>
+      <c r="X1" s="113"/>
+      <c r="Y1" s="114"/>
+      <c r="Z1" s="114"/>
+      <c r="AA1" s="115"/>
+      <c r="AB1" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="AC1" s="90"/>
-      <c r="AD1" s="90"/>
-      <c r="AE1" s="90"/>
-      <c r="AF1" s="90"/>
-      <c r="AG1" s="91"/>
-      <c r="AH1" s="91"/>
-      <c r="AI1" s="92"/>
-      <c r="AJ1" s="89" t="s">
+      <c r="AC1" s="113"/>
+      <c r="AD1" s="113"/>
+      <c r="AE1" s="113"/>
+      <c r="AF1" s="113"/>
+      <c r="AG1" s="114"/>
+      <c r="AH1" s="114"/>
+      <c r="AI1" s="115"/>
+      <c r="AJ1" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="AK1" s="90"/>
-      <c r="AL1" s="90"/>
-      <c r="AM1" s="90"/>
-      <c r="AN1" s="90"/>
-      <c r="AO1" s="91"/>
-      <c r="AP1" s="91"/>
-      <c r="AQ1" s="92"/>
-      <c r="AR1" s="89" t="s">
+      <c r="AK1" s="113"/>
+      <c r="AL1" s="113"/>
+      <c r="AM1" s="113"/>
+      <c r="AN1" s="113"/>
+      <c r="AO1" s="114"/>
+      <c r="AP1" s="114"/>
+      <c r="AQ1" s="115"/>
+      <c r="AR1" s="112" t="s">
         <v>17</v>
       </c>
-      <c r="AS1" s="90"/>
-      <c r="AT1" s="90"/>
-      <c r="AU1" s="90"/>
-      <c r="AV1" s="90"/>
-      <c r="AW1" s="91"/>
-      <c r="AX1" s="91"/>
-      <c r="AY1" s="92"/>
-      <c r="AZ1" s="89" t="s">
+      <c r="AS1" s="113"/>
+      <c r="AT1" s="113"/>
+      <c r="AU1" s="113"/>
+      <c r="AV1" s="113"/>
+      <c r="AW1" s="114"/>
+      <c r="AX1" s="114"/>
+      <c r="AY1" s="115"/>
+      <c r="AZ1" s="112" t="s">
         <v>19</v>
       </c>
-      <c r="BA1" s="90"/>
-      <c r="BB1" s="90"/>
-      <c r="BC1" s="90"/>
-      <c r="BD1" s="90"/>
-      <c r="BE1" s="91"/>
-      <c r="BF1" s="91"/>
-      <c r="BG1" s="92"/>
-      <c r="BH1" s="89" t="s">
+      <c r="BA1" s="113"/>
+      <c r="BB1" s="113"/>
+      <c r="BC1" s="113"/>
+      <c r="BD1" s="113"/>
+      <c r="BE1" s="114"/>
+      <c r="BF1" s="114"/>
+      <c r="BG1" s="115"/>
+      <c r="BH1" s="112" t="s">
         <v>20</v>
       </c>
-      <c r="BI1" s="90"/>
-      <c r="BJ1" s="90"/>
-      <c r="BK1" s="90"/>
-      <c r="BL1" s="90"/>
-      <c r="BM1" s="91"/>
-      <c r="BN1" s="91"/>
-      <c r="BO1" s="92"/>
-      <c r="BP1" s="89" t="s">
+      <c r="BI1" s="113"/>
+      <c r="BJ1" s="113"/>
+      <c r="BK1" s="113"/>
+      <c r="BL1" s="113"/>
+      <c r="BM1" s="114"/>
+      <c r="BN1" s="114"/>
+      <c r="BO1" s="115"/>
+      <c r="BP1" s="112" t="s">
         <v>16</v>
       </c>
-      <c r="BQ1" s="90"/>
-      <c r="BR1" s="90"/>
-      <c r="BS1" s="90"/>
-      <c r="BT1" s="90"/>
-      <c r="BU1" s="91"/>
-      <c r="BV1" s="91"/>
-      <c r="BW1" s="92"/>
-      <c r="BX1" s="89" t="s">
+      <c r="BQ1" s="113"/>
+      <c r="BR1" s="113"/>
+      <c r="BS1" s="113"/>
+      <c r="BT1" s="113"/>
+      <c r="BU1" s="114"/>
+      <c r="BV1" s="114"/>
+      <c r="BW1" s="115"/>
+      <c r="BX1" s="112" t="s">
         <v>18</v>
       </c>
-      <c r="BY1" s="90"/>
-      <c r="BZ1" s="90"/>
-      <c r="CA1" s="90"/>
-      <c r="CB1" s="90"/>
-      <c r="CC1" s="91"/>
-      <c r="CD1" s="91"/>
-      <c r="CE1" s="92"/>
-      <c r="CF1" s="93" t="s">
+      <c r="BY1" s="113"/>
+      <c r="BZ1" s="113"/>
+      <c r="CA1" s="113"/>
+      <c r="CB1" s="113"/>
+      <c r="CC1" s="114"/>
+      <c r="CD1" s="114"/>
+      <c r="CE1" s="115"/>
+      <c r="CF1" s="116" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:92" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="83"/>
-      <c r="B2" s="87"/>
-      <c r="C2" s="88"/>
-      <c r="D2" s="96">
+      <c r="A2" s="106"/>
+      <c r="B2" s="110"/>
+      <c r="C2" s="111"/>
+      <c r="D2" s="119">
         <v>46083</v>
       </c>
-      <c r="E2" s="97"/>
-      <c r="F2" s="97"/>
-      <c r="G2" s="97"/>
-      <c r="H2" s="97"/>
-      <c r="I2" s="98"/>
-      <c r="J2" s="98"/>
-      <c r="K2" s="99"/>
-      <c r="L2" s="96">
+      <c r="E2" s="120"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="121"/>
+      <c r="J2" s="121"/>
+      <c r="K2" s="122"/>
+      <c r="L2" s="119">
         <v>46084</v>
       </c>
-      <c r="M2" s="97"/>
-      <c r="N2" s="97"/>
-      <c r="O2" s="97"/>
-      <c r="P2" s="97"/>
-      <c r="Q2" s="98"/>
-      <c r="R2" s="98"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="96">
+      <c r="M2" s="120"/>
+      <c r="N2" s="120"/>
+      <c r="O2" s="120"/>
+      <c r="P2" s="120"/>
+      <c r="Q2" s="121"/>
+      <c r="R2" s="121"/>
+      <c r="S2" s="122"/>
+      <c r="T2" s="119">
         <v>46085</v>
       </c>
-      <c r="U2" s="97"/>
-      <c r="V2" s="97"/>
-      <c r="W2" s="97"/>
-      <c r="X2" s="97"/>
-      <c r="Y2" s="98"/>
-      <c r="Z2" s="98"/>
-      <c r="AA2" s="99"/>
-      <c r="AB2" s="96">
+      <c r="U2" s="120"/>
+      <c r="V2" s="120"/>
+      <c r="W2" s="120"/>
+      <c r="X2" s="120"/>
+      <c r="Y2" s="121"/>
+      <c r="Z2" s="121"/>
+      <c r="AA2" s="122"/>
+      <c r="AB2" s="119">
         <v>46086</v>
       </c>
-      <c r="AC2" s="97"/>
-      <c r="AD2" s="97"/>
-      <c r="AE2" s="97"/>
-      <c r="AF2" s="97"/>
-      <c r="AG2" s="98"/>
-      <c r="AH2" s="98"/>
-      <c r="AI2" s="99"/>
-      <c r="AJ2" s="96">
+      <c r="AC2" s="120"/>
+      <c r="AD2" s="120"/>
+      <c r="AE2" s="120"/>
+      <c r="AF2" s="120"/>
+      <c r="AG2" s="121"/>
+      <c r="AH2" s="121"/>
+      <c r="AI2" s="122"/>
+      <c r="AJ2" s="119">
         <v>46087</v>
       </c>
-      <c r="AK2" s="97"/>
-      <c r="AL2" s="97"/>
-      <c r="AM2" s="97"/>
-      <c r="AN2" s="97"/>
-      <c r="AO2" s="98"/>
-      <c r="AP2" s="98"/>
-      <c r="AQ2" s="99"/>
-      <c r="AR2" s="96">
+      <c r="AK2" s="120"/>
+      <c r="AL2" s="120"/>
+      <c r="AM2" s="120"/>
+      <c r="AN2" s="120"/>
+      <c r="AO2" s="121"/>
+      <c r="AP2" s="121"/>
+      <c r="AQ2" s="122"/>
+      <c r="AR2" s="119">
         <v>46090</v>
       </c>
-      <c r="AS2" s="97"/>
-      <c r="AT2" s="97"/>
-      <c r="AU2" s="97"/>
-      <c r="AV2" s="97"/>
-      <c r="AW2" s="98"/>
-      <c r="AX2" s="98"/>
-      <c r="AY2" s="99"/>
-      <c r="AZ2" s="96">
+      <c r="AS2" s="120"/>
+      <c r="AT2" s="120"/>
+      <c r="AU2" s="120"/>
+      <c r="AV2" s="120"/>
+      <c r="AW2" s="121"/>
+      <c r="AX2" s="121"/>
+      <c r="AY2" s="122"/>
+      <c r="AZ2" s="119">
         <v>46091</v>
       </c>
-      <c r="BA2" s="97"/>
-      <c r="BB2" s="97"/>
-      <c r="BC2" s="97"/>
-      <c r="BD2" s="97"/>
-      <c r="BE2" s="98"/>
-      <c r="BF2" s="98"/>
-      <c r="BG2" s="99"/>
-      <c r="BH2" s="96">
+      <c r="BA2" s="120"/>
+      <c r="BB2" s="120"/>
+      <c r="BC2" s="120"/>
+      <c r="BD2" s="120"/>
+      <c r="BE2" s="121"/>
+      <c r="BF2" s="121"/>
+      <c r="BG2" s="122"/>
+      <c r="BH2" s="119">
         <v>46092</v>
       </c>
-      <c r="BI2" s="97"/>
-      <c r="BJ2" s="97"/>
-      <c r="BK2" s="97"/>
-      <c r="BL2" s="97"/>
-      <c r="BM2" s="98"/>
-      <c r="BN2" s="98"/>
-      <c r="BO2" s="99"/>
-      <c r="BP2" s="96">
+      <c r="BI2" s="120"/>
+      <c r="BJ2" s="120"/>
+      <c r="BK2" s="120"/>
+      <c r="BL2" s="120"/>
+      <c r="BM2" s="121"/>
+      <c r="BN2" s="121"/>
+      <c r="BO2" s="122"/>
+      <c r="BP2" s="119">
         <v>46093</v>
       </c>
-      <c r="BQ2" s="97"/>
-      <c r="BR2" s="97"/>
-      <c r="BS2" s="97"/>
-      <c r="BT2" s="97"/>
-      <c r="BU2" s="98"/>
-      <c r="BV2" s="98"/>
-      <c r="BW2" s="99"/>
-      <c r="BX2" s="96">
+      <c r="BQ2" s="120"/>
+      <c r="BR2" s="120"/>
+      <c r="BS2" s="120"/>
+      <c r="BT2" s="120"/>
+      <c r="BU2" s="121"/>
+      <c r="BV2" s="121"/>
+      <c r="BW2" s="122"/>
+      <c r="BX2" s="119">
         <v>46094</v>
       </c>
-      <c r="BY2" s="97"/>
-      <c r="BZ2" s="97"/>
-      <c r="CA2" s="97"/>
-      <c r="CB2" s="97"/>
-      <c r="CC2" s="98"/>
-      <c r="CD2" s="98"/>
-      <c r="CE2" s="99"/>
-      <c r="CF2" s="94"/>
+      <c r="BY2" s="120"/>
+      <c r="BZ2" s="120"/>
+      <c r="CA2" s="120"/>
+      <c r="CB2" s="120"/>
+      <c r="CC2" s="121"/>
+      <c r="CD2" s="121"/>
+      <c r="CE2" s="122"/>
+      <c r="CF2" s="117"/>
     </row>
     <row r="3" spans="1:92" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="84"/>
+      <c r="A3" s="107"/>
       <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
@@ -1964,17 +1964,17 @@
       <c r="CE3" s="11">
         <v>8</v>
       </c>
-      <c r="CF3" s="95"/>
+      <c r="CF3" s="118"/>
     </row>
     <row r="4" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="109" t="s">
-        <v>42</v>
-      </c>
-      <c r="B4" s="105">
+      <c r="A4" s="91" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="89">
         <v>4</v>
       </c>
-      <c r="C4" s="107">
-        <v>2.5</v>
+      <c r="C4" s="87">
+        <v>4</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="13"/>
@@ -2056,16 +2056,16 @@
       <c r="CC4" s="16"/>
       <c r="CD4" s="14"/>
       <c r="CE4" s="52"/>
-      <c r="CF4" s="124"/>
+      <c r="CF4" s="83"/>
       <c r="CH4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="CI4" s="3"/>
     </row>
     <row r="5" spans="1:92" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="110"/>
-      <c r="B5" s="106"/>
-      <c r="C5" s="108"/>
+      <c r="A5" s="98"/>
+      <c r="B5" s="96"/>
+      <c r="C5" s="94"/>
       <c r="D5" s="17"/>
       <c r="E5" s="18"/>
       <c r="F5" s="18"/>
@@ -2145,21 +2145,21 @@
       <c r="CB5" s="18"/>
       <c r="CC5" s="25"/>
       <c r="CD5" s="19"/>
-      <c r="CE5" s="19"/>
-      <c r="CF5" s="123"/>
+      <c r="CE5" s="71"/>
+      <c r="CF5" s="84"/>
       <c r="CH5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="CI5" s="5"/>
     </row>
     <row r="6" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A6" s="109" t="s">
+      <c r="A6" s="91" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="105">
+      <c r="B6" s="89">
         <v>2</v>
       </c>
-      <c r="C6" s="107">
+      <c r="C6" s="87">
         <v>2</v>
       </c>
       <c r="D6" s="57"/>
@@ -2242,12 +2242,12 @@
       <c r="CC6" s="25"/>
       <c r="CD6" s="19"/>
       <c r="CE6" s="19"/>
-      <c r="CF6" s="123"/>
+      <c r="CF6" s="84"/>
     </row>
     <row r="7" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A7" s="110"/>
-      <c r="B7" s="106"/>
-      <c r="C7" s="108"/>
+      <c r="A7" s="98"/>
+      <c r="B7" s="96"/>
+      <c r="C7" s="94"/>
       <c r="D7" s="68"/>
       <c r="E7" s="69"/>
       <c r="F7" s="27"/>
@@ -2328,17 +2328,17 @@
       <c r="CC7" s="25"/>
       <c r="CD7" s="19"/>
       <c r="CE7" s="19"/>
-      <c r="CF7" s="123"/>
+      <c r="CF7" s="84"/>
     </row>
     <row r="8" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="109" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="105">
+      <c r="A8" s="91" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="89">
         <v>14</v>
       </c>
-      <c r="C8" s="107">
-        <v>9</v>
+      <c r="C8" s="87">
+        <v>16</v>
       </c>
       <c r="D8" s="26"/>
       <c r="E8" s="27"/>
@@ -2420,12 +2420,12 @@
       <c r="CC8" s="25"/>
       <c r="CD8" s="19"/>
       <c r="CE8" s="19"/>
-      <c r="CF8" s="123"/>
+      <c r="CF8" s="84"/>
     </row>
     <row r="9" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="110"/>
-      <c r="B9" s="106"/>
-      <c r="C9" s="108"/>
+      <c r="A9" s="98"/>
+      <c r="B9" s="96"/>
+      <c r="C9" s="94"/>
       <c r="D9" s="26"/>
       <c r="E9" s="27"/>
       <c r="F9" s="69"/>
@@ -2506,16 +2506,16 @@
       <c r="CC9" s="25"/>
       <c r="CD9" s="19"/>
       <c r="CE9" s="19"/>
-      <c r="CF9" s="123"/>
+      <c r="CF9" s="84"/>
     </row>
     <row r="10" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="109" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="105">
+      <c r="A10" s="91" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="89">
         <v>1</v>
       </c>
-      <c r="C10" s="107">
+      <c r="C10" s="87">
         <v>1</v>
       </c>
       <c r="D10" s="26"/>
@@ -2598,12 +2598,12 @@
       <c r="CC10" s="25"/>
       <c r="CD10" s="19"/>
       <c r="CE10" s="19"/>
-      <c r="CF10" s="123"/>
+      <c r="CF10" s="84"/>
     </row>
     <row r="11" spans="1:92" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="110"/>
-      <c r="B11" s="106"/>
-      <c r="C11" s="108"/>
+      <c r="A11" s="98"/>
+      <c r="B11" s="96"/>
+      <c r="C11" s="94"/>
       <c r="D11" s="26"/>
       <c r="E11" s="27"/>
       <c r="F11" s="27"/>
@@ -2684,17 +2684,17 @@
       <c r="CC11" s="25"/>
       <c r="CD11" s="19"/>
       <c r="CE11" s="19"/>
-      <c r="CF11" s="123"/>
+      <c r="CF11" s="84"/>
     </row>
     <row r="12" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A12" s="109" t="s">
+      <c r="A12" s="91" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="105">
+      <c r="B12" s="89">
         <v>3</v>
       </c>
-      <c r="C12" s="107">
-        <v>1</v>
+      <c r="C12" s="87">
+        <v>3</v>
       </c>
       <c r="D12" s="17"/>
       <c r="E12" s="18"/>
@@ -2776,12 +2776,12 @@
       <c r="CC12" s="25"/>
       <c r="CD12" s="19"/>
       <c r="CE12" s="19"/>
-      <c r="CF12" s="123"/>
+      <c r="CF12" s="84"/>
     </row>
     <row r="13" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="112"/>
-      <c r="B13" s="114"/>
-      <c r="C13" s="116"/>
+      <c r="A13" s="92"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="88"/>
       <c r="D13" s="28"/>
       <c r="E13" s="29"/>
       <c r="F13" s="29"/>
@@ -2862,16 +2862,16 @@
       <c r="CC13" s="32"/>
       <c r="CD13" s="33"/>
       <c r="CE13" s="30"/>
-      <c r="CF13" s="122"/>
+      <c r="CF13" s="85"/>
     </row>
     <row r="14" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A14" s="111" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14" s="113">
+      <c r="A14" s="97" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="95">
         <v>1</v>
       </c>
-      <c r="C14" s="115">
+      <c r="C14" s="93">
         <v>1</v>
       </c>
       <c r="D14" s="34"/>
@@ -2954,14 +2954,14 @@
       <c r="CC14" s="16"/>
       <c r="CD14" s="14"/>
       <c r="CE14" s="14"/>
-      <c r="CF14" s="121" t="s">
+      <c r="CF14" s="86" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:92" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="110"/>
-      <c r="B15" s="106"/>
-      <c r="C15" s="108"/>
+      <c r="A15" s="98"/>
+      <c r="B15" s="96"/>
+      <c r="C15" s="94"/>
       <c r="D15" s="17"/>
       <c r="E15" s="18"/>
       <c r="F15" s="18"/>
@@ -3042,16 +3042,16 @@
       <c r="CC15" s="25"/>
       <c r="CD15" s="19"/>
       <c r="CE15" s="19"/>
-      <c r="CF15" s="123"/>
+      <c r="CF15" s="84"/>
     </row>
     <row r="16" spans="1:92" x14ac:dyDescent="0.3">
-      <c r="A16" s="111" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="113">
+      <c r="A16" s="97" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" s="95">
         <v>1</v>
       </c>
-      <c r="C16" s="115">
+      <c r="C16" s="93">
         <v>1</v>
       </c>
       <c r="D16" s="12"/>
@@ -3134,7 +3134,7 @@
       <c r="CC16" s="16"/>
       <c r="CD16" s="14"/>
       <c r="CE16" s="14"/>
-      <c r="CF16" s="121" t="s">
+      <c r="CF16" s="86" t="s">
         <v>7</v>
       </c>
       <c r="CJ16" s="4"/>
@@ -3143,9 +3143,9 @@
       <c r="CN16" s="4"/>
     </row>
     <row r="17" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A17" s="110"/>
-      <c r="B17" s="106"/>
-      <c r="C17" s="108"/>
+      <c r="A17" s="98"/>
+      <c r="B17" s="96"/>
+      <c r="C17" s="94"/>
       <c r="D17" s="17"/>
       <c r="E17" s="18"/>
       <c r="F17" s="18"/>
@@ -3226,20 +3226,20 @@
       <c r="CC17" s="25"/>
       <c r="CD17" s="19"/>
       <c r="CE17" s="19"/>
-      <c r="CF17" s="123"/>
+      <c r="CF17" s="84"/>
       <c r="CJ17" s="4"/>
       <c r="CK17" s="4"/>
       <c r="CM17" s="4"/>
       <c r="CN17" s="4"/>
     </row>
     <row r="18" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A18" s="109" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="105">
+      <c r="A18" s="91" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="89">
         <v>1</v>
       </c>
-      <c r="C18" s="107">
+      <c r="C18" s="87">
         <v>1</v>
       </c>
       <c r="D18" s="17"/>
@@ -3322,7 +3322,7 @@
       <c r="CC18" s="25"/>
       <c r="CD18" s="19"/>
       <c r="CE18" s="19"/>
-      <c r="CF18" s="123"/>
+      <c r="CF18" s="84"/>
       <c r="CI18" s="4"/>
       <c r="CJ18" s="4"/>
       <c r="CK18" s="4"/>
@@ -3330,9 +3330,9 @@
       <c r="CN18" s="4"/>
     </row>
     <row r="19" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A19" s="110"/>
-      <c r="B19" s="106"/>
-      <c r="C19" s="108"/>
+      <c r="A19" s="98"/>
+      <c r="B19" s="96"/>
+      <c r="C19" s="94"/>
       <c r="D19" s="17"/>
       <c r="E19" s="18"/>
       <c r="F19" s="18"/>
@@ -3413,16 +3413,16 @@
       <c r="CC19" s="25"/>
       <c r="CD19" s="19"/>
       <c r="CE19" s="19"/>
-      <c r="CF19" s="123"/>
+      <c r="CF19" s="84"/>
     </row>
     <row r="20" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="109" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="105">
+      <c r="A20" s="91" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="89">
         <v>1.5</v>
       </c>
-      <c r="C20" s="107">
+      <c r="C20" s="87">
         <v>1</v>
       </c>
       <c r="D20" s="17"/>
@@ -3505,13 +3505,13 @@
       <c r="CC20" s="25"/>
       <c r="CD20" s="19"/>
       <c r="CE20" s="19"/>
-      <c r="CF20" s="123"/>
+      <c r="CF20" s="84"/>
       <c r="CJ20" s="4"/>
     </row>
     <row r="21" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="110"/>
-      <c r="B21" s="106"/>
-      <c r="C21" s="108"/>
+      <c r="A21" s="98"/>
+      <c r="B21" s="96"/>
+      <c r="C21" s="94"/>
       <c r="D21" s="17"/>
       <c r="E21" s="18"/>
       <c r="F21" s="18"/>
@@ -3592,7 +3592,7 @@
       <c r="CC21" s="25"/>
       <c r="CD21" s="19"/>
       <c r="CE21" s="19"/>
-      <c r="CF21" s="123"/>
+      <c r="CF21" s="84"/>
       <c r="CI21" s="4"/>
       <c r="CJ21" s="4"/>
       <c r="CM21" s="4"/>
@@ -3600,13 +3600,13 @@
       <c r="CO21" s="4"/>
     </row>
     <row r="22" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="117" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="105">
+      <c r="A22" s="103" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="89">
         <v>1.5</v>
       </c>
-      <c r="C22" s="107">
+      <c r="C22" s="87">
         <v>1</v>
       </c>
       <c r="D22" s="17"/>
@@ -3689,7 +3689,7 @@
       <c r="CC22" s="25"/>
       <c r="CD22" s="19"/>
       <c r="CE22" s="19"/>
-      <c r="CF22" s="123"/>
+      <c r="CF22" s="84"/>
       <c r="CI22" s="4"/>
       <c r="CJ22" s="4"/>
       <c r="CM22" s="4"/>
@@ -3697,9 +3697,9 @@
       <c r="CO22" s="4"/>
     </row>
     <row r="23" spans="1:93" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="118"/>
-      <c r="B23" s="106"/>
-      <c r="C23" s="108"/>
+      <c r="A23" s="104"/>
+      <c r="B23" s="96"/>
+      <c r="C23" s="94"/>
       <c r="D23" s="17"/>
       <c r="E23" s="18"/>
       <c r="F23" s="18"/>
@@ -3780,7 +3780,7 @@
       <c r="CC23" s="25"/>
       <c r="CD23" s="19"/>
       <c r="CE23" s="19"/>
-      <c r="CF23" s="123"/>
+      <c r="CF23" s="84"/>
       <c r="CI23" s="4"/>
       <c r="CJ23" s="4"/>
       <c r="CM23" s="4"/>
@@ -3788,13 +3788,13 @@
       <c r="CO23" s="4"/>
     </row>
     <row r="24" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A24" s="109" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24" s="105">
+      <c r="A24" s="91" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="89">
         <v>2</v>
       </c>
-      <c r="C24" s="107">
+      <c r="C24" s="87">
         <v>2</v>
       </c>
       <c r="D24" s="17"/>
@@ -3877,7 +3877,7 @@
       <c r="CC24" s="25"/>
       <c r="CD24" s="19"/>
       <c r="CE24" s="19"/>
-      <c r="CF24" s="123"/>
+      <c r="CF24" s="84"/>
       <c r="CJ24" s="4"/>
       <c r="CK24" s="4"/>
       <c r="CM24" s="4"/>
@@ -3885,9 +3885,9 @@
       <c r="CO24" s="4"/>
     </row>
     <row r="25" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="112"/>
-      <c r="B25" s="114"/>
-      <c r="C25" s="116"/>
+      <c r="A25" s="92"/>
+      <c r="B25" s="90"/>
+      <c r="C25" s="88"/>
       <c r="D25" s="36"/>
       <c r="E25" s="37"/>
       <c r="F25" s="37"/>
@@ -3968,19 +3968,19 @@
       <c r="CC25" s="39"/>
       <c r="CD25" s="33"/>
       <c r="CE25" s="33"/>
-      <c r="CF25" s="122"/>
+      <c r="CF25" s="85"/>
       <c r="CK25" s="4"/>
       <c r="CL25" s="4"/>
       <c r="CM25" s="4"/>
     </row>
     <row r="26" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A26" s="111" t="s">
+      <c r="A26" s="97" t="s">
         <v>8</v>
       </c>
-      <c r="B26" s="113">
+      <c r="B26" s="95">
         <v>2</v>
       </c>
-      <c r="C26" s="115">
+      <c r="C26" s="93">
         <v>2</v>
       </c>
       <c r="D26" s="12"/>
@@ -4063,14 +4063,14 @@
       <c r="CC26" s="16"/>
       <c r="CD26" s="14"/>
       <c r="CE26" s="14"/>
-      <c r="CF26" s="121" t="s">
+      <c r="CF26" s="86" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="27" spans="1:93" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="112"/>
-      <c r="B27" s="114"/>
-      <c r="C27" s="116"/>
+      <c r="A27" s="92"/>
+      <c r="B27" s="90"/>
+      <c r="C27" s="88"/>
       <c r="D27" s="36"/>
       <c r="E27" s="37"/>
       <c r="F27" s="37"/>
@@ -4151,16 +4151,16 @@
       <c r="CC27" s="39"/>
       <c r="CD27" s="33"/>
       <c r="CE27" s="33"/>
-      <c r="CF27" s="122"/>
+      <c r="CF27" s="85"/>
     </row>
     <row r="28" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A28" s="111" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" s="113">
+      <c r="A28" s="97" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="95">
         <v>1</v>
       </c>
-      <c r="C28" s="115">
+      <c r="C28" s="93">
         <v>1</v>
       </c>
       <c r="D28" s="12"/>
@@ -4243,14 +4243,14 @@
       <c r="CC28" s="16"/>
       <c r="CD28" s="14"/>
       <c r="CE28" s="14"/>
-      <c r="CF28" s="121" t="s">
+      <c r="CF28" s="86" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A29" s="110"/>
-      <c r="B29" s="106"/>
-      <c r="C29" s="108"/>
+      <c r="A29" s="98"/>
+      <c r="B29" s="96"/>
+      <c r="C29" s="94"/>
       <c r="D29" s="17"/>
       <c r="E29" s="18"/>
       <c r="F29" s="18"/>
@@ -4331,16 +4331,16 @@
       <c r="CC29" s="25"/>
       <c r="CD29" s="19"/>
       <c r="CE29" s="19"/>
-      <c r="CF29" s="123"/>
+      <c r="CF29" s="84"/>
     </row>
     <row r="30" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="109" t="s">
-        <v>36</v>
-      </c>
-      <c r="B30" s="105">
+      <c r="A30" s="91" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="89">
         <v>2</v>
       </c>
-      <c r="C30" s="107">
+      <c r="C30" s="87">
         <v>2</v>
       </c>
       <c r="D30" s="17"/>
@@ -4423,12 +4423,12 @@
       <c r="CC30" s="25"/>
       <c r="CD30" s="19"/>
       <c r="CE30" s="19"/>
-      <c r="CF30" s="123"/>
+      <c r="CF30" s="84"/>
     </row>
     <row r="31" spans="1:93" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="110"/>
-      <c r="B31" s="106"/>
-      <c r="C31" s="108"/>
+      <c r="A31" s="98"/>
+      <c r="B31" s="96"/>
+      <c r="C31" s="94"/>
       <c r="D31" s="17"/>
       <c r="E31" s="18"/>
       <c r="F31" s="18"/>
@@ -4509,16 +4509,16 @@
       <c r="CC31" s="25"/>
       <c r="CD31" s="19"/>
       <c r="CE31" s="19"/>
-      <c r="CF31" s="123"/>
+      <c r="CF31" s="84"/>
     </row>
     <row r="32" spans="1:93" x14ac:dyDescent="0.3">
-      <c r="A32" s="109" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32" s="105">
+      <c r="A32" s="91" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="89">
         <v>4</v>
       </c>
-      <c r="C32" s="107">
+      <c r="C32" s="87">
         <v>4</v>
       </c>
       <c r="D32" s="17"/>
@@ -4601,12 +4601,12 @@
       <c r="CC32" s="25"/>
       <c r="CD32" s="19"/>
       <c r="CE32" s="19"/>
-      <c r="CF32" s="123"/>
+      <c r="CF32" s="84"/>
     </row>
     <row r="33" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A33" s="110"/>
-      <c r="B33" s="106"/>
-      <c r="C33" s="108"/>
+      <c r="A33" s="98"/>
+      <c r="B33" s="96"/>
+      <c r="C33" s="94"/>
       <c r="D33" s="17"/>
       <c r="E33" s="18"/>
       <c r="F33" s="18"/>
@@ -4687,16 +4687,16 @@
       <c r="CC33" s="25"/>
       <c r="CD33" s="19"/>
       <c r="CE33" s="19"/>
-      <c r="CF33" s="123"/>
+      <c r="CF33" s="84"/>
     </row>
     <row r="34" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A34" s="109" t="s">
-        <v>35</v>
-      </c>
-      <c r="B34" s="105">
+      <c r="A34" s="91" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="89">
         <v>4</v>
       </c>
-      <c r="C34" s="107">
+      <c r="C34" s="87">
         <v>3.5</v>
       </c>
       <c r="D34" s="17"/>
@@ -4779,12 +4779,12 @@
       <c r="CC34" s="25"/>
       <c r="CD34" s="19"/>
       <c r="CE34" s="19"/>
-      <c r="CF34" s="123"/>
+      <c r="CF34" s="84"/>
     </row>
     <row r="35" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A35" s="110"/>
-      <c r="B35" s="106"/>
-      <c r="C35" s="108"/>
+      <c r="A35" s="98"/>
+      <c r="B35" s="96"/>
+      <c r="C35" s="94"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
       <c r="F35" s="18"/>
@@ -4865,16 +4865,16 @@
       <c r="CC35" s="25"/>
       <c r="CD35" s="19"/>
       <c r="CE35" s="19"/>
-      <c r="CF35" s="123"/>
+      <c r="CF35" s="84"/>
     </row>
     <row r="36" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A36" s="109" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="105">
+      <c r="A36" s="91" t="s">
+        <v>37</v>
+      </c>
+      <c r="B36" s="89">
         <v>9</v>
       </c>
-      <c r="C36" s="107">
+      <c r="C36" s="87">
         <v>11</v>
       </c>
       <c r="D36" s="17"/>
@@ -4957,12 +4957,12 @@
       <c r="CC36" s="25"/>
       <c r="CD36" s="19"/>
       <c r="CE36" s="19"/>
-      <c r="CF36" s="123"/>
+      <c r="CF36" s="84"/>
     </row>
     <row r="37" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A37" s="110"/>
-      <c r="B37" s="106"/>
-      <c r="C37" s="108"/>
+      <c r="A37" s="98"/>
+      <c r="B37" s="96"/>
+      <c r="C37" s="94"/>
       <c r="D37" s="17"/>
       <c r="E37" s="18"/>
       <c r="F37" s="18"/>
@@ -5043,16 +5043,16 @@
       <c r="CC37" s="25"/>
       <c r="CD37" s="19"/>
       <c r="CE37" s="19"/>
-      <c r="CF37" s="123"/>
+      <c r="CF37" s="84"/>
     </row>
     <row r="38" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A38" s="103" t="s">
-        <v>39</v>
-      </c>
-      <c r="B38" s="105">
+      <c r="A38" s="101" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" s="89">
         <v>5</v>
       </c>
-      <c r="C38" s="107">
+      <c r="C38" s="87">
         <v>5.5</v>
       </c>
       <c r="D38" s="17"/>
@@ -5135,12 +5135,12 @@
       <c r="CC38" s="25"/>
       <c r="CD38" s="19"/>
       <c r="CE38" s="19"/>
-      <c r="CF38" s="123"/>
+      <c r="CF38" s="84"/>
     </row>
     <row r="39" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A39" s="104"/>
-      <c r="B39" s="106"/>
-      <c r="C39" s="108"/>
+      <c r="A39" s="102"/>
+      <c r="B39" s="96"/>
+      <c r="C39" s="94"/>
       <c r="D39" s="17"/>
       <c r="E39" s="18"/>
       <c r="F39" s="18"/>
@@ -5221,17 +5221,17 @@
       <c r="CC39" s="25"/>
       <c r="CD39" s="19"/>
       <c r="CE39" s="19"/>
-      <c r="CF39" s="123"/>
+      <c r="CF39" s="84"/>
     </row>
     <row r="40" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A40" s="103" t="s">
-        <v>40</v>
-      </c>
-      <c r="B40" s="105">
+      <c r="A40" s="101" t="s">
+        <v>39</v>
+      </c>
+      <c r="B40" s="89">
         <v>4</v>
       </c>
-      <c r="C40" s="107">
-        <v>0</v>
+      <c r="C40" s="87">
+        <v>4</v>
       </c>
       <c r="D40" s="17"/>
       <c r="E40" s="18"/>
@@ -5313,12 +5313,12 @@
       <c r="CC40" s="25"/>
       <c r="CD40" s="19"/>
       <c r="CE40" s="19"/>
-      <c r="CF40" s="123"/>
+      <c r="CF40" s="84"/>
     </row>
     <row r="41" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A41" s="104"/>
-      <c r="B41" s="106"/>
-      <c r="C41" s="108"/>
+      <c r="A41" s="102"/>
+      <c r="B41" s="96"/>
+      <c r="C41" s="94"/>
       <c r="D41" s="17"/>
       <c r="E41" s="18"/>
       <c r="F41" s="18"/>
@@ -5399,17 +5399,17 @@
       <c r="CC41" s="25"/>
       <c r="CD41" s="19"/>
       <c r="CE41" s="19"/>
-      <c r="CF41" s="123"/>
+      <c r="CF41" s="84"/>
     </row>
     <row r="42" spans="1:84" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="109" t="s">
-        <v>41</v>
-      </c>
-      <c r="B42" s="105">
+      <c r="A42" s="91" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="89">
         <v>2</v>
       </c>
-      <c r="C42" s="107">
-        <v>0</v>
+      <c r="C42" s="87">
+        <v>2</v>
       </c>
       <c r="D42" s="17"/>
       <c r="E42" s="18"/>
@@ -5491,12 +5491,12 @@
       <c r="CC42" s="25"/>
       <c r="CD42" s="19"/>
       <c r="CE42" s="19"/>
-      <c r="CF42" s="123"/>
+      <c r="CF42" s="84"/>
     </row>
     <row r="43" spans="1:84" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="110"/>
-      <c r="B43" s="106"/>
-      <c r="C43" s="108"/>
+      <c r="A43" s="98"/>
+      <c r="B43" s="96"/>
+      <c r="C43" s="94"/>
       <c r="D43" s="17"/>
       <c r="E43" s="18"/>
       <c r="F43" s="18"/>
@@ -5577,17 +5577,17 @@
       <c r="CC43" s="25"/>
       <c r="CD43" s="19"/>
       <c r="CE43" s="19"/>
-      <c r="CF43" s="123"/>
+      <c r="CF43" s="84"/>
     </row>
     <row r="44" spans="1:84" x14ac:dyDescent="0.3">
-      <c r="A44" s="111" t="s">
+      <c r="A44" s="97" t="s">
         <v>22</v>
       </c>
-      <c r="B44" s="113">
+      <c r="B44" s="95">
         <v>5</v>
       </c>
-      <c r="C44" s="115">
-        <v>0</v>
+      <c r="C44" s="93">
+        <v>4</v>
       </c>
       <c r="D44" s="12"/>
       <c r="E44" s="13"/>
@@ -5669,14 +5669,14 @@
       <c r="CC44" s="16"/>
       <c r="CD44" s="14"/>
       <c r="CE44" s="14"/>
-      <c r="CF44" s="121" t="s">
+      <c r="CF44" s="86" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="45" spans="1:84" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="110"/>
-      <c r="B45" s="106"/>
-      <c r="C45" s="108"/>
+      <c r="A45" s="98"/>
+      <c r="B45" s="96"/>
+      <c r="C45" s="94"/>
       <c r="D45" s="17"/>
       <c r="E45" s="18"/>
       <c r="F45" s="18"/>
@@ -5757,17 +5757,17 @@
       <c r="CC45" s="25"/>
       <c r="CD45" s="19"/>
       <c r="CE45" s="19"/>
-      <c r="CF45" s="123"/>
+      <c r="CF45" s="84"/>
     </row>
     <row r="46" spans="1:84" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="109" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" s="105">
+      <c r="A46" s="91" t="s">
+        <v>36</v>
+      </c>
+      <c r="B46" s="89">
         <v>3</v>
       </c>
-      <c r="C46" s="107">
-        <v>0</v>
+      <c r="C46" s="87">
+        <v>3</v>
       </c>
       <c r="D46" s="17"/>
       <c r="E46" s="18"/>
@@ -5849,12 +5849,12 @@
       <c r="CC46" s="25"/>
       <c r="CD46" s="19"/>
       <c r="CE46" s="19"/>
-      <c r="CF46" s="123"/>
+      <c r="CF46" s="84"/>
     </row>
     <row r="47" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="112"/>
-      <c r="B47" s="114"/>
-      <c r="C47" s="116"/>
+      <c r="A47" s="92"/>
+      <c r="B47" s="90"/>
+      <c r="C47" s="88"/>
       <c r="D47" s="36"/>
       <c r="E47" s="37"/>
       <c r="F47" s="37"/>
@@ -5926,7 +5926,7 @@
       <c r="BT47" s="37"/>
       <c r="BU47" s="78"/>
       <c r="BV47" s="77"/>
-      <c r="BW47" s="125"/>
+      <c r="BW47" s="82"/>
       <c r="BX47" s="36"/>
       <c r="BY47" s="37"/>
       <c r="BZ47" s="37"/>
@@ -5935,17 +5935,17 @@
       <c r="CC47" s="39"/>
       <c r="CD47" s="33"/>
       <c r="CE47" s="33"/>
-      <c r="CF47" s="122"/>
+      <c r="CF47" s="85"/>
     </row>
     <row r="48" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="111" t="s">
+      <c r="A48" s="97" t="s">
         <v>23</v>
       </c>
-      <c r="B48" s="113">
+      <c r="B48" s="95">
         <v>3</v>
       </c>
-      <c r="C48" s="119">
-        <v>0</v>
+      <c r="C48" s="99">
+        <v>3</v>
       </c>
       <c r="D48" s="42"/>
       <c r="E48" s="43"/>
@@ -6027,14 +6027,14 @@
       <c r="CC48" s="47"/>
       <c r="CD48" s="44"/>
       <c r="CE48" s="47"/>
-      <c r="CF48" s="121" t="s">
+      <c r="CF48" s="86" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="112"/>
-      <c r="B49" s="114"/>
-      <c r="C49" s="120"/>
+      <c r="A49" s="92"/>
+      <c r="B49" s="90"/>
+      <c r="C49" s="100"/>
       <c r="D49" s="36"/>
       <c r="E49" s="33"/>
       <c r="F49" s="33"/>
@@ -6107,25 +6107,25 @@
       <c r="BU49" s="33"/>
       <c r="BV49" s="33"/>
       <c r="BW49" s="38"/>
-      <c r="BX49" s="37"/>
-      <c r="BY49" s="33"/>
-      <c r="BZ49" s="33"/>
+      <c r="BX49" s="77"/>
+      <c r="BY49" s="78"/>
+      <c r="BZ49" s="78"/>
       <c r="CA49" s="33"/>
       <c r="CB49" s="33"/>
       <c r="CC49" s="33"/>
       <c r="CD49" s="33"/>
       <c r="CE49" s="38"/>
-      <c r="CF49" s="122"/>
+      <c r="CF49" s="85"/>
     </row>
     <row r="50" spans="1:84" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="111" t="s">
-        <v>24</v>
-      </c>
-      <c r="B50" s="113">
+      <c r="A50" s="97" t="s">
+        <v>42</v>
+      </c>
+      <c r="B50" s="95">
         <v>5</v>
       </c>
-      <c r="C50" s="119">
-        <v>0</v>
+      <c r="C50" s="99">
+        <v>5</v>
       </c>
       <c r="D50" s="53"/>
       <c r="E50" s="54"/>
@@ -6207,12 +6207,12 @@
       <c r="CC50" s="64"/>
       <c r="CD50" s="65"/>
       <c r="CE50" s="64"/>
-      <c r="CF50" s="121"/>
+      <c r="CF50" s="86"/>
     </row>
     <row r="51" spans="1:84" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="112"/>
-      <c r="B51" s="114"/>
-      <c r="C51" s="120"/>
+      <c r="A51" s="92"/>
+      <c r="B51" s="90"/>
+      <c r="C51" s="100"/>
       <c r="D51" s="17"/>
       <c r="E51" s="19"/>
       <c r="F51" s="19"/>
@@ -6288,12 +6288,12 @@
       <c r="BX51" s="18"/>
       <c r="BY51" s="19"/>
       <c r="BZ51" s="19"/>
-      <c r="CA51" s="19"/>
-      <c r="CB51" s="19"/>
-      <c r="CC51" s="19"/>
-      <c r="CD51" s="19"/>
-      <c r="CE51" s="20"/>
-      <c r="CF51" s="122"/>
+      <c r="CA51" s="71"/>
+      <c r="CB51" s="71"/>
+      <c r="CC51" s="71"/>
+      <c r="CD51" s="71"/>
+      <c r="CE51" s="73"/>
+      <c r="CF51" s="85"/>
     </row>
     <row r="52" spans="1:84" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A52" s="48" t="s">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="C52" s="49">
         <f>SUM(C4:C51)</f>
-        <v>51.5</v>
+        <v>83</v>
       </c>
       <c r="CD52" s="2"/>
       <c r="CE52" s="2"/>
@@ -6343,29 +6343,62 @@
     </row>
   </sheetData>
   <mergeCells count="103">
-    <mergeCell ref="CF4:CF13"/>
-    <mergeCell ref="CF14:CF15"/>
-    <mergeCell ref="CF16:CF25"/>
-    <mergeCell ref="C24:C25"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="A24:A25"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="C12:C13"/>
-    <mergeCell ref="B12:B13"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:C2"/>
+    <mergeCell ref="BP1:BW1"/>
+    <mergeCell ref="BX1:CE1"/>
+    <mergeCell ref="CF1:CF3"/>
+    <mergeCell ref="D2:K2"/>
+    <mergeCell ref="L2:S2"/>
+    <mergeCell ref="T2:AA2"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AJ2:AQ2"/>
+    <mergeCell ref="AR2:AY2"/>
+    <mergeCell ref="AJ1:AQ1"/>
+    <mergeCell ref="AR1:AY1"/>
+    <mergeCell ref="AZ1:BG1"/>
+    <mergeCell ref="BH1:BO1"/>
+    <mergeCell ref="D1:K1"/>
+    <mergeCell ref="L1:S1"/>
+    <mergeCell ref="T1:AA1"/>
+    <mergeCell ref="AB1:AI1"/>
+    <mergeCell ref="AZ2:BG2"/>
+    <mergeCell ref="BH2:BO2"/>
+    <mergeCell ref="BP2:BW2"/>
+    <mergeCell ref="BX2:CE2"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="B40:B41"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="A42:A43"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C34:C35"/>
+    <mergeCell ref="A36:A37"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="A28:A29"/>
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="A30:A31"/>
+    <mergeCell ref="B30:B31"/>
+    <mergeCell ref="C30:C31"/>
     <mergeCell ref="A50:A51"/>
     <mergeCell ref="B50:B51"/>
     <mergeCell ref="C50:C51"/>
@@ -6390,62 +6423,29 @@
     <mergeCell ref="B32:B33"/>
     <mergeCell ref="C32:C33"/>
     <mergeCell ref="A34:A35"/>
-    <mergeCell ref="A36:A37"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="A28:A29"/>
-    <mergeCell ref="B28:B29"/>
-    <mergeCell ref="C28:C29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="B30:B31"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="B40:B41"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="A42:A43"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="C16:C17"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="A10:A11"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="A38:A39"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="C34:C35"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:C2"/>
-    <mergeCell ref="BP1:BW1"/>
-    <mergeCell ref="BX1:CE1"/>
-    <mergeCell ref="CF1:CF3"/>
-    <mergeCell ref="D2:K2"/>
-    <mergeCell ref="L2:S2"/>
-    <mergeCell ref="T2:AA2"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AJ2:AQ2"/>
-    <mergeCell ref="AR2:AY2"/>
-    <mergeCell ref="AJ1:AQ1"/>
-    <mergeCell ref="AR1:AY1"/>
-    <mergeCell ref="AZ1:BG1"/>
-    <mergeCell ref="BH1:BO1"/>
-    <mergeCell ref="D1:K1"/>
-    <mergeCell ref="L1:S1"/>
-    <mergeCell ref="T1:AA1"/>
-    <mergeCell ref="AB1:AI1"/>
-    <mergeCell ref="AZ2:BG2"/>
-    <mergeCell ref="BH2:BO2"/>
-    <mergeCell ref="BP2:BW2"/>
-    <mergeCell ref="BX2:CE2"/>
+    <mergeCell ref="CF4:CF13"/>
+    <mergeCell ref="CF14:CF15"/>
+    <mergeCell ref="CF16:CF25"/>
+    <mergeCell ref="C24:C25"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="A24:A25"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6463,12 +6463,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x0101000E5D27F8F9D77246958595755BE80D85" ma:contentTypeVersion="3" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="523cc66e991d1db8e1b1ff070bf6a3d3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="17b83e7a-435f-4364-88cb-373732b2cb78" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="b191d266e13279e8e3bfd50054307905" ns2:_="">
     <xsd:import namespace="17b83e7a-435f-4364-88cb-373732b2cb78"/>
@@ -6606,6 +6600,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{10E482C8-652F-469A-8C0D-A272F20BD8F0}">
   <ds:schemaRefs>
@@ -6615,22 +6615,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26B24723-3DEB-4B9B-91AB-D29006D23A51}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="17b83e7a-435f-4364-88cb-373732b2cb78"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{627A0659-6CE6-4668-B0C2-81E0CF5BEAC7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6646,4 +6630,20 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{26B24723-3DEB-4B9B-91AB-D29006D23A51}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="17b83e7a-435f-4364-88cb-373732b2cb78"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>